<commit_message>
QA: agregar caso real de Reintegros mobile al Excel (hoja estaba vacia)
La hoja "Reintegros" no tenia ninguna fila pese a existir un test real en
mobile/specs/vetify/reintegros.spec.ts (documenta BUG-007/IMAS-4279 en vivo,
sin equivalente Desktop). Encontrado al re-verificar la auditoria a pedido
explicito del usuario en vez de darla por cerrada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Casos de Prueba.xlsx
+++ b/documentation/Casos de Prueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ike\vetify-automation\automation\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{728B035C-A3B9-4C1C-8D27-75D866672AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA228187-C254-439A-A3A9-4C429D0BFE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2264" uniqueCount="614">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2272" uniqueCount="619">
   <si>
     <t>Total de Casos de Prueba</t>
   </si>
@@ -2227,6 +2227,22 @@
   </si>
   <si>
     <t>El sistema permite cambiar únicamente el número de teléfono. Nombre, Apellido y Número de Identificación NO son editables: se muestra un aviso fijo indicando que deben corregirse llamando al 0800 122 1183 (confirmado en vivo 2026-08-08 — contradice el criterio original de este caso, que asumía los 4 campos editables).</t>
+  </si>
+  <si>
+    <t>TS-01 Reintegros - Cuentas de acreditacion e historial (Mobile, sin equivalente Desktop)</t>
+  </si>
+  <si>
+    <t>Reintegros - Vetify - Muestra la seccion de cuentas de acreditacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Usuario autenticado con un plan vigente.</t>
+  </si>
+  <si>
+    <t>1. Abrir el menu lateral.
+2. Presionar "Reintegros".</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - La pantalla carga con la seccion "Cuentas de acreditacion" visible (unica seccion confirmada sin depender del historial, que hoy falla por BUG-007/IMAS-4279 en la cuenta usada para probarlo).</t>
   </si>
 </sst>
 </file>
@@ -2536,7 +2552,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2630,15 +2646,6 @@
     <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2659,19 +2666,28 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2688,6 +2704,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4523,734 +4542,734 @@
   <sheetData>
     <row r="2" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="3" spans="3:24">
-      <c r="C3" s="47" t="s">
+      <c r="C3" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="49"/>
-      <c r="K3" s="47" t="s">
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="46"/>
+      <c r="K3" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="49"/>
-      <c r="S3" s="47" t="s">
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="45"/>
+      <c r="P3" s="46"/>
+      <c r="S3" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="T3" s="48"/>
-      <c r="U3" s="48"/>
-      <c r="V3" s="48"/>
-      <c r="W3" s="48"/>
-      <c r="X3" s="49"/>
+      <c r="T3" s="45"/>
+      <c r="U3" s="45"/>
+      <c r="V3" s="45"/>
+      <c r="W3" s="45"/>
+      <c r="X3" s="46"/>
     </row>
     <row r="4" spans="3:24">
-      <c r="C4" s="43"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="42"/>
-      <c r="K4" s="43"/>
-      <c r="L4" s="41"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="41"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="42"/>
-      <c r="S4" s="43"/>
-      <c r="T4" s="41"/>
-      <c r="U4" s="41"/>
-      <c r="V4" s="41"/>
-      <c r="W4" s="41"/>
-      <c r="X4" s="42"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="39"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="38"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="39"/>
+      <c r="S4" s="40"/>
+      <c r="T4" s="38"/>
+      <c r="U4" s="38"/>
+      <c r="V4" s="38"/>
+      <c r="W4" s="38"/>
+      <c r="X4" s="39"/>
     </row>
     <row r="5" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C5" s="40">
+      <c r="C5" s="37">
         <f>COUNTA('Flujo de Compra'!C3:C496,'Gestión de Usuario'!C3:C357,Perfil!C3:C199,Credenciales!C3:C199,Videollamadas!C3:C199,Reintegros!C2:C199,Misceláneas!C2:C199)</f>
-        <v>253</v>
-      </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
-      <c r="K5" s="40">
+        <v>254</v>
+      </c>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
+      <c r="K5" s="37">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")+COUNTIF(Reintegros!G:G,"Si")</f>
         <v>188</v>
       </c>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-      <c r="O5" s="41"/>
-      <c r="P5" s="42"/>
-      <c r="S5" s="51">
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="39"/>
+      <c r="S5" s="48">
         <f>K5/C5</f>
-        <v>0.74308300395256921</v>
-      </c>
-      <c r="T5" s="41"/>
-      <c r="U5" s="41"/>
-      <c r="V5" s="41"/>
-      <c r="W5" s="41"/>
-      <c r="X5" s="42"/>
+        <v>0.74015748031496065</v>
+      </c>
+      <c r="T5" s="38"/>
+      <c r="U5" s="38"/>
+      <c r="V5" s="38"/>
+      <c r="W5" s="38"/>
+      <c r="X5" s="39"/>
     </row>
     <row r="6" spans="3:24">
-      <c r="C6" s="43"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="42"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="41"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="42"/>
-      <c r="S6" s="43"/>
-      <c r="T6" s="41"/>
-      <c r="U6" s="41"/>
-      <c r="V6" s="41"/>
-      <c r="W6" s="41"/>
-      <c r="X6" s="42"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="39"/>
+      <c r="K6" s="40"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="38"/>
+      <c r="P6" s="39"/>
+      <c r="S6" s="40"/>
+      <c r="T6" s="38"/>
+      <c r="U6" s="38"/>
+      <c r="V6" s="38"/>
+      <c r="W6" s="38"/>
+      <c r="X6" s="39"/>
     </row>
     <row r="7" spans="3:24">
-      <c r="C7" s="43"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="42"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="42"/>
-      <c r="S7" s="43"/>
-      <c r="T7" s="41"/>
-      <c r="U7" s="41"/>
-      <c r="V7" s="41"/>
-      <c r="W7" s="41"/>
-      <c r="X7" s="42"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="39"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
+      <c r="N7" s="38"/>
+      <c r="O7" s="38"/>
+      <c r="P7" s="39"/>
+      <c r="S7" s="40"/>
+      <c r="T7" s="38"/>
+      <c r="U7" s="38"/>
+      <c r="V7" s="38"/>
+      <c r="W7" s="38"/>
+      <c r="X7" s="39"/>
     </row>
     <row r="8" spans="3:24">
-      <c r="C8" s="43"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="42"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="41"/>
-      <c r="P8" s="42"/>
-      <c r="S8" s="43"/>
-      <c r="T8" s="41"/>
-      <c r="U8" s="41"/>
-      <c r="V8" s="41"/>
-      <c r="W8" s="41"/>
-      <c r="X8" s="42"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="39"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="38"/>
+      <c r="P8" s="39"/>
+      <c r="S8" s="40"/>
+      <c r="T8" s="38"/>
+      <c r="U8" s="38"/>
+      <c r="V8" s="38"/>
+      <c r="W8" s="38"/>
+      <c r="X8" s="39"/>
     </row>
     <row r="9" spans="3:24">
-      <c r="C9" s="43"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="42"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="41"/>
-      <c r="P9" s="42"/>
-      <c r="S9" s="43"/>
-      <c r="T9" s="41"/>
-      <c r="U9" s="41"/>
-      <c r="V9" s="41"/>
-      <c r="W9" s="41"/>
-      <c r="X9" s="42"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="39"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
+      <c r="P9" s="39"/>
+      <c r="S9" s="40"/>
+      <c r="T9" s="38"/>
+      <c r="U9" s="38"/>
+      <c r="V9" s="38"/>
+      <c r="W9" s="38"/>
+      <c r="X9" s="39"/>
     </row>
     <row r="10" spans="3:24">
-      <c r="C10" s="43"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="42"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
-      <c r="P10" s="42"/>
-      <c r="S10" s="43"/>
-      <c r="T10" s="41"/>
-      <c r="U10" s="41"/>
-      <c r="V10" s="41"/>
-      <c r="W10" s="41"/>
-      <c r="X10" s="42"/>
+      <c r="C10" s="40"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="39"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="38"/>
+      <c r="M10" s="38"/>
+      <c r="N10" s="38"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="39"/>
+      <c r="S10" s="40"/>
+      <c r="T10" s="38"/>
+      <c r="U10" s="38"/>
+      <c r="V10" s="38"/>
+      <c r="W10" s="38"/>
+      <c r="X10" s="39"/>
     </row>
     <row r="11" spans="3:24">
-      <c r="C11" s="43"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="42"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
-      <c r="N11" s="41"/>
-      <c r="O11" s="41"/>
-      <c r="P11" s="42"/>
-      <c r="S11" s="43"/>
-      <c r="T11" s="41"/>
-      <c r="U11" s="41"/>
-      <c r="V11" s="41"/>
-      <c r="W11" s="41"/>
-      <c r="X11" s="42"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="39"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="38"/>
+      <c r="M11" s="38"/>
+      <c r="N11" s="38"/>
+      <c r="O11" s="38"/>
+      <c r="P11" s="39"/>
+      <c r="S11" s="40"/>
+      <c r="T11" s="38"/>
+      <c r="U11" s="38"/>
+      <c r="V11" s="38"/>
+      <c r="W11" s="38"/>
+      <c r="X11" s="39"/>
     </row>
     <row r="12" spans="3:24">
-      <c r="C12" s="43"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="42"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
-      <c r="N12" s="41"/>
-      <c r="O12" s="41"/>
-      <c r="P12" s="42"/>
-      <c r="S12" s="43"/>
-      <c r="T12" s="41"/>
-      <c r="U12" s="41"/>
-      <c r="V12" s="41"/>
-      <c r="W12" s="41"/>
-      <c r="X12" s="42"/>
+      <c r="C12" s="40"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="39"/>
+      <c r="K12" s="40"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="38"/>
+      <c r="P12" s="39"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="38"/>
+      <c r="U12" s="38"/>
+      <c r="V12" s="38"/>
+      <c r="W12" s="38"/>
+      <c r="X12" s="39"/>
     </row>
     <row r="13" spans="3:24">
-      <c r="C13" s="43"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="42"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="41"/>
-      <c r="M13" s="41"/>
-      <c r="N13" s="41"/>
-      <c r="O13" s="41"/>
-      <c r="P13" s="42"/>
-      <c r="S13" s="43"/>
-      <c r="T13" s="41"/>
-      <c r="U13" s="41"/>
-      <c r="V13" s="41"/>
-      <c r="W13" s="41"/>
-      <c r="X13" s="42"/>
+      <c r="C13" s="40"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="39"/>
+      <c r="K13" s="40"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="38"/>
+      <c r="P13" s="39"/>
+      <c r="S13" s="40"/>
+      <c r="T13" s="38"/>
+      <c r="U13" s="38"/>
+      <c r="V13" s="38"/>
+      <c r="W13" s="38"/>
+      <c r="X13" s="39"/>
     </row>
     <row r="14" spans="3:24">
-      <c r="C14" s="43"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="42"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="41"/>
-      <c r="M14" s="41"/>
-      <c r="N14" s="41"/>
-      <c r="O14" s="41"/>
-      <c r="P14" s="42"/>
-      <c r="S14" s="43"/>
-      <c r="T14" s="41"/>
-      <c r="U14" s="41"/>
-      <c r="V14" s="41"/>
-      <c r="W14" s="41"/>
-      <c r="X14" s="42"/>
+      <c r="C14" s="40"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="39"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="38"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="38"/>
+      <c r="P14" s="39"/>
+      <c r="S14" s="40"/>
+      <c r="T14" s="38"/>
+      <c r="U14" s="38"/>
+      <c r="V14" s="38"/>
+      <c r="W14" s="38"/>
+      <c r="X14" s="39"/>
     </row>
     <row r="15" spans="3:24">
-      <c r="C15" s="43"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="42"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="41"/>
-      <c r="M15" s="41"/>
-      <c r="N15" s="41"/>
-      <c r="O15" s="41"/>
-      <c r="P15" s="42"/>
-      <c r="S15" s="43"/>
-      <c r="T15" s="41"/>
-      <c r="U15" s="41"/>
-      <c r="V15" s="41"/>
-      <c r="W15" s="41"/>
-      <c r="X15" s="42"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="39"/>
+      <c r="K15" s="40"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="38"/>
+      <c r="N15" s="38"/>
+      <c r="O15" s="38"/>
+      <c r="P15" s="39"/>
+      <c r="S15" s="40"/>
+      <c r="T15" s="38"/>
+      <c r="U15" s="38"/>
+      <c r="V15" s="38"/>
+      <c r="W15" s="38"/>
+      <c r="X15" s="39"/>
     </row>
     <row r="16" spans="3:24">
-      <c r="C16" s="43"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="42"/>
-      <c r="K16" s="43"/>
-      <c r="L16" s="41"/>
-      <c r="M16" s="41"/>
-      <c r="N16" s="41"/>
-      <c r="O16" s="41"/>
-      <c r="P16" s="42"/>
-      <c r="S16" s="43"/>
-      <c r="T16" s="41"/>
-      <c r="U16" s="41"/>
-      <c r="V16" s="41"/>
-      <c r="W16" s="41"/>
-      <c r="X16" s="42"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="39"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="38"/>
+      <c r="N16" s="38"/>
+      <c r="O16" s="38"/>
+      <c r="P16" s="39"/>
+      <c r="S16" s="40"/>
+      <c r="T16" s="38"/>
+      <c r="U16" s="38"/>
+      <c r="V16" s="38"/>
+      <c r="W16" s="38"/>
+      <c r="X16" s="39"/>
     </row>
     <row r="17" spans="3:24">
-      <c r="C17" s="43"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="42"/>
-      <c r="K17" s="43"/>
-      <c r="L17" s="41"/>
-      <c r="M17" s="41"/>
-      <c r="N17" s="41"/>
-      <c r="O17" s="41"/>
-      <c r="P17" s="42"/>
-      <c r="S17" s="43"/>
-      <c r="T17" s="41"/>
-      <c r="U17" s="41"/>
-      <c r="V17" s="41"/>
-      <c r="W17" s="41"/>
-      <c r="X17" s="42"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="39"/>
+      <c r="K17" s="40"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="38"/>
+      <c r="N17" s="38"/>
+      <c r="O17" s="38"/>
+      <c r="P17" s="39"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="38"/>
+      <c r="U17" s="38"/>
+      <c r="V17" s="38"/>
+      <c r="W17" s="38"/>
+      <c r="X17" s="39"/>
     </row>
     <row r="18" spans="3:24">
-      <c r="C18" s="43"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="41"/>
-      <c r="M18" s="41"/>
-      <c r="N18" s="41"/>
-      <c r="O18" s="41"/>
-      <c r="P18" s="42"/>
-      <c r="S18" s="43"/>
-      <c r="T18" s="41"/>
-      <c r="U18" s="41"/>
-      <c r="V18" s="41"/>
-      <c r="W18" s="41"/>
-      <c r="X18" s="42"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="39"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="38"/>
+      <c r="N18" s="38"/>
+      <c r="O18" s="38"/>
+      <c r="P18" s="39"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="38"/>
+      <c r="U18" s="38"/>
+      <c r="V18" s="38"/>
+      <c r="W18" s="38"/>
+      <c r="X18" s="39"/>
     </row>
     <row r="19" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C19" s="44"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="46"/>
-      <c r="K19" s="44"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="45"/>
-      <c r="O19" s="45"/>
-      <c r="P19" s="46"/>
-      <c r="S19" s="44"/>
-      <c r="T19" s="45"/>
-      <c r="U19" s="45"/>
-      <c r="V19" s="45"/>
-      <c r="W19" s="45"/>
-      <c r="X19" s="46"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="43"/>
+      <c r="K19" s="41"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42"/>
+      <c r="N19" s="42"/>
+      <c r="O19" s="42"/>
+      <c r="P19" s="43"/>
+      <c r="S19" s="41"/>
+      <c r="T19" s="42"/>
+      <c r="U19" s="42"/>
+      <c r="V19" s="42"/>
+      <c r="W19" s="42"/>
+      <c r="X19" s="43"/>
     </row>
     <row r="22" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="23" spans="3:24">
-      <c r="C23" s="47" t="s">
+      <c r="C23" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="48"/>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="48"/>
-      <c r="H23" s="49"/>
-      <c r="K23" s="47" t="s">
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="45"/>
+      <c r="H23" s="46"/>
+      <c r="K23" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="L23" s="48"/>
-      <c r="M23" s="48"/>
-      <c r="N23" s="48"/>
-      <c r="O23" s="48"/>
-      <c r="P23" s="49"/>
-      <c r="S23" s="47" t="s">
+      <c r="L23" s="45"/>
+      <c r="M23" s="45"/>
+      <c r="N23" s="45"/>
+      <c r="O23" s="45"/>
+      <c r="P23" s="46"/>
+      <c r="S23" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="T23" s="48"/>
-      <c r="U23" s="48"/>
-      <c r="V23" s="48"/>
-      <c r="W23" s="48"/>
-      <c r="X23" s="49"/>
+      <c r="T23" s="45"/>
+      <c r="U23" s="45"/>
+      <c r="V23" s="45"/>
+      <c r="W23" s="45"/>
+      <c r="X23" s="46"/>
     </row>
     <row r="24" spans="3:24">
-      <c r="C24" s="43"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="42"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="41"/>
-      <c r="O24" s="41"/>
-      <c r="P24" s="42"/>
-      <c r="S24" s="43"/>
-      <c r="T24" s="41"/>
-      <c r="U24" s="41"/>
-      <c r="V24" s="41"/>
-      <c r="W24" s="41"/>
-      <c r="X24" s="42"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="39"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="38"/>
+      <c r="N24" s="38"/>
+      <c r="O24" s="38"/>
+      <c r="P24" s="39"/>
+      <c r="S24" s="40"/>
+      <c r="T24" s="38"/>
+      <c r="U24" s="38"/>
+      <c r="V24" s="38"/>
+      <c r="W24" s="38"/>
+      <c r="X24" s="39"/>
     </row>
     <row r="25" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C25" s="40">
+      <c r="C25" s="37">
         <f>COUNTIF('Flujo de Compra'!G:G,"Si")+COUNTIF('Gestión de Usuario'!G:G,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!G:G,"Si")+COUNTIF(Videollamadas!G:G,"Si")+COUNTIF(Reintegros!G:G,"Si")</f>
         <v>140</v>
       </c>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="41"/>
-      <c r="H25" s="42"/>
-      <c r="K25" s="40">
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="39"/>
+      <c r="K25" s="37">
         <f>COUNTIFS('Flujo de Compra'!G:G,"Si",'Flujo de Compra'!H:H,"Si")+COUNTIFS('Gestión de Usuario'!G:G,"Si",'Gestión de Usuario'!H:H,"Si")+COUNTIFS(Perfil!G:G,"Si",Perfil!H:H,"Si")+COUNTIFS(Credenciales!G:G,"Si",Credenciales!H:H,"Si")+COUNTIFS(Videollamadas!G:G,"Si",Videollamadas!H:H,"Si")+COUNTIFS(Reintegros!G:G,"Si",Reintegros!H:H,"Si")+COUNTIFS(Misceláneas!G:G,"Si",Misceláneas!H:H,"Si")</f>
         <v>109</v>
       </c>
-      <c r="L25" s="41"/>
-      <c r="M25" s="41"/>
-      <c r="N25" s="41"/>
-      <c r="O25" s="41"/>
-      <c r="P25" s="42"/>
-      <c r="S25" s="51">
+      <c r="L25" s="38"/>
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
+      <c r="O25" s="38"/>
+      <c r="P25" s="39"/>
+      <c r="S25" s="48">
         <f>K25/C25</f>
         <v>0.77857142857142858</v>
       </c>
-      <c r="T25" s="41"/>
-      <c r="U25" s="41"/>
-      <c r="V25" s="41"/>
-      <c r="W25" s="41"/>
-      <c r="X25" s="42"/>
+      <c r="T25" s="38"/>
+      <c r="U25" s="38"/>
+      <c r="V25" s="38"/>
+      <c r="W25" s="38"/>
+      <c r="X25" s="39"/>
     </row>
     <row r="26" spans="3:24">
-      <c r="C26" s="43"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="42"/>
-      <c r="K26" s="43"/>
-      <c r="L26" s="41"/>
-      <c r="M26" s="41"/>
-      <c r="N26" s="41"/>
-      <c r="O26" s="41"/>
-      <c r="P26" s="42"/>
-      <c r="S26" s="43"/>
-      <c r="T26" s="41"/>
-      <c r="U26" s="41"/>
-      <c r="V26" s="41"/>
-      <c r="W26" s="41"/>
-      <c r="X26" s="42"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="39"/>
+      <c r="K26" s="40"/>
+      <c r="L26" s="38"/>
+      <c r="M26" s="38"/>
+      <c r="N26" s="38"/>
+      <c r="O26" s="38"/>
+      <c r="P26" s="39"/>
+      <c r="S26" s="40"/>
+      <c r="T26" s="38"/>
+      <c r="U26" s="38"/>
+      <c r="V26" s="38"/>
+      <c r="W26" s="38"/>
+      <c r="X26" s="39"/>
     </row>
     <row r="27" spans="3:24">
-      <c r="C27" s="43"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="41"/>
-      <c r="M27" s="41"/>
-      <c r="N27" s="41"/>
-      <c r="O27" s="41"/>
-      <c r="P27" s="42"/>
-      <c r="S27" s="43"/>
-      <c r="T27" s="41"/>
-      <c r="U27" s="41"/>
-      <c r="V27" s="41"/>
-      <c r="W27" s="41"/>
-      <c r="X27" s="42"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="39"/>
+      <c r="K27" s="40"/>
+      <c r="L27" s="38"/>
+      <c r="M27" s="38"/>
+      <c r="N27" s="38"/>
+      <c r="O27" s="38"/>
+      <c r="P27" s="39"/>
+      <c r="S27" s="40"/>
+      <c r="T27" s="38"/>
+      <c r="U27" s="38"/>
+      <c r="V27" s="38"/>
+      <c r="W27" s="38"/>
+      <c r="X27" s="39"/>
     </row>
     <row r="28" spans="3:24">
-      <c r="C28" s="43"/>
-      <c r="D28" s="41"/>
-      <c r="E28" s="41"/>
-      <c r="F28" s="41"/>
-      <c r="G28" s="41"/>
-      <c r="H28" s="42"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="41"/>
-      <c r="M28" s="41"/>
-      <c r="N28" s="41"/>
-      <c r="O28" s="41"/>
-      <c r="P28" s="42"/>
-      <c r="S28" s="43"/>
-      <c r="T28" s="41"/>
-      <c r="U28" s="41"/>
-      <c r="V28" s="41"/>
-      <c r="W28" s="41"/>
-      <c r="X28" s="42"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="39"/>
+      <c r="K28" s="40"/>
+      <c r="L28" s="38"/>
+      <c r="M28" s="38"/>
+      <c r="N28" s="38"/>
+      <c r="O28" s="38"/>
+      <c r="P28" s="39"/>
+      <c r="S28" s="40"/>
+      <c r="T28" s="38"/>
+      <c r="U28" s="38"/>
+      <c r="V28" s="38"/>
+      <c r="W28" s="38"/>
+      <c r="X28" s="39"/>
     </row>
     <row r="29" spans="3:24">
-      <c r="C29" s="43"/>
-      <c r="D29" s="41"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="41"/>
-      <c r="G29" s="41"/>
-      <c r="H29" s="42"/>
-      <c r="K29" s="43"/>
-      <c r="L29" s="41"/>
-      <c r="M29" s="41"/>
-      <c r="N29" s="41"/>
-      <c r="O29" s="41"/>
-      <c r="P29" s="42"/>
-      <c r="S29" s="43"/>
-      <c r="T29" s="41"/>
-      <c r="U29" s="41"/>
-      <c r="V29" s="41"/>
-      <c r="W29" s="41"/>
-      <c r="X29" s="42"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="39"/>
+      <c r="K29" s="40"/>
+      <c r="L29" s="38"/>
+      <c r="M29" s="38"/>
+      <c r="N29" s="38"/>
+      <c r="O29" s="38"/>
+      <c r="P29" s="39"/>
+      <c r="S29" s="40"/>
+      <c r="T29" s="38"/>
+      <c r="U29" s="38"/>
+      <c r="V29" s="38"/>
+      <c r="W29" s="38"/>
+      <c r="X29" s="39"/>
     </row>
     <row r="30" spans="3:24">
-      <c r="C30" s="43"/>
-      <c r="D30" s="41"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="41"/>
-      <c r="H30" s="42"/>
-      <c r="K30" s="43"/>
-      <c r="L30" s="41"/>
-      <c r="M30" s="41"/>
-      <c r="N30" s="41"/>
-      <c r="O30" s="41"/>
-      <c r="P30" s="42"/>
-      <c r="S30" s="43"/>
-      <c r="T30" s="41"/>
-      <c r="U30" s="41"/>
-      <c r="V30" s="41"/>
-      <c r="W30" s="41"/>
-      <c r="X30" s="42"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="39"/>
+      <c r="K30" s="40"/>
+      <c r="L30" s="38"/>
+      <c r="M30" s="38"/>
+      <c r="N30" s="38"/>
+      <c r="O30" s="38"/>
+      <c r="P30" s="39"/>
+      <c r="S30" s="40"/>
+      <c r="T30" s="38"/>
+      <c r="U30" s="38"/>
+      <c r="V30" s="38"/>
+      <c r="W30" s="38"/>
+      <c r="X30" s="39"/>
     </row>
     <row r="31" spans="3:24">
-      <c r="C31" s="43"/>
-      <c r="D31" s="41"/>
-      <c r="E31" s="41"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="41"/>
-      <c r="H31" s="42"/>
-      <c r="K31" s="43"/>
-      <c r="L31" s="41"/>
-      <c r="M31" s="41"/>
-      <c r="N31" s="41"/>
-      <c r="O31" s="41"/>
-      <c r="P31" s="42"/>
-      <c r="S31" s="43"/>
-      <c r="T31" s="41"/>
-      <c r="U31" s="41"/>
-      <c r="V31" s="41"/>
-      <c r="W31" s="41"/>
-      <c r="X31" s="42"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="39"/>
+      <c r="K31" s="40"/>
+      <c r="L31" s="38"/>
+      <c r="M31" s="38"/>
+      <c r="N31" s="38"/>
+      <c r="O31" s="38"/>
+      <c r="P31" s="39"/>
+      <c r="S31" s="40"/>
+      <c r="T31" s="38"/>
+      <c r="U31" s="38"/>
+      <c r="V31" s="38"/>
+      <c r="W31" s="38"/>
+      <c r="X31" s="39"/>
     </row>
     <row r="32" spans="3:24">
-      <c r="C32" s="43"/>
-      <c r="D32" s="41"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="41"/>
-      <c r="H32" s="42"/>
-      <c r="K32" s="43"/>
-      <c r="L32" s="41"/>
-      <c r="M32" s="41"/>
-      <c r="N32" s="41"/>
-      <c r="O32" s="41"/>
-      <c r="P32" s="42"/>
-      <c r="S32" s="43"/>
-      <c r="T32" s="41"/>
-      <c r="U32" s="41"/>
-      <c r="V32" s="41"/>
-      <c r="W32" s="41"/>
-      <c r="X32" s="42"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="39"/>
+      <c r="K32" s="40"/>
+      <c r="L32" s="38"/>
+      <c r="M32" s="38"/>
+      <c r="N32" s="38"/>
+      <c r="O32" s="38"/>
+      <c r="P32" s="39"/>
+      <c r="S32" s="40"/>
+      <c r="T32" s="38"/>
+      <c r="U32" s="38"/>
+      <c r="V32" s="38"/>
+      <c r="W32" s="38"/>
+      <c r="X32" s="39"/>
     </row>
     <row r="33" spans="3:24">
-      <c r="C33" s="43"/>
-      <c r="D33" s="41"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="42"/>
-      <c r="K33" s="43"/>
-      <c r="L33" s="41"/>
-      <c r="M33" s="41"/>
-      <c r="N33" s="41"/>
-      <c r="O33" s="41"/>
-      <c r="P33" s="42"/>
-      <c r="S33" s="43"/>
-      <c r="T33" s="41"/>
-      <c r="U33" s="41"/>
-      <c r="V33" s="41"/>
-      <c r="W33" s="41"/>
-      <c r="X33" s="42"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="39"/>
+      <c r="K33" s="40"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="38"/>
+      <c r="N33" s="38"/>
+      <c r="O33" s="38"/>
+      <c r="P33" s="39"/>
+      <c r="S33" s="40"/>
+      <c r="T33" s="38"/>
+      <c r="U33" s="38"/>
+      <c r="V33" s="38"/>
+      <c r="W33" s="38"/>
+      <c r="X33" s="39"/>
     </row>
     <row r="34" spans="3:24">
-      <c r="C34" s="43"/>
-      <c r="D34" s="41"/>
-      <c r="E34" s="41"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="41"/>
-      <c r="H34" s="42"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="41"/>
-      <c r="M34" s="41"/>
-      <c r="N34" s="41"/>
-      <c r="O34" s="41"/>
-      <c r="P34" s="42"/>
-      <c r="S34" s="43"/>
-      <c r="T34" s="41"/>
-      <c r="U34" s="41"/>
-      <c r="V34" s="41"/>
-      <c r="W34" s="41"/>
-      <c r="X34" s="42"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="39"/>
+      <c r="K34" s="40"/>
+      <c r="L34" s="38"/>
+      <c r="M34" s="38"/>
+      <c r="N34" s="38"/>
+      <c r="O34" s="38"/>
+      <c r="P34" s="39"/>
+      <c r="S34" s="40"/>
+      <c r="T34" s="38"/>
+      <c r="U34" s="38"/>
+      <c r="V34" s="38"/>
+      <c r="W34" s="38"/>
+      <c r="X34" s="39"/>
     </row>
     <row r="35" spans="3:24">
-      <c r="C35" s="43"/>
-      <c r="D35" s="41"/>
-      <c r="E35" s="41"/>
-      <c r="F35" s="41"/>
-      <c r="G35" s="41"/>
-      <c r="H35" s="42"/>
-      <c r="K35" s="43"/>
-      <c r="L35" s="41"/>
-      <c r="M35" s="41"/>
-      <c r="N35" s="41"/>
-      <c r="O35" s="41"/>
-      <c r="P35" s="42"/>
-      <c r="S35" s="43"/>
-      <c r="T35" s="41"/>
-      <c r="U35" s="41"/>
-      <c r="V35" s="41"/>
-      <c r="W35" s="41"/>
-      <c r="X35" s="42"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="39"/>
+      <c r="K35" s="40"/>
+      <c r="L35" s="38"/>
+      <c r="M35" s="38"/>
+      <c r="N35" s="38"/>
+      <c r="O35" s="38"/>
+      <c r="P35" s="39"/>
+      <c r="S35" s="40"/>
+      <c r="T35" s="38"/>
+      <c r="U35" s="38"/>
+      <c r="V35" s="38"/>
+      <c r="W35" s="38"/>
+      <c r="X35" s="39"/>
     </row>
     <row r="36" spans="3:24">
-      <c r="C36" s="43"/>
-      <c r="D36" s="41"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="41"/>
-      <c r="H36" s="42"/>
-      <c r="K36" s="43"/>
-      <c r="L36" s="41"/>
-      <c r="M36" s="41"/>
-      <c r="N36" s="41"/>
-      <c r="O36" s="41"/>
-      <c r="P36" s="42"/>
-      <c r="S36" s="43"/>
-      <c r="T36" s="41"/>
-      <c r="U36" s="41"/>
-      <c r="V36" s="41"/>
-      <c r="W36" s="41"/>
-      <c r="X36" s="42"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="39"/>
+      <c r="K36" s="40"/>
+      <c r="L36" s="38"/>
+      <c r="M36" s="38"/>
+      <c r="N36" s="38"/>
+      <c r="O36" s="38"/>
+      <c r="P36" s="39"/>
+      <c r="S36" s="40"/>
+      <c r="T36" s="38"/>
+      <c r="U36" s="38"/>
+      <c r="V36" s="38"/>
+      <c r="W36" s="38"/>
+      <c r="X36" s="39"/>
     </row>
     <row r="37" spans="3:24">
-      <c r="C37" s="43"/>
-      <c r="D37" s="41"/>
-      <c r="E37" s="41"/>
-      <c r="F37" s="41"/>
-      <c r="G37" s="41"/>
-      <c r="H37" s="42"/>
-      <c r="K37" s="43"/>
-      <c r="L37" s="41"/>
-      <c r="M37" s="41"/>
-      <c r="N37" s="41"/>
-      <c r="O37" s="41"/>
-      <c r="P37" s="42"/>
-      <c r="S37" s="43"/>
-      <c r="T37" s="41"/>
-      <c r="U37" s="41"/>
-      <c r="V37" s="41"/>
-      <c r="W37" s="41"/>
-      <c r="X37" s="42"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="39"/>
+      <c r="K37" s="40"/>
+      <c r="L37" s="38"/>
+      <c r="M37" s="38"/>
+      <c r="N37" s="38"/>
+      <c r="O37" s="38"/>
+      <c r="P37" s="39"/>
+      <c r="S37" s="40"/>
+      <c r="T37" s="38"/>
+      <c r="U37" s="38"/>
+      <c r="V37" s="38"/>
+      <c r="W37" s="38"/>
+      <c r="X37" s="39"/>
     </row>
     <row r="38" spans="3:24">
-      <c r="C38" s="43"/>
-      <c r="D38" s="41"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="41"/>
-      <c r="G38" s="41"/>
-      <c r="H38" s="42"/>
-      <c r="K38" s="43"/>
-      <c r="L38" s="41"/>
-      <c r="M38" s="41"/>
-      <c r="N38" s="41"/>
-      <c r="O38" s="41"/>
-      <c r="P38" s="42"/>
-      <c r="S38" s="43"/>
-      <c r="T38" s="41"/>
-      <c r="U38" s="41"/>
-      <c r="V38" s="41"/>
-      <c r="W38" s="41"/>
-      <c r="X38" s="42"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="39"/>
+      <c r="K38" s="40"/>
+      <c r="L38" s="38"/>
+      <c r="M38" s="38"/>
+      <c r="N38" s="38"/>
+      <c r="O38" s="38"/>
+      <c r="P38" s="39"/>
+      <c r="S38" s="40"/>
+      <c r="T38" s="38"/>
+      <c r="U38" s="38"/>
+      <c r="V38" s="38"/>
+      <c r="W38" s="38"/>
+      <c r="X38" s="39"/>
     </row>
     <row r="39" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C39" s="44"/>
-      <c r="D39" s="45"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="46"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="45"/>
-      <c r="M39" s="45"/>
-      <c r="N39" s="45"/>
-      <c r="O39" s="45"/>
-      <c r="P39" s="46"/>
-      <c r="S39" s="44"/>
-      <c r="T39" s="45"/>
-      <c r="U39" s="45"/>
-      <c r="V39" s="45"/>
-      <c r="W39" s="45"/>
-      <c r="X39" s="46"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+      <c r="H39" s="43"/>
+      <c r="K39" s="41"/>
+      <c r="L39" s="42"/>
+      <c r="M39" s="42"/>
+      <c r="N39" s="42"/>
+      <c r="O39" s="42"/>
+      <c r="P39" s="43"/>
+      <c r="S39" s="41"/>
+      <c r="T39" s="42"/>
+      <c r="U39" s="42"/>
+      <c r="V39" s="42"/>
+      <c r="W39" s="42"/>
+      <c r="X39" s="43"/>
     </row>
     <row r="41" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="42" spans="3:24">
-      <c r="C42" s="47" t="s">
+      <c r="C42" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="48"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="48"/>
-      <c r="H42" s="49"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="45"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="46"/>
     </row>
     <row r="43" spans="3:24">
-      <c r="C43" s="43"/>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="41"/>
-      <c r="H43" s="42"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="39"/>
       <c r="K43" s="28"/>
       <c r="L43" s="28"/>
       <c r="M43" s="28"/>
@@ -5259,31 +5278,31 @@
       <c r="P43" s="28"/>
     </row>
     <row r="44" spans="3:24" ht="21" customHeight="1">
-      <c r="C44" s="51">
+      <c r="C44" s="48">
         <f>C25/C5</f>
-        <v>0.55335968379446643</v>
-      </c>
-      <c r="D44" s="41"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="42"/>
+        <v>0.55118110236220474</v>
+      </c>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="39"/>
       <c r="K44" s="28"/>
-      <c r="L44" s="50" t="s">
+      <c r="L44" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="M44" s="41"/>
-      <c r="N44" s="41"/>
-      <c r="O44" s="41"/>
+      <c r="M44" s="38"/>
+      <c r="N44" s="38"/>
+      <c r="O44" s="38"/>
       <c r="P44" s="29"/>
     </row>
     <row r="45" spans="3:24">
-      <c r="C45" s="43"/>
-      <c r="D45" s="41"/>
-      <c r="E45" s="41"/>
-      <c r="F45" s="41"/>
-      <c r="G45" s="41"/>
-      <c r="H45" s="42"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38"/>
+      <c r="F45" s="38"/>
+      <c r="G45" s="38"/>
+      <c r="H45" s="39"/>
       <c r="K45" s="28"/>
       <c r="L45" s="30"/>
       <c r="M45" s="30"/>
@@ -5292,12 +5311,12 @@
       <c r="P45" s="29"/>
     </row>
     <row r="46" spans="3:24">
-      <c r="C46" s="43"/>
-      <c r="D46" s="41"/>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="42"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="39"/>
       <c r="K46" s="28"/>
       <c r="L46" s="31"/>
       <c r="M46" s="28" t="s">
@@ -5308,12 +5327,12 @@
       <c r="P46" s="28"/>
     </row>
     <row r="47" spans="3:24">
-      <c r="C47" s="43"/>
-      <c r="D47" s="41"/>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="42"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="38"/>
+      <c r="G47" s="38"/>
+      <c r="H47" s="39"/>
       <c r="K47" s="28"/>
       <c r="L47" s="32"/>
       <c r="M47" s="28" t="s">
@@ -5324,12 +5343,12 @@
       <c r="P47" s="28"/>
     </row>
     <row r="48" spans="3:24">
-      <c r="C48" s="43"/>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="42"/>
+      <c r="C48" s="40"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="39"/>
       <c r="K48" s="28"/>
       <c r="L48" s="33"/>
       <c r="M48" s="28" t="s">
@@ -5340,12 +5359,12 @@
       <c r="P48" s="28"/>
     </row>
     <row r="49" spans="3:16">
-      <c r="C49" s="43"/>
-      <c r="D49" s="41"/>
-      <c r="E49" s="41"/>
-      <c r="F49" s="41"/>
-      <c r="G49" s="41"/>
-      <c r="H49" s="42"/>
+      <c r="C49" s="40"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="39"/>
       <c r="K49" s="28"/>
       <c r="L49" s="34"/>
       <c r="M49" s="28" t="s">
@@ -5356,12 +5375,12 @@
       <c r="P49" s="28"/>
     </row>
     <row r="50" spans="3:16">
-      <c r="C50" s="43"/>
-      <c r="D50" s="41"/>
-      <c r="E50" s="41"/>
-      <c r="F50" s="41"/>
-      <c r="G50" s="41"/>
-      <c r="H50" s="42"/>
+      <c r="C50" s="40"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38"/>
+      <c r="F50" s="38"/>
+      <c r="G50" s="38"/>
+      <c r="H50" s="39"/>
       <c r="K50" s="28"/>
       <c r="L50" s="35"/>
       <c r="M50" s="28" t="s">
@@ -5372,12 +5391,12 @@
       <c r="P50" s="28"/>
     </row>
     <row r="51" spans="3:16">
-      <c r="C51" s="43"/>
-      <c r="D51" s="41"/>
-      <c r="E51" s="41"/>
-      <c r="F51" s="41"/>
-      <c r="G51" s="41"/>
-      <c r="H51" s="42"/>
+      <c r="C51" s="40"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="38"/>
+      <c r="F51" s="38"/>
+      <c r="G51" s="38"/>
+      <c r="H51" s="39"/>
       <c r="K51" s="28"/>
       <c r="L51" s="28"/>
       <c r="M51" s="28"/>
@@ -5386,230 +5405,230 @@
       <c r="P51" s="28"/>
     </row>
     <row r="52" spans="3:16">
-      <c r="C52" s="43"/>
-      <c r="D52" s="41"/>
-      <c r="E52" s="41"/>
-      <c r="F52" s="41"/>
-      <c r="G52" s="41"/>
-      <c r="H52" s="42"/>
+      <c r="C52" s="40"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="38"/>
+      <c r="F52" s="38"/>
+      <c r="G52" s="38"/>
+      <c r="H52" s="39"/>
     </row>
     <row r="53" spans="3:16">
-      <c r="C53" s="43"/>
-      <c r="D53" s="41"/>
-      <c r="E53" s="41"/>
-      <c r="F53" s="41"/>
-      <c r="G53" s="41"/>
-      <c r="H53" s="42"/>
+      <c r="C53" s="40"/>
+      <c r="D53" s="38"/>
+      <c r="E53" s="38"/>
+      <c r="F53" s="38"/>
+      <c r="G53" s="38"/>
+      <c r="H53" s="39"/>
     </row>
     <row r="54" spans="3:16">
-      <c r="C54" s="43"/>
-      <c r="D54" s="41"/>
-      <c r="E54" s="41"/>
-      <c r="F54" s="41"/>
-      <c r="G54" s="41"/>
-      <c r="H54" s="42"/>
+      <c r="C54" s="40"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="38"/>
+      <c r="F54" s="38"/>
+      <c r="G54" s="38"/>
+      <c r="H54" s="39"/>
     </row>
     <row r="55" spans="3:16">
-      <c r="C55" s="43"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-      <c r="F55" s="41"/>
-      <c r="G55" s="41"/>
-      <c r="H55" s="42"/>
+      <c r="C55" s="40"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="38"/>
+      <c r="F55" s="38"/>
+      <c r="G55" s="38"/>
+      <c r="H55" s="39"/>
     </row>
     <row r="56" spans="3:16">
-      <c r="C56" s="43"/>
-      <c r="D56" s="41"/>
-      <c r="E56" s="41"/>
-      <c r="F56" s="41"/>
-      <c r="G56" s="41"/>
-      <c r="H56" s="42"/>
+      <c r="C56" s="40"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
+      <c r="G56" s="38"/>
+      <c r="H56" s="39"/>
     </row>
     <row r="57" spans="3:16">
-      <c r="C57" s="43"/>
-      <c r="D57" s="41"/>
-      <c r="E57" s="41"/>
-      <c r="F57" s="41"/>
-      <c r="G57" s="41"/>
-      <c r="H57" s="42"/>
+      <c r="C57" s="40"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="39"/>
     </row>
     <row r="58" spans="3:16" ht="15.75" customHeight="1">
-      <c r="C58" s="44"/>
-      <c r="D58" s="45"/>
-      <c r="E58" s="45"/>
-      <c r="F58" s="45"/>
-      <c r="G58" s="45"/>
-      <c r="H58" s="46"/>
+      <c r="C58" s="41"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="42"/>
+      <c r="F58" s="42"/>
+      <c r="G58" s="42"/>
+      <c r="H58" s="43"/>
     </row>
     <row r="62" spans="3:16">
-      <c r="C62" s="37" t="s">
+      <c r="C62" s="49" t="s">
         <v>585</v>
       </c>
-      <c r="D62" s="37"/>
-      <c r="E62" s="37"/>
-      <c r="F62" s="37"/>
-      <c r="H62" s="37" t="s">
+      <c r="D62" s="49"/>
+      <c r="E62" s="49"/>
+      <c r="F62" s="49"/>
+      <c r="H62" s="49" t="s">
         <v>586</v>
       </c>
-      <c r="I62" s="37"/>
-      <c r="J62" s="37"/>
-      <c r="K62" s="37"/>
-      <c r="M62" s="37" t="s">
+      <c r="I62" s="49"/>
+      <c r="J62" s="49"/>
+      <c r="K62" s="49"/>
+      <c r="M62" s="49" t="s">
         <v>587</v>
       </c>
-      <c r="N62" s="37"/>
-      <c r="O62" s="37"/>
-      <c r="P62" s="37"/>
+      <c r="N62" s="49"/>
+      <c r="O62" s="49"/>
+      <c r="P62" s="49"/>
     </row>
     <row r="63" spans="3:16">
-      <c r="C63" s="37"/>
-      <c r="D63" s="37"/>
-      <c r="E63" s="37"/>
-      <c r="F63" s="37"/>
-      <c r="H63" s="37"/>
-      <c r="I63" s="37"/>
-      <c r="J63" s="37"/>
-      <c r="K63" s="37"/>
-      <c r="M63" s="37"/>
-      <c r="N63" s="37"/>
-      <c r="O63" s="37"/>
-      <c r="P63" s="37"/>
+      <c r="C63" s="49"/>
+      <c r="D63" s="49"/>
+      <c r="E63" s="49"/>
+      <c r="F63" s="49"/>
+      <c r="H63" s="49"/>
+      <c r="I63" s="49"/>
+      <c r="J63" s="49"/>
+      <c r="K63" s="49"/>
+      <c r="M63" s="49"/>
+      <c r="N63" s="49"/>
+      <c r="O63" s="49"/>
+      <c r="P63" s="49"/>
     </row>
     <row r="64" spans="3:16">
-      <c r="C64" s="38">
+      <c r="C64" s="50">
         <f>COUNTIF('Flujo de Compra'!I:I,"Si")+COUNTIF('Gestión de Usuario'!I:I,"Si")+COUNTIF(Perfil!J:J,"Si")+COUNTIF(Credenciales!J:J,"Si")+COUNTIF(Videollamadas!J:J,"Si")</f>
         <v>250</v>
       </c>
-      <c r="D64" s="38"/>
-      <c r="E64" s="38"/>
-      <c r="F64" s="38"/>
-      <c r="H64" s="38">
+      <c r="D64" s="50"/>
+      <c r="E64" s="50"/>
+      <c r="F64" s="50"/>
+      <c r="H64" s="50">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")</f>
         <v>188</v>
       </c>
-      <c r="I64" s="38"/>
-      <c r="J64" s="38"/>
-      <c r="K64" s="38"/>
-      <c r="M64" s="39">
+      <c r="I64" s="50"/>
+      <c r="J64" s="50"/>
+      <c r="K64" s="50"/>
+      <c r="M64" s="51">
         <f t="shared" ref="M64" si="0">H64/C64</f>
         <v>0.752</v>
       </c>
-      <c r="N64" s="39"/>
-      <c r="O64" s="39"/>
-      <c r="P64" s="39"/>
+      <c r="N64" s="51"/>
+      <c r="O64" s="51"/>
+      <c r="P64" s="51"/>
     </row>
     <row r="65" spans="3:16">
-      <c r="C65" s="38"/>
-      <c r="D65" s="38"/>
-      <c r="E65" s="38"/>
-      <c r="F65" s="38"/>
-      <c r="H65" s="38"/>
-      <c r="I65" s="38"/>
-      <c r="J65" s="38"/>
-      <c r="K65" s="38"/>
-      <c r="M65" s="39"/>
-      <c r="N65" s="39"/>
-      <c r="O65" s="39"/>
-      <c r="P65" s="39"/>
+      <c r="C65" s="50"/>
+      <c r="D65" s="50"/>
+      <c r="E65" s="50"/>
+      <c r="F65" s="50"/>
+      <c r="H65" s="50"/>
+      <c r="I65" s="50"/>
+      <c r="J65" s="50"/>
+      <c r="K65" s="50"/>
+      <c r="M65" s="51"/>
+      <c r="N65" s="51"/>
+      <c r="O65" s="51"/>
+      <c r="P65" s="51"/>
     </row>
     <row r="66" spans="3:16">
-      <c r="C66" s="38"/>
-      <c r="D66" s="38"/>
-      <c r="E66" s="38"/>
-      <c r="F66" s="38"/>
-      <c r="H66" s="38"/>
-      <c r="I66" s="38"/>
-      <c r="J66" s="38"/>
-      <c r="K66" s="38"/>
-      <c r="M66" s="39"/>
-      <c r="N66" s="39"/>
-      <c r="O66" s="39"/>
-      <c r="P66" s="39"/>
+      <c r="C66" s="50"/>
+      <c r="D66" s="50"/>
+      <c r="E66" s="50"/>
+      <c r="F66" s="50"/>
+      <c r="H66" s="50"/>
+      <c r="I66" s="50"/>
+      <c r="J66" s="50"/>
+      <c r="K66" s="50"/>
+      <c r="M66" s="51"/>
+      <c r="N66" s="51"/>
+      <c r="O66" s="51"/>
+      <c r="P66" s="51"/>
     </row>
     <row r="69" spans="3:16">
-      <c r="C69" s="37" t="s">
+      <c r="C69" s="49" t="s">
         <v>588</v>
       </c>
-      <c r="D69" s="37"/>
-      <c r="E69" s="37"/>
-      <c r="F69" s="37"/>
-      <c r="H69" s="37" t="s">
+      <c r="D69" s="49"/>
+      <c r="E69" s="49"/>
+      <c r="F69" s="49"/>
+      <c r="H69" s="49" t="s">
         <v>589</v>
       </c>
-      <c r="I69" s="37"/>
-      <c r="J69" s="37"/>
-      <c r="K69" s="37"/>
-      <c r="M69" s="37" t="s">
+      <c r="I69" s="49"/>
+      <c r="J69" s="49"/>
+      <c r="K69" s="49"/>
+      <c r="M69" s="49" t="s">
         <v>587</v>
       </c>
-      <c r="N69" s="37"/>
-      <c r="O69" s="37"/>
-      <c r="P69" s="37"/>
+      <c r="N69" s="49"/>
+      <c r="O69" s="49"/>
+      <c r="P69" s="49"/>
     </row>
     <row r="70" spans="3:16">
-      <c r="C70" s="37"/>
-      <c r="D70" s="37"/>
-      <c r="E70" s="37"/>
-      <c r="F70" s="37"/>
-      <c r="H70" s="37"/>
-      <c r="I70" s="37"/>
-      <c r="J70" s="37"/>
-      <c r="K70" s="37"/>
-      <c r="M70" s="37"/>
-      <c r="N70" s="37"/>
-      <c r="O70" s="37"/>
-      <c r="P70" s="37"/>
+      <c r="C70" s="49"/>
+      <c r="D70" s="49"/>
+      <c r="E70" s="49"/>
+      <c r="F70" s="49"/>
+      <c r="H70" s="49"/>
+      <c r="I70" s="49"/>
+      <c r="J70" s="49"/>
+      <c r="K70" s="49"/>
+      <c r="M70" s="49"/>
+      <c r="N70" s="49"/>
+      <c r="O70" s="49"/>
+      <c r="P70" s="49"/>
     </row>
     <row r="71" spans="3:16">
-      <c r="C71" s="38">
+      <c r="C71" s="50">
         <f>COUNTIF(Perfil!K:K,"Si")+COUNTIF(Credenciales!K:K,"Si")+COUNTIF(Videollamadas!K:K,"Si")</f>
         <v>71</v>
       </c>
-      <c r="D71" s="38"/>
-      <c r="E71" s="38"/>
-      <c r="F71" s="38"/>
-      <c r="H71" s="38">
+      <c r="D71" s="50"/>
+      <c r="E71" s="50"/>
+      <c r="F71" s="50"/>
+      <c r="H71" s="50">
         <f>COUNTIF(Perfil!I:I,"Si")+COUNTIF(Credenciales!I:I,"Si")+COUNTIF(Videollamadas!I:I,"Si")</f>
         <v>60</v>
       </c>
-      <c r="I71" s="38"/>
-      <c r="J71" s="38"/>
-      <c r="K71" s="38"/>
-      <c r="M71" s="39">
+      <c r="I71" s="50"/>
+      <c r="J71" s="50"/>
+      <c r="K71" s="50"/>
+      <c r="M71" s="51">
         <f t="shared" ref="M71" si="1">H71/C71</f>
         <v>0.84507042253521125</v>
       </c>
-      <c r="N71" s="39"/>
-      <c r="O71" s="39"/>
-      <c r="P71" s="39"/>
+      <c r="N71" s="51"/>
+      <c r="O71" s="51"/>
+      <c r="P71" s="51"/>
     </row>
     <row r="72" spans="3:16">
-      <c r="C72" s="38"/>
-      <c r="D72" s="38"/>
-      <c r="E72" s="38"/>
-      <c r="F72" s="38"/>
-      <c r="H72" s="38"/>
-      <c r="I72" s="38"/>
-      <c r="J72" s="38"/>
-      <c r="K72" s="38"/>
-      <c r="M72" s="39"/>
-      <c r="N72" s="39"/>
-      <c r="O72" s="39"/>
-      <c r="P72" s="39"/>
+      <c r="C72" s="50"/>
+      <c r="D72" s="50"/>
+      <c r="E72" s="50"/>
+      <c r="F72" s="50"/>
+      <c r="H72" s="50"/>
+      <c r="I72" s="50"/>
+      <c r="J72" s="50"/>
+      <c r="K72" s="50"/>
+      <c r="M72" s="51"/>
+      <c r="N72" s="51"/>
+      <c r="O72" s="51"/>
+      <c r="P72" s="51"/>
     </row>
     <row r="73" spans="3:16">
-      <c r="C73" s="38"/>
-      <c r="D73" s="38"/>
-      <c r="E73" s="38"/>
-      <c r="F73" s="38"/>
-      <c r="H73" s="38"/>
-      <c r="I73" s="38"/>
-      <c r="J73" s="38"/>
-      <c r="K73" s="38"/>
-      <c r="M73" s="39"/>
-      <c r="N73" s="39"/>
-      <c r="O73" s="39"/>
-      <c r="P73" s="39"/>
+      <c r="C73" s="50"/>
+      <c r="D73" s="50"/>
+      <c r="E73" s="50"/>
+      <c r="F73" s="50"/>
+      <c r="H73" s="50"/>
+      <c r="I73" s="50"/>
+      <c r="J73" s="50"/>
+      <c r="K73" s="50"/>
+      <c r="M73" s="51"/>
+      <c r="N73" s="51"/>
+      <c r="O73" s="51"/>
+      <c r="P73" s="51"/>
     </row>
     <row r="76" spans="3:16">
       <c r="C76" s="36" t="s">
@@ -5618,6 +5637,18 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C69:F70"/>
+    <mergeCell ref="C71:F73"/>
+    <mergeCell ref="H69:K70"/>
+    <mergeCell ref="H71:K73"/>
+    <mergeCell ref="M69:P70"/>
+    <mergeCell ref="M71:P73"/>
+    <mergeCell ref="C62:F63"/>
+    <mergeCell ref="C64:F66"/>
+    <mergeCell ref="H62:K63"/>
+    <mergeCell ref="H64:K66"/>
+    <mergeCell ref="M62:P63"/>
+    <mergeCell ref="M64:P66"/>
     <mergeCell ref="K5:P19"/>
     <mergeCell ref="K25:P39"/>
     <mergeCell ref="S3:X4"/>
@@ -5633,18 +5664,6 @@
     <mergeCell ref="C3:H4"/>
     <mergeCell ref="C25:H39"/>
     <mergeCell ref="K23:P24"/>
-    <mergeCell ref="C62:F63"/>
-    <mergeCell ref="C64:F66"/>
-    <mergeCell ref="H62:K63"/>
-    <mergeCell ref="H64:K66"/>
-    <mergeCell ref="M62:P63"/>
-    <mergeCell ref="M64:P66"/>
-    <mergeCell ref="C69:F70"/>
-    <mergeCell ref="C71:F73"/>
-    <mergeCell ref="H69:K70"/>
-    <mergeCell ref="H71:K73"/>
-    <mergeCell ref="M69:P70"/>
-    <mergeCell ref="M71:P73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5701,7 +5720,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="52" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="53"/>
@@ -5710,7 +5729,7 @@
       <c r="E2" s="53"/>
       <c r="F2" s="53"/>
       <c r="G2" s="53"/>
-      <c r="H2" s="56"/>
+      <c r="H2" s="54"/>
       <c r="I2" s="12" t="s">
         <v>27</v>
       </c>
@@ -5719,7 +5738,7 @@
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="56" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -5947,7 +5966,7 @@
       <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="52" t="s">
+      <c r="B12" s="55" t="s">
         <v>51</v>
       </c>
       <c r="C12" s="22" t="s">
@@ -6013,7 +6032,7 @@
       <c r="A15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="54" t="s">
+      <c r="B15" s="56" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -6106,7 +6125,7 @@
       <c r="A19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="52" t="s">
+      <c r="B19" s="55" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="22" t="s">
@@ -6307,7 +6326,7 @@
       <c r="A27" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="54" t="s">
+      <c r="B27" s="56" t="s">
         <v>90</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -6427,7 +6446,7 @@
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="52" t="s">
+      <c r="B32" s="55" t="s">
         <v>104</v>
       </c>
       <c r="C32" s="22" t="s">
@@ -6574,7 +6593,7 @@
       <c r="A38" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="54" t="s">
+      <c r="B38" s="56" t="s">
         <v>120</v>
       </c>
       <c r="C38" s="18" t="s">
@@ -6627,7 +6646,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A40" s="55" t="s">
+      <c r="A40" s="52" t="s">
         <v>127</v>
       </c>
       <c r="B40" s="53"/>
@@ -6636,7 +6655,7 @@
       <c r="E40" s="53"/>
       <c r="F40" s="53"/>
       <c r="G40" s="53"/>
-      <c r="H40" s="56"/>
+      <c r="H40" s="54"/>
       <c r="I40" s="12" t="s">
         <v>27</v>
       </c>
@@ -6645,7 +6664,7 @@
       <c r="A41" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="52" t="s">
+      <c r="B41" s="55" t="s">
         <v>22</v>
       </c>
       <c r="C41" s="22" t="s">
@@ -6873,7 +6892,7 @@
       <c r="A50" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="54" t="s">
+      <c r="B50" s="56" t="s">
         <v>51</v>
       </c>
       <c r="C50" s="18" t="s">
@@ -6939,7 +6958,7 @@
       <c r="A53" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="52" t="s">
+      <c r="B53" s="55" t="s">
         <v>58</v>
       </c>
       <c r="C53" s="22" t="s">
@@ -7032,7 +7051,7 @@
       <c r="A57" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="54" t="s">
+      <c r="B57" s="56" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="18" t="s">
@@ -7233,7 +7252,7 @@
       <c r="A65" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B65" s="52" t="s">
+      <c r="B65" s="55" t="s">
         <v>90</v>
       </c>
       <c r="C65" s="22" t="s">
@@ -7353,7 +7372,7 @@
       <c r="A70" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B70" s="54" t="s">
+      <c r="B70" s="56" t="s">
         <v>104</v>
       </c>
       <c r="C70" s="18" t="s">
@@ -7500,7 +7519,7 @@
       <c r="A76" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B76" s="52" t="s">
+      <c r="B76" s="55" t="s">
         <v>120</v>
       </c>
       <c r="C76" s="22" t="s">
@@ -7553,7 +7572,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A78" s="55" t="s">
+      <c r="A78" s="52" t="s">
         <v>140</v>
       </c>
       <c r="B78" s="53"/>
@@ -7562,7 +7581,7 @@
       <c r="E78" s="53"/>
       <c r="F78" s="53"/>
       <c r="G78" s="53"/>
-      <c r="H78" s="56"/>
+      <c r="H78" s="54"/>
       <c r="I78" s="12" t="s">
         <v>27</v>
       </c>
@@ -7571,7 +7590,7 @@
       <c r="A79" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B79" s="54" t="s">
+      <c r="B79" s="56" t="s">
         <v>141</v>
       </c>
       <c r="C79" s="18" t="s">
@@ -7662,7 +7681,7 @@
       <c r="A83" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B83" s="52" t="s">
+      <c r="B83" s="55" t="s">
         <v>153</v>
       </c>
       <c r="C83" s="22" t="s">
@@ -7711,7 +7730,7 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A85" s="55" t="s">
+      <c r="A85" s="52" t="s">
         <v>159</v>
       </c>
       <c r="B85" s="53"/>
@@ -7720,7 +7739,7 @@
       <c r="E85" s="53"/>
       <c r="F85" s="53"/>
       <c r="G85" s="53"/>
-      <c r="H85" s="56"/>
+      <c r="H85" s="54"/>
       <c r="I85" s="12" t="s">
         <v>27</v>
       </c>
@@ -7729,7 +7748,7 @@
       <c r="A86" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B86" s="54" t="s">
+      <c r="B86" s="56" t="s">
         <v>141</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -7820,7 +7839,7 @@
       <c r="A90" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B90" s="52" t="s">
+      <c r="B90" s="55" t="s">
         <v>153</v>
       </c>
       <c r="C90" s="22" t="s">
@@ -7880,6 +7899,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B86:B88"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A85:H85"/>
     <mergeCell ref="B32:B36"/>
@@ -7896,12 +7921,6 @@
     <mergeCell ref="B53:B55"/>
     <mergeCell ref="B19:B25"/>
     <mergeCell ref="B57:B63"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B86:B88"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="153" priority="564" operator="equal">
@@ -8131,7 +8150,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="52" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="53"/>
@@ -8140,13 +8159,13 @@
       <c r="E2" s="53"/>
       <c r="F2" s="53"/>
       <c r="G2" s="53"/>
-      <c r="H2" s="56"/>
+      <c r="H2" s="54"/>
     </row>
     <row r="3" spans="1:9" ht="76.5" customHeight="1">
       <c r="A3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="56" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -8287,7 +8306,7 @@
       <c r="A9" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="55" t="s">
         <v>182</v>
       </c>
       <c r="C9" s="22" t="s">
@@ -8405,7 +8424,7 @@
       <c r="A14" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="56" t="s">
         <v>192</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -8552,7 +8571,7 @@
       <c r="A20" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="54" t="s">
         <v>612</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -8696,7 +8715,7 @@
       <c r="A26" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B26" s="56" t="s">
+      <c r="B26" s="54" t="s">
         <v>208</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -8785,7 +8804,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A31" s="55" t="s">
+      <c r="A31" s="52" t="s">
         <v>213</v>
       </c>
       <c r="B31" s="53"/>
@@ -8794,13 +8813,13 @@
       <c r="E31" s="53"/>
       <c r="F31" s="53"/>
       <c r="G31" s="53"/>
-      <c r="H31" s="56"/>
+      <c r="H31" s="54"/>
     </row>
     <row r="32" spans="1:9" ht="76.5" customHeight="1">
       <c r="A32" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B32" s="54" t="s">
+      <c r="B32" s="56" t="s">
         <v>162</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -8941,7 +8960,7 @@
       <c r="A38" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B38" s="52" t="s">
+      <c r="B38" s="55" t="s">
         <v>182</v>
       </c>
       <c r="C38" s="22" t="s">
@@ -9059,7 +9078,7 @@
       <c r="A43" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B43" s="54" t="s">
+      <c r="B43" s="56" t="s">
         <v>192</v>
       </c>
       <c r="C43" s="18" t="s">
@@ -9206,7 +9225,7 @@
       <c r="A49" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B49" s="56" t="s">
+      <c r="B49" s="54" t="s">
         <v>612</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -9350,7 +9369,7 @@
       <c r="A55" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="56" t="s">
+      <c r="B55" s="54" t="s">
         <v>208</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -9439,7 +9458,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A60" s="55" t="s">
+      <c r="A60" s="52" t="s">
         <v>140</v>
       </c>
       <c r="B60" s="53"/>
@@ -9448,13 +9467,13 @@
       <c r="E60" s="53"/>
       <c r="F60" s="53"/>
       <c r="G60" s="53"/>
-      <c r="H60" s="56"/>
+      <c r="H60" s="54"/>
     </row>
     <row r="61" spans="1:9" ht="76.5" customHeight="1">
       <c r="A61" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B61" s="54" t="s">
+      <c r="B61" s="56" t="s">
         <v>162</v>
       </c>
       <c r="C61" s="18" t="s">
@@ -9595,7 +9614,7 @@
       <c r="A67" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B67" s="52" t="s">
+      <c r="B67" s="55" t="s">
         <v>182</v>
       </c>
       <c r="C67" s="22" t="s">
@@ -9713,7 +9732,7 @@
       <c r="A72" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B72" s="54" t="s">
+      <c r="B72" s="56" t="s">
         <v>192</v>
       </c>
       <c r="C72" s="18" t="s">
@@ -9860,7 +9879,7 @@
       <c r="A78" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B78" s="56" t="s">
+      <c r="B78" s="54" t="s">
         <v>611</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -10004,7 +10023,7 @@
       <c r="A84" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B84" s="56" t="s">
+      <c r="B84" s="54" t="s">
         <v>208</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -10093,7 +10112,7 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A89" s="55" t="s">
+      <c r="A89" s="52" t="s">
         <v>159</v>
       </c>
       <c r="B89" s="53"/>
@@ -10102,13 +10121,13 @@
       <c r="E89" s="53"/>
       <c r="F89" s="53"/>
       <c r="G89" s="53"/>
-      <c r="H89" s="56"/>
+      <c r="H89" s="54"/>
     </row>
     <row r="90" spans="1:9" ht="76.5" customHeight="1">
       <c r="A90" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="54" t="s">
+      <c r="B90" s="56" t="s">
         <v>162</v>
       </c>
       <c r="C90" s="18" t="s">
@@ -10249,7 +10268,7 @@
       <c r="A96" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B96" s="52" t="s">
+      <c r="B96" s="55" t="s">
         <v>182</v>
       </c>
       <c r="C96" s="22" t="s">
@@ -10367,7 +10386,7 @@
       <c r="A101" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B101" s="54" t="s">
+      <c r="B101" s="56" t="s">
         <v>192</v>
       </c>
       <c r="C101" s="18" t="s">
@@ -10514,7 +10533,7 @@
       <c r="A107" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B107" s="56" t="s">
+      <c r="B107" s="54" t="s">
         <v>591</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -10658,7 +10677,7 @@
       <c r="A113" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B113" s="56" t="s">
+      <c r="B113" s="54" t="s">
         <v>208</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -10748,14 +10767,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B101:B105"/>
-    <mergeCell ref="B107:B108"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="B96:B99"/>
     <mergeCell ref="A2:H2"/>
@@ -10772,6 +10783,14 @@
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="B55:B59"/>
     <mergeCell ref="B43:B47"/>
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B101:B105"/>
+    <mergeCell ref="B107:B108"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="111" priority="525" operator="equal">
@@ -11177,7 +11196,7 @@
       <c r="A2" s="57" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="56"/>
+      <c r="B2" s="54"/>
       <c r="C2" s="58"/>
       <c r="D2" s="53"/>
       <c r="E2" s="58"/>
@@ -11186,7 +11205,7 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="198" customHeight="1">
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="54" t="s">
         <v>216</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -11218,8 +11237,8 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="76.5" customHeight="1">
-      <c r="A4" s="56"/>
-      <c r="B4" s="56"/>
+      <c r="A4" s="54"/>
+      <c r="B4" s="54"/>
       <c r="C4" s="58" t="s">
         <v>221</v>
       </c>
@@ -11250,7 +11269,7 @@
     </row>
     <row r="5" spans="1:11" ht="45.75" customHeight="1">
       <c r="A5" s="58"/>
-      <c r="B5" s="56"/>
+      <c r="B5" s="54"/>
       <c r="C5" s="58"/>
       <c r="D5" s="53"/>
       <c r="E5" s="6" t="s">
@@ -11262,7 +11281,7 @@
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:11" ht="121.5" customHeight="1">
-      <c r="B6" s="56"/>
+      <c r="B6" s="54"/>
       <c r="C6" s="58" t="s">
         <v>226</v>
       </c>
@@ -11292,7 +11311,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="45.75" customHeight="1">
-      <c r="B7" s="56"/>
+      <c r="B7" s="54"/>
       <c r="C7" s="58"/>
       <c r="D7" s="53"/>
       <c r="E7" s="13" t="s">
@@ -11304,7 +11323,7 @@
       <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B8" s="56"/>
+      <c r="B8" s="54"/>
       <c r="C8" s="13" t="s">
         <v>229</v>
       </c>
@@ -11320,7 +11339,7 @@
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B9" s="56"/>
+      <c r="B9" s="54"/>
       <c r="C9" s="13" t="s">
         <v>231</v>
       </c>
@@ -11336,7 +11355,7 @@
       <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="91.5" customHeight="1">
-      <c r="B10" s="56"/>
+      <c r="B10" s="54"/>
       <c r="C10" s="13" t="s">
         <v>232</v>
       </c>
@@ -11366,7 +11385,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="140.25" customHeight="1">
-      <c r="B11" s="56"/>
+      <c r="B11" s="54"/>
       <c r="C11" s="13" t="s">
         <v>235</v>
       </c>
@@ -11409,7 +11428,7 @@
       <c r="A13" s="57" t="s">
         <v>238</v>
       </c>
-      <c r="B13" s="56"/>
+      <c r="B13" s="54"/>
       <c r="C13" s="58"/>
       <c r="D13" s="53"/>
       <c r="E13" s="58"/>
@@ -11547,7 +11566,7 @@
       <c r="A3" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="56" t="s">
         <v>239</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -11582,7 +11601,7 @@
       <c r="A4" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="56"/>
+      <c r="B4" s="54"/>
       <c r="C4" s="18" t="s">
         <v>244</v>
       </c>
@@ -11615,7 +11634,7 @@
       <c r="A5" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="56"/>
+      <c r="B5" s="54"/>
       <c r="C5" s="18" t="s">
         <v>247</v>
       </c>
@@ -11648,7 +11667,7 @@
       <c r="A6" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B6" s="56"/>
+      <c r="B6" s="54"/>
       <c r="C6" s="18" t="s">
         <v>251</v>
       </c>
@@ -11691,7 +11710,7 @@
       <c r="A8" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="55" t="s">
         <v>254</v>
       </c>
       <c r="C8" s="22" t="s">
@@ -11726,7 +11745,7 @@
       <c r="A9" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="56"/>
+      <c r="B9" s="54"/>
       <c r="C9" s="22" t="s">
         <v>259</v>
       </c>
@@ -11759,7 +11778,7 @@
       <c r="A10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="56"/>
+      <c r="B10" s="54"/>
       <c r="C10" s="59" t="s">
         <v>262</v>
       </c>
@@ -11772,7 +11791,7 @@
       <c r="F10" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G10" s="56" t="s">
+      <c r="G10" s="54" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="12" t="s">
@@ -11792,7 +11811,7 @@
       <c r="A11" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="56"/>
+      <c r="B11" s="54"/>
       <c r="C11" s="53"/>
       <c r="D11" s="58"/>
       <c r="E11" s="11" t="s">
@@ -11801,7 +11820,7 @@
       <c r="F11" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G11" s="56"/>
+      <c r="G11" s="54"/>
       <c r="H11" s="12" t="s">
         <v>27</v>
       </c>
@@ -11819,7 +11838,7 @@
       <c r="A12" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="B12" s="56"/>
+      <c r="B12" s="54"/>
       <c r="C12" s="22" t="s">
         <v>267</v>
       </c>
@@ -11852,7 +11871,7 @@
       <c r="A13" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="B13" s="56"/>
+      <c r="B13" s="54"/>
       <c r="C13" s="22" t="s">
         <v>271</v>
       </c>
@@ -11885,7 +11904,7 @@
       <c r="A14" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="56"/>
+      <c r="B14" s="54"/>
       <c r="C14" s="22" t="s">
         <v>274</v>
       </c>
@@ -11918,7 +11937,7 @@
       <c r="A15" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B15" s="56"/>
+      <c r="B15" s="54"/>
       <c r="C15" s="22" t="s">
         <v>279</v>
       </c>
@@ -11951,7 +11970,7 @@
       <c r="A16" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="56"/>
+      <c r="B16" s="54"/>
       <c r="C16" s="22" t="s">
         <v>282</v>
       </c>
@@ -11984,7 +12003,7 @@
       <c r="A17" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B17" s="56"/>
+      <c r="B17" s="54"/>
       <c r="C17" s="22" t="s">
         <v>286</v>
       </c>
@@ -12017,7 +12036,7 @@
       <c r="A18" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="B18" s="56"/>
+      <c r="B18" s="54"/>
       <c r="C18" s="22" t="s">
         <v>289</v>
       </c>
@@ -12050,7 +12069,7 @@
       <c r="A19" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B19" s="56"/>
+      <c r="B19" s="54"/>
       <c r="C19" s="22" t="s">
         <v>294</v>
       </c>
@@ -12083,7 +12102,7 @@
       <c r="A20" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B20" s="56"/>
+      <c r="B20" s="54"/>
       <c r="C20" s="22" t="s">
         <v>298</v>
       </c>
@@ -12116,7 +12135,7 @@
       <c r="A21" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="B21" s="56"/>
+      <c r="B21" s="54"/>
       <c r="C21" s="22" t="s">
         <v>303</v>
       </c>
@@ -12149,7 +12168,7 @@
       <c r="A22" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B22" s="56"/>
+      <c r="B22" s="54"/>
       <c r="C22" s="22" t="s">
         <v>305</v>
       </c>
@@ -12182,7 +12201,7 @@
       <c r="A23" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="B23" s="56"/>
+      <c r="B23" s="54"/>
       <c r="C23" s="22" t="s">
         <v>310</v>
       </c>
@@ -12215,7 +12234,7 @@
       <c r="A24" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="B24" s="56"/>
+      <c r="B24" s="54"/>
       <c r="C24" s="22" t="s">
         <v>314</v>
       </c>
@@ -12248,7 +12267,7 @@
       <c r="A25" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="B25" s="56"/>
+      <c r="B25" s="54"/>
       <c r="C25" s="22" t="s">
         <v>316</v>
       </c>
@@ -12278,7 +12297,7 @@
       <c r="A26" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="B26" s="56"/>
+      <c r="B26" s="54"/>
       <c r="C26" s="59" t="s">
         <v>321</v>
       </c>
@@ -12291,10 +12310,10 @@
       <c r="F26" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G26" s="56" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="56" t="s">
+      <c r="G26" s="54" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="54" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="12" t="s">
@@ -12308,7 +12327,7 @@
       <c r="A27" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B27" s="56"/>
+      <c r="B27" s="54"/>
       <c r="C27" s="53"/>
       <c r="D27" s="58"/>
       <c r="E27" s="11" t="s">
@@ -12317,14 +12336,14 @@
       <c r="F27" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="G27" s="56"/>
+      <c r="G27" s="54"/>
       <c r="H27" s="58"/>
     </row>
     <row r="28" spans="1:11" ht="76.5" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="B28" s="56"/>
+      <c r="B28" s="54"/>
       <c r="C28" s="22" t="s">
         <v>329</v>
       </c>
@@ -12357,7 +12376,7 @@
       <c r="A29" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="B29" s="56"/>
+      <c r="B29" s="54"/>
       <c r="C29" s="22" t="s">
         <v>334</v>
       </c>
@@ -12390,7 +12409,7 @@
       <c r="A30" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B30" s="56"/>
+      <c r="B30" s="54"/>
       <c r="C30" s="22" t="s">
         <v>338</v>
       </c>
@@ -12423,7 +12442,7 @@
       <c r="A31" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B31" s="56"/>
+      <c r="B31" s="54"/>
       <c r="C31" s="22" t="s">
         <v>341</v>
       </c>
@@ -12538,7 +12557,7 @@
       <c r="A36" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B36" s="54" t="s">
+      <c r="B36" s="56" t="s">
         <v>349</v>
       </c>
       <c r="C36" s="22" t="s">
@@ -12573,7 +12592,7 @@
       <c r="A37" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B37" s="56"/>
+      <c r="B37" s="54"/>
       <c r="C37" s="23" t="s">
         <v>354</v>
       </c>
@@ -12710,7 +12729,7 @@
       <c r="A3" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B3" s="54" t="s">
+      <c r="B3" s="56" t="s">
         <v>359</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -12899,7 +12918,7 @@
       <c r="A10" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="B10" s="52" t="s">
+      <c r="B10" s="55" t="s">
         <v>385</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -13187,7 +13206,7 @@
       <c r="A20" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="54" t="s">
+      <c r="B20" s="56" t="s">
         <v>422</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -13805,7 +13824,7 @@
       <c r="A40" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="B40" s="52" t="s">
+      <c r="B40" s="55" t="s">
         <v>505</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -13961,7 +13980,7 @@
       <c r="A46" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B46" s="54" t="s">
+      <c r="B46" s="56" t="s">
         <v>526</v>
       </c>
       <c r="C46" s="8" t="s">
@@ -14239,7 +14258,7 @@
       <c r="A56" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B56" s="41" t="s">
+      <c r="B56" s="38" t="s">
         <v>560</v>
       </c>
       <c r="C56" s="8" t="s">
@@ -14471,7 +14490,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
@@ -14513,13 +14532,39 @@
       <c r="A2" s="57" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+    </row>
+    <row r="3" spans="1:8" ht="30">
+      <c r="A3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" t="s">
+        <v>614</v>
+      </c>
+      <c r="C3" t="s">
+        <v>615</v>
+      </c>
+      <c r="D3" t="s">
+        <v>616</v>
+      </c>
+      <c r="E3" s="62" t="s">
+        <v>617</v>
+      </c>
+      <c r="F3" t="s">
+        <v>618</v>
+      </c>
+      <c r="G3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -14581,13 +14626,13 @@
       <c r="A2" s="57" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
QA: automatizar Compra fallida - Problema tarjeta (Vetify B2C + OSDE Adquirente)
TC-02 nuevo en ambos purchase-flow.spec.ts, usando el codigo de tarjeta de prueba
OTHE de MercadoPago (rechazo real, a diferencia de CTNA que es una regla de negocio
de Vetify). Verificado en vivo: el rechazo real de MercadoPago responde HTTP 200 con
el detalle embebido en el body, no HTTP 400 como el caso de tarjeta prepaga.

De paso se encontro y corrigio un bug real preexistente en el TC-01 de ambos
productos: el patron de page.waitForResponse() tenia barras invertidas mal escapadas
que JS descartaba en silencio, dejando un patron que nunca podia matchear la URL
real. Los 4 tests (TC-01/TC-02 x 2 productos) quedan verificados pasando.

Excel actualizado (Flujo de Compra filas 13/51, Automatizado No->Si) y dashboard
verificado sin corrupcion.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Casos de Prueba.xlsx
+++ b/documentation/Casos de Prueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ike\vetify-automation\automation\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3F6A3A-1DD1-4625-AE09-7F04C559B93D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC7EDF8-291D-44D7-90E5-3B3220A8C45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2914,6 +2914,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2934,28 +2943,19 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4807,734 +4807,734 @@
   <sheetData>
     <row r="2" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="3" spans="3:24">
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="51"/>
-      <c r="K3" s="49" t="s">
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="54"/>
+      <c r="K3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="51"/>
-      <c r="S3" s="49" t="s">
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="54"/>
+      <c r="S3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
-      <c r="V3" s="50"/>
-      <c r="W3" s="50"/>
-      <c r="X3" s="51"/>
+      <c r="T3" s="53"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="54"/>
     </row>
     <row r="4" spans="3:24">
-      <c r="C4" s="45"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="44"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="43"/>
-      <c r="O4" s="43"/>
-      <c r="P4" s="44"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="43"/>
-      <c r="U4" s="43"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="43"/>
-      <c r="X4" s="44"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="47"/>
+      <c r="S4" s="48"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="46"/>
+      <c r="V4" s="46"/>
+      <c r="W4" s="46"/>
+      <c r="X4" s="47"/>
     </row>
     <row r="5" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C5" s="42">
+      <c r="C5" s="45">
         <f>COUNTA('Flujo de Compra'!C3:C496,'Gestión de Usuario'!C3:C357,Perfil!C3:C199,Credenciales!C3:C199,Videollamadas!C3:C199,Reintegros!C2:C199,Misceláneas!C2:C199,'Control de Acceso'!C2:C199,'Sistema Caído'!C2:C199)</f>
         <v>273</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-      <c r="K5" s="42">
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
+      <c r="K5" s="45">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")+COUNTIF(Reintegros!G:G,"Si")+COUNTIF(Misceláneas!H:H,"Si")+COUNTIF('Control de Acceso'!H:H,"Si")+COUNTIF('Sistema Caído'!H:H,"Si")</f>
-        <v>202</v>
-      </c>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="44"/>
-      <c r="S5" s="53">
+        <v>204</v>
+      </c>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="47"/>
+      <c r="S5" s="56">
         <f>K5/C5</f>
-        <v>0.73992673992673996</v>
-      </c>
-      <c r="T5" s="43"/>
-      <c r="U5" s="43"/>
-      <c r="V5" s="43"/>
-      <c r="W5" s="43"/>
-      <c r="X5" s="44"/>
+        <v>0.74725274725274726</v>
+      </c>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="47"/>
     </row>
     <row r="6" spans="3:24">
-      <c r="C6" s="45"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="43"/>
-      <c r="O6" s="43"/>
-      <c r="P6" s="44"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="43"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="43"/>
-      <c r="W6" s="43"/>
-      <c r="X6" s="44"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="47"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="46"/>
+      <c r="U6" s="46"/>
+      <c r="V6" s="46"/>
+      <c r="W6" s="46"/>
+      <c r="X6" s="47"/>
     </row>
     <row r="7" spans="3:24">
-      <c r="C7" s="45"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="44"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="44"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="43"/>
-      <c r="V7" s="43"/>
-      <c r="W7" s="43"/>
-      <c r="X7" s="44"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="47"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
+      <c r="O7" s="46"/>
+      <c r="P7" s="47"/>
+      <c r="S7" s="48"/>
+      <c r="T7" s="46"/>
+      <c r="U7" s="46"/>
+      <c r="V7" s="46"/>
+      <c r="W7" s="46"/>
+      <c r="X7" s="47"/>
     </row>
     <row r="8" spans="3:24">
-      <c r="C8" s="45"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="44"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="44"/>
-      <c r="S8" s="45"/>
-      <c r="T8" s="43"/>
-      <c r="U8" s="43"/>
-      <c r="V8" s="43"/>
-      <c r="W8" s="43"/>
-      <c r="X8" s="44"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="47"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="46"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="46"/>
+      <c r="O8" s="46"/>
+      <c r="P8" s="47"/>
+      <c r="S8" s="48"/>
+      <c r="T8" s="46"/>
+      <c r="U8" s="46"/>
+      <c r="V8" s="46"/>
+      <c r="W8" s="46"/>
+      <c r="X8" s="47"/>
     </row>
     <row r="9" spans="3:24">
-      <c r="C9" s="45"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="44"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="43"/>
-      <c r="U9" s="43"/>
-      <c r="V9" s="43"/>
-      <c r="W9" s="43"/>
-      <c r="X9" s="44"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46"/>
+      <c r="P9" s="47"/>
+      <c r="S9" s="48"/>
+      <c r="T9" s="46"/>
+      <c r="U9" s="46"/>
+      <c r="V9" s="46"/>
+      <c r="W9" s="46"/>
+      <c r="X9" s="47"/>
     </row>
     <row r="10" spans="3:24">
-      <c r="C10" s="45"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="44"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="43"/>
-      <c r="U10" s="43"/>
-      <c r="V10" s="43"/>
-      <c r="W10" s="43"/>
-      <c r="X10" s="44"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46"/>
+      <c r="P10" s="47"/>
+      <c r="S10" s="48"/>
+      <c r="T10" s="46"/>
+      <c r="U10" s="46"/>
+      <c r="V10" s="46"/>
+      <c r="W10" s="46"/>
+      <c r="X10" s="47"/>
     </row>
     <row r="11" spans="3:24">
-      <c r="C11" s="45"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="44"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="43"/>
-      <c r="U11" s="43"/>
-      <c r="V11" s="43"/>
-      <c r="W11" s="43"/>
-      <c r="X11" s="44"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="47"/>
+      <c r="S11" s="48"/>
+      <c r="T11" s="46"/>
+      <c r="U11" s="46"/>
+      <c r="V11" s="46"/>
+      <c r="W11" s="46"/>
+      <c r="X11" s="47"/>
     </row>
     <row r="12" spans="3:24">
-      <c r="C12" s="45"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="44"/>
-      <c r="S12" s="45"/>
-      <c r="T12" s="43"/>
-      <c r="U12" s="43"/>
-      <c r="V12" s="43"/>
-      <c r="W12" s="43"/>
-      <c r="X12" s="44"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="47"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="46"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
+      <c r="O12" s="46"/>
+      <c r="P12" s="47"/>
+      <c r="S12" s="48"/>
+      <c r="T12" s="46"/>
+      <c r="U12" s="46"/>
+      <c r="V12" s="46"/>
+      <c r="W12" s="46"/>
+      <c r="X12" s="47"/>
     </row>
     <row r="13" spans="3:24">
-      <c r="C13" s="45"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="44"/>
-      <c r="S13" s="45"/>
-      <c r="T13" s="43"/>
-      <c r="U13" s="43"/>
-      <c r="V13" s="43"/>
-      <c r="W13" s="43"/>
-      <c r="X13" s="44"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="47"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="47"/>
+      <c r="S13" s="48"/>
+      <c r="T13" s="46"/>
+      <c r="U13" s="46"/>
+      <c r="V13" s="46"/>
+      <c r="W13" s="46"/>
+      <c r="X13" s="47"/>
     </row>
     <row r="14" spans="3:24">
-      <c r="C14" s="45"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="44"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="43"/>
-      <c r="U14" s="43"/>
-      <c r="V14" s="43"/>
-      <c r="W14" s="43"/>
-      <c r="X14" s="44"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="47"/>
+      <c r="S14" s="48"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="47"/>
     </row>
     <row r="15" spans="3:24">
-      <c r="C15" s="45"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="43"/>
-      <c r="N15" s="43"/>
-      <c r="O15" s="43"/>
-      <c r="P15" s="44"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="43"/>
-      <c r="U15" s="43"/>
-      <c r="V15" s="43"/>
-      <c r="W15" s="43"/>
-      <c r="X15" s="44"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="47"/>
+      <c r="S15" s="48"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="47"/>
     </row>
     <row r="16" spans="3:24">
-      <c r="C16" s="45"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="44"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="43"/>
-      <c r="M16" s="43"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="44"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="43"/>
-      <c r="U16" s="43"/>
-      <c r="V16" s="43"/>
-      <c r="W16" s="43"/>
-      <c r="X16" s="44"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
+      <c r="P16" s="47"/>
+      <c r="S16" s="48"/>
+      <c r="T16" s="46"/>
+      <c r="U16" s="46"/>
+      <c r="V16" s="46"/>
+      <c r="W16" s="46"/>
+      <c r="X16" s="47"/>
     </row>
     <row r="17" spans="3:24">
-      <c r="C17" s="45"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="43"/>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="44"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="43"/>
-      <c r="U17" s="43"/>
-      <c r="V17" s="43"/>
-      <c r="W17" s="43"/>
-      <c r="X17" s="44"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="46"/>
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+      <c r="O17" s="46"/>
+      <c r="P17" s="47"/>
+      <c r="S17" s="48"/>
+      <c r="T17" s="46"/>
+      <c r="U17" s="46"/>
+      <c r="V17" s="46"/>
+      <c r="W17" s="46"/>
+      <c r="X17" s="47"/>
     </row>
     <row r="18" spans="3:24">
-      <c r="C18" s="45"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="43"/>
-      <c r="N18" s="43"/>
-      <c r="O18" s="43"/>
-      <c r="P18" s="44"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="43"/>
-      <c r="U18" s="43"/>
-      <c r="V18" s="43"/>
-      <c r="W18" s="43"/>
-      <c r="X18" s="44"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="47"/>
+      <c r="S18" s="48"/>
+      <c r="T18" s="46"/>
+      <c r="U18" s="46"/>
+      <c r="V18" s="46"/>
+      <c r="W18" s="46"/>
+      <c r="X18" s="47"/>
     </row>
     <row r="19" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C19" s="46"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
-      <c r="K19" s="46"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="48"/>
-      <c r="S19" s="46"/>
-      <c r="T19" s="47"/>
-      <c r="U19" s="47"/>
-      <c r="V19" s="47"/>
-      <c r="W19" s="47"/>
-      <c r="X19" s="48"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="51"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="51"/>
+      <c r="S19" s="49"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="50"/>
+      <c r="V19" s="50"/>
+      <c r="W19" s="50"/>
+      <c r="X19" s="51"/>
     </row>
     <row r="22" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="23" spans="3:24">
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="51"/>
-      <c r="K23" s="49" t="s">
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="54"/>
+      <c r="K23" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="L23" s="50"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
-      <c r="O23" s="50"/>
-      <c r="P23" s="51"/>
-      <c r="S23" s="49" t="s">
+      <c r="L23" s="53"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="53"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="54"/>
+      <c r="S23" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T23" s="50"/>
-      <c r="U23" s="50"/>
-      <c r="V23" s="50"/>
-      <c r="W23" s="50"/>
-      <c r="X23" s="51"/>
+      <c r="T23" s="53"/>
+      <c r="U23" s="53"/>
+      <c r="V23" s="53"/>
+      <c r="W23" s="53"/>
+      <c r="X23" s="54"/>
     </row>
     <row r="24" spans="3:24">
-      <c r="C24" s="45"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="44"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="43"/>
-      <c r="U24" s="43"/>
-      <c r="V24" s="43"/>
-      <c r="W24" s="43"/>
-      <c r="X24" s="44"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="47"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="47"/>
+      <c r="S24" s="48"/>
+      <c r="T24" s="46"/>
+      <c r="U24" s="46"/>
+      <c r="V24" s="46"/>
+      <c r="W24" s="46"/>
+      <c r="X24" s="47"/>
     </row>
     <row r="25" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C25" s="42">
+      <c r="C25" s="45">
         <f>COUNTIF('Flujo de Compra'!G:G,"Si")+COUNTIF('Gestión de Usuario'!G:G,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!G:G,"Si")+COUNTIF(Videollamadas!G:G,"Si")+COUNTIF(Reintegros!G:G,"Si")+COUNTIF(Misceláneas!G:G,"Si")+COUNTIF('Control de Acceso'!G:G,"Si")+COUNTIF('Sistema Caído'!G:G,"Si")</f>
         <v>146</v>
       </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
-      <c r="K25" s="42">
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
+      <c r="K25" s="45">
         <f>COUNTIFS('Flujo de Compra'!G:G,"Si",'Flujo de Compra'!H:H,"Si")+COUNTIFS('Gestión de Usuario'!G:G,"Si",'Gestión de Usuario'!H:H,"Si")+COUNTIFS(Perfil!G:G,"Si",Perfil!H:H,"Si")+COUNTIFS(Credenciales!G:G,"Si",Credenciales!H:H,"Si")+COUNTIFS(Videollamadas!G:G,"Si",Videollamadas!H:H,"Si")+COUNTIFS(Reintegros!G:G,"Si",Reintegros!H:H,"Si")+COUNTIFS(Misceláneas!G:G,"Si",Misceláneas!H:H,"Si")+COUNTIFS('Control de Acceso'!G:G,"Si",'Control de Acceso'!H:H,"Si")+COUNTIFS('Sistema Caído'!G:G,"Si",'Sistema Caído'!H:H,"Si")</f>
-        <v>114</v>
-      </c>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
-      <c r="N25" s="43"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="44"/>
-      <c r="S25" s="53">
+        <v>116</v>
+      </c>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="47"/>
+      <c r="S25" s="56">
         <f>K25/C25</f>
-        <v>0.78082191780821919</v>
-      </c>
-      <c r="T25" s="43"/>
-      <c r="U25" s="43"/>
-      <c r="V25" s="43"/>
-      <c r="W25" s="43"/>
-      <c r="X25" s="44"/>
+        <v>0.79452054794520544</v>
+      </c>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+      <c r="V25" s="46"/>
+      <c r="W25" s="46"/>
+      <c r="X25" s="47"/>
     </row>
     <row r="26" spans="3:24">
-      <c r="C26" s="45"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="44"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
-      <c r="N26" s="43"/>
-      <c r="O26" s="43"/>
-      <c r="P26" s="44"/>
-      <c r="S26" s="45"/>
-      <c r="T26" s="43"/>
-      <c r="U26" s="43"/>
-      <c r="V26" s="43"/>
-      <c r="W26" s="43"/>
-      <c r="X26" s="44"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="47"/>
+      <c r="S26" s="48"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+      <c r="V26" s="46"/>
+      <c r="W26" s="46"/>
+      <c r="X26" s="47"/>
     </row>
     <row r="27" spans="3:24">
-      <c r="C27" s="45"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="44"/>
-      <c r="S27" s="45"/>
-      <c r="T27" s="43"/>
-      <c r="U27" s="43"/>
-      <c r="V27" s="43"/>
-      <c r="W27" s="43"/>
-      <c r="X27" s="44"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="47"/>
+      <c r="S27" s="48"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+      <c r="V27" s="46"/>
+      <c r="W27" s="46"/>
+      <c r="X27" s="47"/>
     </row>
     <row r="28" spans="3:24">
-      <c r="C28" s="45"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="44"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="43"/>
-      <c r="P28" s="44"/>
-      <c r="S28" s="45"/>
-      <c r="T28" s="43"/>
-      <c r="U28" s="43"/>
-      <c r="V28" s="43"/>
-      <c r="W28" s="43"/>
-      <c r="X28" s="44"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="47"/>
+      <c r="K28" s="48"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
+      <c r="S28" s="48"/>
+      <c r="T28" s="46"/>
+      <c r="U28" s="46"/>
+      <c r="V28" s="46"/>
+      <c r="W28" s="46"/>
+      <c r="X28" s="47"/>
     </row>
     <row r="29" spans="3:24">
-      <c r="C29" s="45"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="43"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="44"/>
-      <c r="S29" s="45"/>
-      <c r="T29" s="43"/>
-      <c r="U29" s="43"/>
-      <c r="V29" s="43"/>
-      <c r="W29" s="43"/>
-      <c r="X29" s="44"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="47"/>
+      <c r="K29" s="48"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="47"/>
+      <c r="S29" s="48"/>
+      <c r="T29" s="46"/>
+      <c r="U29" s="46"/>
+      <c r="V29" s="46"/>
+      <c r="W29" s="46"/>
+      <c r="X29" s="47"/>
     </row>
     <row r="30" spans="3:24">
-      <c r="C30" s="45"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
-      <c r="K30" s="45"/>
-      <c r="L30" s="43"/>
-      <c r="M30" s="43"/>
-      <c r="N30" s="43"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="44"/>
-      <c r="S30" s="45"/>
-      <c r="T30" s="43"/>
-      <c r="U30" s="43"/>
-      <c r="V30" s="43"/>
-      <c r="W30" s="43"/>
-      <c r="X30" s="44"/>
+      <c r="C30" s="48"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="47"/>
+      <c r="K30" s="48"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="47"/>
+      <c r="S30" s="48"/>
+      <c r="T30" s="46"/>
+      <c r="U30" s="46"/>
+      <c r="V30" s="46"/>
+      <c r="W30" s="46"/>
+      <c r="X30" s="47"/>
     </row>
     <row r="31" spans="3:24">
-      <c r="C31" s="45"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="44"/>
-      <c r="K31" s="45"/>
-      <c r="L31" s="43"/>
-      <c r="M31" s="43"/>
-      <c r="N31" s="43"/>
-      <c r="O31" s="43"/>
-      <c r="P31" s="44"/>
-      <c r="S31" s="45"/>
-      <c r="T31" s="43"/>
-      <c r="U31" s="43"/>
-      <c r="V31" s="43"/>
-      <c r="W31" s="43"/>
-      <c r="X31" s="44"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="47"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="47"/>
+      <c r="S31" s="48"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+      <c r="V31" s="46"/>
+      <c r="W31" s="46"/>
+      <c r="X31" s="47"/>
     </row>
     <row r="32" spans="3:24">
-      <c r="C32" s="45"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="44"/>
-      <c r="K32" s="45"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="43"/>
-      <c r="N32" s="43"/>
-      <c r="O32" s="43"/>
-      <c r="P32" s="44"/>
-      <c r="S32" s="45"/>
-      <c r="T32" s="43"/>
-      <c r="U32" s="43"/>
-      <c r="V32" s="43"/>
-      <c r="W32" s="43"/>
-      <c r="X32" s="44"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="47"/>
+      <c r="K32" s="48"/>
+      <c r="L32" s="46"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
+      <c r="P32" s="47"/>
+      <c r="S32" s="48"/>
+      <c r="T32" s="46"/>
+      <c r="U32" s="46"/>
+      <c r="V32" s="46"/>
+      <c r="W32" s="46"/>
+      <c r="X32" s="47"/>
     </row>
     <row r="33" spans="3:24">
-      <c r="C33" s="45"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="44"/>
-      <c r="K33" s="45"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="43"/>
-      <c r="P33" s="44"/>
-      <c r="S33" s="45"/>
-      <c r="T33" s="43"/>
-      <c r="U33" s="43"/>
-      <c r="V33" s="43"/>
-      <c r="W33" s="43"/>
-      <c r="X33" s="44"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="47"/>
+      <c r="K33" s="48"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="47"/>
+      <c r="S33" s="48"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+      <c r="V33" s="46"/>
+      <c r="W33" s="46"/>
+      <c r="X33" s="47"/>
     </row>
     <row r="34" spans="3:24">
-      <c r="C34" s="45"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="44"/>
-      <c r="K34" s="45"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="44"/>
-      <c r="S34" s="45"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="44"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="47"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="46"/>
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="47"/>
+      <c r="S34" s="48"/>
+      <c r="T34" s="46"/>
+      <c r="U34" s="46"/>
+      <c r="V34" s="46"/>
+      <c r="W34" s="46"/>
+      <c r="X34" s="47"/>
     </row>
     <row r="35" spans="3:24">
-      <c r="C35" s="45"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="44"/>
-      <c r="K35" s="45"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="44"/>
-      <c r="S35" s="45"/>
-      <c r="T35" s="43"/>
-      <c r="U35" s="43"/>
-      <c r="V35" s="43"/>
-      <c r="W35" s="43"/>
-      <c r="X35" s="44"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="47"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="47"/>
+      <c r="S35" s="48"/>
+      <c r="T35" s="46"/>
+      <c r="U35" s="46"/>
+      <c r="V35" s="46"/>
+      <c r="W35" s="46"/>
+      <c r="X35" s="47"/>
     </row>
     <row r="36" spans="3:24">
-      <c r="C36" s="45"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="44"/>
-      <c r="K36" s="45"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="44"/>
-      <c r="S36" s="45"/>
-      <c r="T36" s="43"/>
-      <c r="U36" s="43"/>
-      <c r="V36" s="43"/>
-      <c r="W36" s="43"/>
-      <c r="X36" s="44"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="47"/>
+      <c r="K36" s="48"/>
+      <c r="L36" s="46"/>
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="47"/>
+      <c r="S36" s="48"/>
+      <c r="T36" s="46"/>
+      <c r="U36" s="46"/>
+      <c r="V36" s="46"/>
+      <c r="W36" s="46"/>
+      <c r="X36" s="47"/>
     </row>
     <row r="37" spans="3:24">
-      <c r="C37" s="45"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
-      <c r="K37" s="45"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="44"/>
-      <c r="S37" s="45"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="44"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="46"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="47"/>
+      <c r="K37" s="48"/>
+      <c r="L37" s="46"/>
+      <c r="M37" s="46"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="46"/>
+      <c r="P37" s="47"/>
+      <c r="S37" s="48"/>
+      <c r="T37" s="46"/>
+      <c r="U37" s="46"/>
+      <c r="V37" s="46"/>
+      <c r="W37" s="46"/>
+      <c r="X37" s="47"/>
     </row>
     <row r="38" spans="3:24">
-      <c r="C38" s="45"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="44"/>
-      <c r="K38" s="45"/>
-      <c r="L38" s="43"/>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="44"/>
-      <c r="S38" s="45"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="44"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="47"/>
+      <c r="K38" s="48"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="47"/>
+      <c r="S38" s="48"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="47"/>
     </row>
     <row r="39" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C39" s="46"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="48"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="47"/>
-      <c r="O39" s="47"/>
-      <c r="P39" s="48"/>
-      <c r="S39" s="46"/>
-      <c r="T39" s="47"/>
-      <c r="U39" s="47"/>
-      <c r="V39" s="47"/>
-      <c r="W39" s="47"/>
-      <c r="X39" s="48"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="50"/>
+      <c r="H39" s="51"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="51"/>
+      <c r="S39" s="49"/>
+      <c r="T39" s="50"/>
+      <c r="U39" s="50"/>
+      <c r="V39" s="50"/>
+      <c r="W39" s="50"/>
+      <c r="X39" s="51"/>
     </row>
     <row r="41" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="42" spans="3:24">
-      <c r="C42" s="49" t="s">
+      <c r="C42" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="50"/>
-      <c r="H42" s="51"/>
+      <c r="D42" s="53"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="53"/>
+      <c r="G42" s="53"/>
+      <c r="H42" s="54"/>
     </row>
     <row r="43" spans="3:24">
-      <c r="C43" s="45"/>
-      <c r="D43" s="43"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="43"/>
-      <c r="G43" s="43"/>
-      <c r="H43" s="44"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="47"/>
       <c r="K43" s="28"/>
       <c r="L43" s="28"/>
       <c r="M43" s="28"/>
@@ -5543,31 +5543,31 @@
       <c r="P43" s="28"/>
     </row>
     <row r="44" spans="3:24" ht="21" customHeight="1">
-      <c r="C44" s="53">
+      <c r="C44" s="56">
         <f>C25/C5</f>
         <v>0.53479853479853479</v>
       </c>
-      <c r="D44" s="43"/>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="44"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="47"/>
       <c r="K44" s="28"/>
-      <c r="L44" s="52" t="s">
+      <c r="L44" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="M44" s="43"/>
-      <c r="N44" s="43"/>
-      <c r="O44" s="43"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
+      <c r="O44" s="46"/>
       <c r="P44" s="29"/>
     </row>
     <row r="45" spans="3:24">
-      <c r="C45" s="45"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="44"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="47"/>
       <c r="K45" s="28"/>
       <c r="L45" s="30"/>
       <c r="M45" s="30"/>
@@ -5576,12 +5576,12 @@
       <c r="P45" s="29"/>
     </row>
     <row r="46" spans="3:24">
-      <c r="C46" s="45"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="44"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="46"/>
+      <c r="E46" s="46"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="46"/>
+      <c r="H46" s="47"/>
       <c r="K46" s="28"/>
       <c r="L46" s="31"/>
       <c r="M46" s="28" t="s">
@@ -5592,12 +5592,12 @@
       <c r="P46" s="28"/>
     </row>
     <row r="47" spans="3:24">
-      <c r="C47" s="45"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="43"/>
-      <c r="H47" s="44"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="46"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="46"/>
+      <c r="H47" s="47"/>
       <c r="K47" s="28"/>
       <c r="L47" s="32"/>
       <c r="M47" s="28" t="s">
@@ -5608,12 +5608,12 @@
       <c r="P47" s="28"/>
     </row>
     <row r="48" spans="3:24">
-      <c r="C48" s="45"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="48"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
       <c r="K48" s="28"/>
       <c r="L48" s="33"/>
       <c r="M48" s="28" t="s">
@@ -5624,12 +5624,12 @@
       <c r="P48" s="28"/>
     </row>
     <row r="49" spans="3:16">
-      <c r="C49" s="45"/>
-      <c r="D49" s="43"/>
-      <c r="E49" s="43"/>
-      <c r="F49" s="43"/>
-      <c r="G49" s="43"/>
-      <c r="H49" s="44"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="46"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="47"/>
       <c r="K49" s="28"/>
       <c r="L49" s="34"/>
       <c r="M49" s="28" t="s">
@@ -5640,12 +5640,12 @@
       <c r="P49" s="28"/>
     </row>
     <row r="50" spans="3:16">
-      <c r="C50" s="45"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="C50" s="48"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="47"/>
       <c r="K50" s="28"/>
       <c r="L50" s="35"/>
       <c r="M50" s="28" t="s">
@@ -5656,12 +5656,12 @@
       <c r="P50" s="28"/>
     </row>
     <row r="51" spans="3:16">
-      <c r="C51" s="45"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="47"/>
       <c r="K51" s="28"/>
       <c r="L51" s="28"/>
       <c r="M51" s="28"/>
@@ -5670,230 +5670,230 @@
       <c r="P51" s="28"/>
     </row>
     <row r="52" spans="3:16">
-      <c r="C52" s="45"/>
-      <c r="D52" s="43"/>
-      <c r="E52" s="43"/>
-      <c r="F52" s="43"/>
-      <c r="G52" s="43"/>
-      <c r="H52" s="44"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="47"/>
     </row>
     <row r="53" spans="3:16">
-      <c r="C53" s="45"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="44"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="47"/>
     </row>
     <row r="54" spans="3:16">
-      <c r="C54" s="45"/>
-      <c r="D54" s="43"/>
-      <c r="E54" s="43"/>
-      <c r="F54" s="43"/>
-      <c r="G54" s="43"/>
-      <c r="H54" s="44"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="47"/>
     </row>
     <row r="55" spans="3:16">
-      <c r="C55" s="45"/>
-      <c r="D55" s="43"/>
-      <c r="E55" s="43"/>
-      <c r="F55" s="43"/>
-      <c r="G55" s="43"/>
-      <c r="H55" s="44"/>
+      <c r="C55" s="48"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="47"/>
     </row>
     <row r="56" spans="3:16">
-      <c r="C56" s="45"/>
-      <c r="D56" s="43"/>
-      <c r="E56" s="43"/>
-      <c r="F56" s="43"/>
-      <c r="G56" s="43"/>
-      <c r="H56" s="44"/>
+      <c r="C56" s="48"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46"/>
+      <c r="F56" s="46"/>
+      <c r="G56" s="46"/>
+      <c r="H56" s="47"/>
     </row>
     <row r="57" spans="3:16">
-      <c r="C57" s="45"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="48"/>
+      <c r="D57" s="46"/>
+      <c r="E57" s="46"/>
+      <c r="F57" s="46"/>
+      <c r="G57" s="46"/>
+      <c r="H57" s="47"/>
     </row>
     <row r="58" spans="3:16" ht="15.75" customHeight="1">
-      <c r="C58" s="46"/>
-      <c r="D58" s="47"/>
-      <c r="E58" s="47"/>
-      <c r="F58" s="47"/>
-      <c r="G58" s="47"/>
-      <c r="H58" s="48"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="50"/>
+      <c r="E58" s="50"/>
+      <c r="F58" s="50"/>
+      <c r="G58" s="50"/>
+      <c r="H58" s="51"/>
     </row>
     <row r="62" spans="3:16">
-      <c r="C62" s="54" t="s">
+      <c r="C62" s="42" t="s">
         <v>585</v>
       </c>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="H62" s="54" t="s">
+      <c r="D62" s="42"/>
+      <c r="E62" s="42"/>
+      <c r="F62" s="42"/>
+      <c r="H62" s="42" t="s">
         <v>586</v>
       </c>
-      <c r="I62" s="54"/>
-      <c r="J62" s="54"/>
-      <c r="K62" s="54"/>
-      <c r="M62" s="54" t="s">
+      <c r="I62" s="42"/>
+      <c r="J62" s="42"/>
+      <c r="K62" s="42"/>
+      <c r="M62" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N62" s="54"/>
-      <c r="O62" s="54"/>
-      <c r="P62" s="54"/>
+      <c r="N62" s="42"/>
+      <c r="O62" s="42"/>
+      <c r="P62" s="42"/>
     </row>
     <row r="63" spans="3:16">
-      <c r="C63" s="54"/>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54"/>
-      <c r="F63" s="54"/>
-      <c r="H63" s="54"/>
-      <c r="I63" s="54"/>
-      <c r="J63" s="54"/>
-      <c r="K63" s="54"/>
-      <c r="M63" s="54"/>
-      <c r="N63" s="54"/>
-      <c r="O63" s="54"/>
-      <c r="P63" s="54"/>
+      <c r="C63" s="42"/>
+      <c r="D63" s="42"/>
+      <c r="E63" s="42"/>
+      <c r="F63" s="42"/>
+      <c r="H63" s="42"/>
+      <c r="I63" s="42"/>
+      <c r="J63" s="42"/>
+      <c r="K63" s="42"/>
+      <c r="M63" s="42"/>
+      <c r="N63" s="42"/>
+      <c r="O63" s="42"/>
+      <c r="P63" s="42"/>
     </row>
     <row r="64" spans="3:16">
-      <c r="C64" s="55">
+      <c r="C64" s="43">
         <f>COUNTIF('Flujo de Compra'!I:I,"Si")+COUNTIF('Gestión de Usuario'!I:I,"Si")+COUNTIF(Perfil!J:J,"Si")+COUNTIF(Credenciales!J:J,"Si")+COUNTIF(Videollamadas!J:J,"Si")</f>
         <v>250</v>
       </c>
-      <c r="D64" s="55"/>
-      <c r="E64" s="55"/>
-      <c r="F64" s="55"/>
-      <c r="H64" s="55">
+      <c r="D64" s="43"/>
+      <c r="E64" s="43"/>
+      <c r="F64" s="43"/>
+      <c r="H64" s="43">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")</f>
-        <v>188</v>
-      </c>
-      <c r="I64" s="55"/>
-      <c r="J64" s="55"/>
-      <c r="K64" s="55"/>
-      <c r="M64" s="56">
+        <v>190</v>
+      </c>
+      <c r="I64" s="43"/>
+      <c r="J64" s="43"/>
+      <c r="K64" s="43"/>
+      <c r="M64" s="44">
         <f t="shared" ref="M64" si="0">H64/C64</f>
-        <v>0.752</v>
-      </c>
-      <c r="N64" s="56"/>
-      <c r="O64" s="56"/>
-      <c r="P64" s="56"/>
+        <v>0.76</v>
+      </c>
+      <c r="N64" s="44"/>
+      <c r="O64" s="44"/>
+      <c r="P64" s="44"/>
     </row>
     <row r="65" spans="3:16">
-      <c r="C65" s="55"/>
-      <c r="D65" s="55"/>
-      <c r="E65" s="55"/>
-      <c r="F65" s="55"/>
-      <c r="H65" s="55"/>
-      <c r="I65" s="55"/>
-      <c r="J65" s="55"/>
-      <c r="K65" s="55"/>
-      <c r="M65" s="56"/>
-      <c r="N65" s="56"/>
-      <c r="O65" s="56"/>
-      <c r="P65" s="56"/>
+      <c r="C65" s="43"/>
+      <c r="D65" s="43"/>
+      <c r="E65" s="43"/>
+      <c r="F65" s="43"/>
+      <c r="H65" s="43"/>
+      <c r="I65" s="43"/>
+      <c r="J65" s="43"/>
+      <c r="K65" s="43"/>
+      <c r="M65" s="44"/>
+      <c r="N65" s="44"/>
+      <c r="O65" s="44"/>
+      <c r="P65" s="44"/>
     </row>
     <row r="66" spans="3:16">
-      <c r="C66" s="55"/>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55"/>
-      <c r="H66" s="55"/>
-      <c r="I66" s="55"/>
-      <c r="J66" s="55"/>
-      <c r="K66" s="55"/>
-      <c r="M66" s="56"/>
-      <c r="N66" s="56"/>
-      <c r="O66" s="56"/>
-      <c r="P66" s="56"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="H66" s="43"/>
+      <c r="I66" s="43"/>
+      <c r="J66" s="43"/>
+      <c r="K66" s="43"/>
+      <c r="M66" s="44"/>
+      <c r="N66" s="44"/>
+      <c r="O66" s="44"/>
+      <c r="P66" s="44"/>
     </row>
     <row r="69" spans="3:16">
-      <c r="C69" s="54" t="s">
+      <c r="C69" s="42" t="s">
         <v>588</v>
       </c>
-      <c r="D69" s="54"/>
-      <c r="E69" s="54"/>
-      <c r="F69" s="54"/>
-      <c r="H69" s="54" t="s">
+      <c r="D69" s="42"/>
+      <c r="E69" s="42"/>
+      <c r="F69" s="42"/>
+      <c r="H69" s="42" t="s">
         <v>589</v>
       </c>
-      <c r="I69" s="54"/>
-      <c r="J69" s="54"/>
-      <c r="K69" s="54"/>
-      <c r="M69" s="54" t="s">
+      <c r="I69" s="42"/>
+      <c r="J69" s="42"/>
+      <c r="K69" s="42"/>
+      <c r="M69" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N69" s="54"/>
-      <c r="O69" s="54"/>
-      <c r="P69" s="54"/>
+      <c r="N69" s="42"/>
+      <c r="O69" s="42"/>
+      <c r="P69" s="42"/>
     </row>
     <row r="70" spans="3:16">
-      <c r="C70" s="54"/>
-      <c r="D70" s="54"/>
-      <c r="E70" s="54"/>
-      <c r="F70" s="54"/>
-      <c r="H70" s="54"/>
-      <c r="I70" s="54"/>
-      <c r="J70" s="54"/>
-      <c r="K70" s="54"/>
-      <c r="M70" s="54"/>
-      <c r="N70" s="54"/>
-      <c r="O70" s="54"/>
-      <c r="P70" s="54"/>
+      <c r="C70" s="42"/>
+      <c r="D70" s="42"/>
+      <c r="E70" s="42"/>
+      <c r="F70" s="42"/>
+      <c r="H70" s="42"/>
+      <c r="I70" s="42"/>
+      <c r="J70" s="42"/>
+      <c r="K70" s="42"/>
+      <c r="M70" s="42"/>
+      <c r="N70" s="42"/>
+      <c r="O70" s="42"/>
+      <c r="P70" s="42"/>
     </row>
     <row r="71" spans="3:16">
-      <c r="C71" s="55">
+      <c r="C71" s="43">
         <f>COUNTIF(Perfil!K:K,"Si")+COUNTIF(Credenciales!K:K,"Si")+COUNTIF(Videollamadas!K:K,"Si")</f>
         <v>71</v>
       </c>
-      <c r="D71" s="55"/>
-      <c r="E71" s="55"/>
-      <c r="F71" s="55"/>
-      <c r="H71" s="55">
+      <c r="D71" s="43"/>
+      <c r="E71" s="43"/>
+      <c r="F71" s="43"/>
+      <c r="H71" s="43">
         <f>COUNTIF(Perfil!I:I,"Si")+COUNTIF(Credenciales!I:I,"Si")+COUNTIF(Videollamadas!I:I,"Si")</f>
         <v>60</v>
       </c>
-      <c r="I71" s="55"/>
-      <c r="J71" s="55"/>
-      <c r="K71" s="55"/>
-      <c r="M71" s="56">
+      <c r="I71" s="43"/>
+      <c r="J71" s="43"/>
+      <c r="K71" s="43"/>
+      <c r="M71" s="44">
         <f t="shared" ref="M71" si="1">H71/C71</f>
         <v>0.84507042253521125</v>
       </c>
-      <c r="N71" s="56"/>
-      <c r="O71" s="56"/>
-      <c r="P71" s="56"/>
+      <c r="N71" s="44"/>
+      <c r="O71" s="44"/>
+      <c r="P71" s="44"/>
     </row>
     <row r="72" spans="3:16">
-      <c r="C72" s="55"/>
-      <c r="D72" s="55"/>
-      <c r="E72" s="55"/>
-      <c r="F72" s="55"/>
-      <c r="H72" s="55"/>
-      <c r="I72" s="55"/>
-      <c r="J72" s="55"/>
-      <c r="K72" s="55"/>
-      <c r="M72" s="56"/>
-      <c r="N72" s="56"/>
-      <c r="O72" s="56"/>
-      <c r="P72" s="56"/>
+      <c r="C72" s="43"/>
+      <c r="D72" s="43"/>
+      <c r="E72" s="43"/>
+      <c r="F72" s="43"/>
+      <c r="H72" s="43"/>
+      <c r="I72" s="43"/>
+      <c r="J72" s="43"/>
+      <c r="K72" s="43"/>
+      <c r="M72" s="44"/>
+      <c r="N72" s="44"/>
+      <c r="O72" s="44"/>
+      <c r="P72" s="44"/>
     </row>
     <row r="73" spans="3:16">
-      <c r="C73" s="55"/>
-      <c r="D73" s="55"/>
-      <c r="E73" s="55"/>
-      <c r="F73" s="55"/>
-      <c r="H73" s="55"/>
-      <c r="I73" s="55"/>
-      <c r="J73" s="55"/>
-      <c r="K73" s="55"/>
-      <c r="M73" s="56"/>
-      <c r="N73" s="56"/>
-      <c r="O73" s="56"/>
-      <c r="P73" s="56"/>
+      <c r="C73" s="43"/>
+      <c r="D73" s="43"/>
+      <c r="E73" s="43"/>
+      <c r="F73" s="43"/>
+      <c r="H73" s="43"/>
+      <c r="I73" s="43"/>
+      <c r="J73" s="43"/>
+      <c r="K73" s="43"/>
+      <c r="M73" s="44"/>
+      <c r="N73" s="44"/>
+      <c r="O73" s="44"/>
+      <c r="P73" s="44"/>
     </row>
     <row r="76" spans="3:16">
       <c r="C76" s="36" t="s">
@@ -5902,18 +5902,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C69:F70"/>
-    <mergeCell ref="C71:F73"/>
-    <mergeCell ref="H69:K70"/>
-    <mergeCell ref="H71:K73"/>
-    <mergeCell ref="M69:P70"/>
-    <mergeCell ref="M71:P73"/>
-    <mergeCell ref="C62:F63"/>
-    <mergeCell ref="C64:F66"/>
-    <mergeCell ref="H62:K63"/>
-    <mergeCell ref="H64:K66"/>
-    <mergeCell ref="M62:P63"/>
-    <mergeCell ref="M64:P66"/>
     <mergeCell ref="K5:P19"/>
     <mergeCell ref="K25:P39"/>
     <mergeCell ref="S3:X4"/>
@@ -5929,6 +5917,18 @@
     <mergeCell ref="C3:H4"/>
     <mergeCell ref="C25:H39"/>
     <mergeCell ref="K23:P24"/>
+    <mergeCell ref="C62:F63"/>
+    <mergeCell ref="C64:F66"/>
+    <mergeCell ref="H62:K63"/>
+    <mergeCell ref="H64:K66"/>
+    <mergeCell ref="M62:P63"/>
+    <mergeCell ref="M64:P66"/>
+    <mergeCell ref="C69:F70"/>
+    <mergeCell ref="C71:F73"/>
+    <mergeCell ref="H69:K70"/>
+    <mergeCell ref="H71:K73"/>
+    <mergeCell ref="M69:P70"/>
+    <mergeCell ref="M71:P73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6143,7 +6143,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -6152,7 +6152,7 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
       <c r="I2" s="12" t="s">
         <v>27</v>
       </c>
@@ -6161,7 +6161,7 @@
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -6389,7 +6389,7 @@
       <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="60" t="s">
+      <c r="B12" s="57" t="s">
         <v>51</v>
       </c>
       <c r="C12" s="22" t="s">
@@ -6435,7 +6435,7 @@
         <v>27</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>27</v>
@@ -6455,7 +6455,7 @@
       <c r="A15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="59" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -6548,7 +6548,7 @@
       <c r="A19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="57" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="22" t="s">
@@ -6749,7 +6749,7 @@
       <c r="A27" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="61" t="s">
+      <c r="B27" s="59" t="s">
         <v>90</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -6869,7 +6869,7 @@
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="57" t="s">
         <v>104</v>
       </c>
       <c r="C32" s="22" t="s">
@@ -7016,7 +7016,7 @@
       <c r="A38" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="59" t="s">
         <v>120</v>
       </c>
       <c r="C38" s="18" t="s">
@@ -7069,7 +7069,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A40" s="57" t="s">
+      <c r="A40" s="60" t="s">
         <v>127</v>
       </c>
       <c r="B40" s="58"/>
@@ -7078,7 +7078,7 @@
       <c r="E40" s="58"/>
       <c r="F40" s="58"/>
       <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
+      <c r="H40" s="61"/>
       <c r="I40" s="12" t="s">
         <v>27</v>
       </c>
@@ -7087,7 +7087,7 @@
       <c r="A41" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="60" t="s">
+      <c r="B41" s="57" t="s">
         <v>22</v>
       </c>
       <c r="C41" s="22" t="s">
@@ -7315,7 +7315,7 @@
       <c r="A50" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="61" t="s">
+      <c r="B50" s="59" t="s">
         <v>51</v>
       </c>
       <c r="C50" s="18" t="s">
@@ -7361,7 +7361,7 @@
         <v>27</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I51" s="12" t="s">
         <v>27</v>
@@ -7381,7 +7381,7 @@
       <c r="A53" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="57" t="s">
         <v>58</v>
       </c>
       <c r="C53" s="22" t="s">
@@ -7474,7 +7474,7 @@
       <c r="A57" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="61" t="s">
+      <c r="B57" s="59" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="18" t="s">
@@ -7675,7 +7675,7 @@
       <c r="A65" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B65" s="60" t="s">
+      <c r="B65" s="57" t="s">
         <v>90</v>
       </c>
       <c r="C65" s="22" t="s">
@@ -7795,7 +7795,7 @@
       <c r="A70" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="59" t="s">
         <v>104</v>
       </c>
       <c r="C70" s="18" t="s">
@@ -7942,7 +7942,7 @@
       <c r="A76" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B76" s="60" t="s">
+      <c r="B76" s="57" t="s">
         <v>120</v>
       </c>
       <c r="C76" s="22" t="s">
@@ -7995,7 +7995,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A78" s="57" t="s">
+      <c r="A78" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B78" s="58"/>
@@ -8004,7 +8004,7 @@
       <c r="E78" s="58"/>
       <c r="F78" s="58"/>
       <c r="G78" s="58"/>
-      <c r="H78" s="59"/>
+      <c r="H78" s="61"/>
       <c r="I78" s="12" t="s">
         <v>27</v>
       </c>
@@ -8013,7 +8013,7 @@
       <c r="A79" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B79" s="61" t="s">
+      <c r="B79" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C79" s="18" t="s">
@@ -8104,7 +8104,7 @@
       <c r="A83" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B83" s="60" t="s">
+      <c r="B83" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C83" s="22" t="s">
@@ -8153,7 +8153,7 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A85" s="57" t="s">
+      <c r="A85" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B85" s="58"/>
@@ -8162,7 +8162,7 @@
       <c r="E85" s="58"/>
       <c r="F85" s="58"/>
       <c r="G85" s="58"/>
-      <c r="H85" s="59"/>
+      <c r="H85" s="61"/>
       <c r="I85" s="12" t="s">
         <v>27</v>
       </c>
@@ -8171,7 +8171,7 @@
       <c r="A86" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B86" s="61" t="s">
+      <c r="B86" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -8262,7 +8262,7 @@
       <c r="A90" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B90" s="60" t="s">
+      <c r="B90" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C90" s="22" t="s">
@@ -8322,12 +8322,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B86:B88"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A85:H85"/>
     <mergeCell ref="B32:B36"/>
@@ -8344,6 +8338,12 @@
     <mergeCell ref="B53:B55"/>
     <mergeCell ref="B19:B25"/>
     <mergeCell ref="B57:B63"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B86:B88"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="153" priority="564" operator="equal">
@@ -8573,7 +8573,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -8582,13 +8582,13 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
     </row>
     <row r="3" spans="1:9" ht="76.5" customHeight="1">
       <c r="A3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -8729,7 +8729,7 @@
       <c r="A9" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C9" s="22" t="s">
@@ -8847,7 +8847,7 @@
       <c r="A14" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -8994,7 +8994,7 @@
       <c r="A20" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -9138,7 +9138,7 @@
       <c r="A26" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -9227,7 +9227,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="60" t="s">
         <v>213</v>
       </c>
       <c r="B31" s="58"/>
@@ -9236,13 +9236,13 @@
       <c r="E31" s="58"/>
       <c r="F31" s="58"/>
       <c r="G31" s="58"/>
-      <c r="H31" s="59"/>
+      <c r="H31" s="61"/>
     </row>
     <row r="32" spans="1:9" ht="76.5" customHeight="1">
       <c r="A32" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -9383,7 +9383,7 @@
       <c r="A38" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C38" s="22" t="s">
@@ -9501,7 +9501,7 @@
       <c r="A43" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B43" s="61" t="s">
+      <c r="B43" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C43" s="18" t="s">
@@ -9648,7 +9648,7 @@
       <c r="A49" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B49" s="59" t="s">
+      <c r="B49" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -9792,7 +9792,7 @@
       <c r="A55" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -9881,7 +9881,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B60" s="58"/>
@@ -9890,13 +9890,13 @@
       <c r="E60" s="58"/>
       <c r="F60" s="58"/>
       <c r="G60" s="58"/>
-      <c r="H60" s="59"/>
+      <c r="H60" s="61"/>
     </row>
     <row r="61" spans="1:9" ht="76.5" customHeight="1">
       <c r="A61" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B61" s="61" t="s">
+      <c r="B61" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C61" s="18" t="s">
@@ -10037,7 +10037,7 @@
       <c r="A67" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B67" s="60" t="s">
+      <c r="B67" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C67" s="22" t="s">
@@ -10155,7 +10155,7 @@
       <c r="A72" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B72" s="61" t="s">
+      <c r="B72" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C72" s="18" t="s">
@@ -10302,7 +10302,7 @@
       <c r="A78" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B78" s="59" t="s">
+      <c r="B78" s="61" t="s">
         <v>611</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -10446,7 +10446,7 @@
       <c r="A84" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B84" s="59" t="s">
+      <c r="B84" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -10535,7 +10535,7 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A89" s="57" t="s">
+      <c r="A89" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B89" s="58"/>
@@ -10544,13 +10544,13 @@
       <c r="E89" s="58"/>
       <c r="F89" s="58"/>
       <c r="G89" s="58"/>
-      <c r="H89" s="59"/>
+      <c r="H89" s="61"/>
     </row>
     <row r="90" spans="1:9" ht="76.5" customHeight="1">
       <c r="A90" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="61" t="s">
+      <c r="B90" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C90" s="18" t="s">
@@ -10691,7 +10691,7 @@
       <c r="A96" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B96" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C96" s="22" t="s">
@@ -10809,7 +10809,7 @@
       <c r="A101" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B101" s="61" t="s">
+      <c r="B101" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C101" s="18" t="s">
@@ -10956,7 +10956,7 @@
       <c r="A107" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B107" s="59" t="s">
+      <c r="B107" s="61" t="s">
         <v>591</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -11100,7 +11100,7 @@
       <c r="A113" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B113" s="59" t="s">
+      <c r="B113" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -11190,6 +11190,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B101:B105"/>
+    <mergeCell ref="B107:B108"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="B96:B99"/>
     <mergeCell ref="A2:H2"/>
@@ -11206,14 +11214,6 @@
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="B55:B59"/>
     <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B101:B105"/>
-    <mergeCell ref="B107:B108"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="111" priority="525" operator="equal">
@@ -11619,7 +11619,7 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="59"/>
+      <c r="B2" s="61"/>
       <c r="C2" s="63"/>
       <c r="D2" s="58"/>
       <c r="E2" s="63"/>
@@ -11628,7 +11628,7 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="198" customHeight="1">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="61" t="s">
         <v>216</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -11660,8 +11660,8 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="76.5" customHeight="1">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="63" t="s">
         <v>221</v>
       </c>
@@ -11692,7 +11692,7 @@
     </row>
     <row r="5" spans="1:11" ht="45.75" customHeight="1">
       <c r="A5" s="63"/>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="63"/>
       <c r="D5" s="58"/>
       <c r="E5" s="6" t="s">
@@ -11704,7 +11704,7 @@
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:11" ht="121.5" customHeight="1">
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="63" t="s">
         <v>226</v>
       </c>
@@ -11734,7 +11734,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="45.75" customHeight="1">
-      <c r="B7" s="59"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="63"/>
       <c r="D7" s="58"/>
       <c r="E7" s="13" t="s">
@@ -11746,7 +11746,7 @@
       <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B8" s="59"/>
+      <c r="B8" s="61"/>
       <c r="C8" s="13" t="s">
         <v>229</v>
       </c>
@@ -11762,7 +11762,7 @@
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="13" t="s">
         <v>231</v>
       </c>
@@ -11778,7 +11778,7 @@
       <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="91.5" customHeight="1">
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="13" t="s">
         <v>232</v>
       </c>
@@ -11808,7 +11808,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="140.25" customHeight="1">
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="13" t="s">
         <v>235</v>
       </c>
@@ -11851,7 +11851,7 @@
       <c r="A13" s="62" t="s">
         <v>238</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="63"/>
       <c r="D13" s="58"/>
       <c r="E13" s="63"/>
@@ -11989,7 +11989,7 @@
       <c r="A3" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>239</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -12024,7 +12024,7 @@
       <c r="A4" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="18" t="s">
         <v>244</v>
       </c>
@@ -12057,7 +12057,7 @@
       <c r="A5" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="18" t="s">
         <v>247</v>
       </c>
@@ -12090,7 +12090,7 @@
       <c r="A6" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="18" t="s">
         <v>251</v>
       </c>
@@ -12133,7 +12133,7 @@
       <c r="A8" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="57" t="s">
         <v>254</v>
       </c>
       <c r="C8" s="22" t="s">
@@ -12168,7 +12168,7 @@
       <c r="A9" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="22" t="s">
         <v>259</v>
       </c>
@@ -12201,7 +12201,7 @@
       <c r="A10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="64" t="s">
         <v>262</v>
       </c>
@@ -12214,7 +12214,7 @@
       <c r="F10" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G10" s="59" t="s">
+      <c r="G10" s="61" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="12" t="s">
@@ -12234,7 +12234,7 @@
       <c r="A11" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="58"/>
       <c r="D11" s="63"/>
       <c r="E11" s="11" t="s">
@@ -12243,7 +12243,7 @@
       <c r="F11" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G11" s="59"/>
+      <c r="G11" s="61"/>
       <c r="H11" s="12" t="s">
         <v>27</v>
       </c>
@@ -12261,7 +12261,7 @@
       <c r="A12" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="B12" s="59"/>
+      <c r="B12" s="61"/>
       <c r="C12" s="22" t="s">
         <v>267</v>
       </c>
@@ -12294,7 +12294,7 @@
       <c r="A13" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="22" t="s">
         <v>271</v>
       </c>
@@ -12327,7 +12327,7 @@
       <c r="A14" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="59"/>
+      <c r="B14" s="61"/>
       <c r="C14" s="22" t="s">
         <v>274</v>
       </c>
@@ -12360,7 +12360,7 @@
       <c r="A15" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B15" s="59"/>
+      <c r="B15" s="61"/>
       <c r="C15" s="22" t="s">
         <v>279</v>
       </c>
@@ -12393,7 +12393,7 @@
       <c r="A16" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="59"/>
+      <c r="B16" s="61"/>
       <c r="C16" s="22" t="s">
         <v>282</v>
       </c>
@@ -12426,7 +12426,7 @@
       <c r="A17" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B17" s="59"/>
+      <c r="B17" s="61"/>
       <c r="C17" s="22" t="s">
         <v>286</v>
       </c>
@@ -12459,7 +12459,7 @@
       <c r="A18" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="B18" s="59"/>
+      <c r="B18" s="61"/>
       <c r="C18" s="22" t="s">
         <v>289</v>
       </c>
@@ -12492,7 +12492,7 @@
       <c r="A19" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B19" s="59"/>
+      <c r="B19" s="61"/>
       <c r="C19" s="22" t="s">
         <v>294</v>
       </c>
@@ -12525,7 +12525,7 @@
       <c r="A20" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B20" s="59"/>
+      <c r="B20" s="61"/>
       <c r="C20" s="22" t="s">
         <v>298</v>
       </c>
@@ -12558,7 +12558,7 @@
       <c r="A21" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="B21" s="59"/>
+      <c r="B21" s="61"/>
       <c r="C21" s="22" t="s">
         <v>303</v>
       </c>
@@ -12591,7 +12591,7 @@
       <c r="A22" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B22" s="59"/>
+      <c r="B22" s="61"/>
       <c r="C22" s="22" t="s">
         <v>305</v>
       </c>
@@ -12624,7 +12624,7 @@
       <c r="A23" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="B23" s="59"/>
+      <c r="B23" s="61"/>
       <c r="C23" s="22" t="s">
         <v>310</v>
       </c>
@@ -12657,7 +12657,7 @@
       <c r="A24" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="B24" s="59"/>
+      <c r="B24" s="61"/>
       <c r="C24" s="22" t="s">
         <v>314</v>
       </c>
@@ -12690,7 +12690,7 @@
       <c r="A25" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="B25" s="59"/>
+      <c r="B25" s="61"/>
       <c r="C25" s="22" t="s">
         <v>316</v>
       </c>
@@ -12720,7 +12720,7 @@
       <c r="A26" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="B26" s="59"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="64" t="s">
         <v>321</v>
       </c>
@@ -12733,10 +12733,10 @@
       <c r="F26" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G26" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="59" t="s">
+      <c r="G26" s="61" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="61" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="12" t="s">
@@ -12750,7 +12750,7 @@
       <c r="A27" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B27" s="59"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="58"/>
       <c r="D27" s="63"/>
       <c r="E27" s="11" t="s">
@@ -12759,14 +12759,14 @@
       <c r="F27" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="G27" s="59"/>
+      <c r="G27" s="61"/>
       <c r="H27" s="63"/>
     </row>
     <row r="28" spans="1:11" ht="76.5" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="B28" s="59"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="22" t="s">
         <v>329</v>
       </c>
@@ -12799,7 +12799,7 @@
       <c r="A29" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="B29" s="59"/>
+      <c r="B29" s="61"/>
       <c r="C29" s="22" t="s">
         <v>334</v>
       </c>
@@ -12832,7 +12832,7 @@
       <c r="A30" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B30" s="59"/>
+      <c r="B30" s="61"/>
       <c r="C30" s="22" t="s">
         <v>338</v>
       </c>
@@ -12865,7 +12865,7 @@
       <c r="A31" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B31" s="59"/>
+      <c r="B31" s="61"/>
       <c r="C31" s="22" t="s">
         <v>341</v>
       </c>
@@ -12980,7 +12980,7 @@
       <c r="A36" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B36" s="61" t="s">
+      <c r="B36" s="59" t="s">
         <v>349</v>
       </c>
       <c r="C36" s="22" t="s">
@@ -13015,7 +13015,7 @@
       <c r="A37" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B37" s="59"/>
+      <c r="B37" s="61"/>
       <c r="C37" s="23" t="s">
         <v>354</v>
       </c>
@@ -13152,7 +13152,7 @@
       <c r="A3" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>359</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -13341,7 +13341,7 @@
       <c r="A10" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="57" t="s">
         <v>385</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -13629,7 +13629,7 @@
       <c r="A20" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="59" t="s">
         <v>422</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -14247,7 +14247,7 @@
       <c r="A40" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="57" t="s">
         <v>505</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -14403,7 +14403,7 @@
       <c r="A46" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="59" t="s">
         <v>526</v>
       </c>
       <c r="C46" s="8" t="s">
@@ -14681,7 +14681,7 @@
       <c r="A56" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B56" s="43" t="s">
+      <c r="B56" s="46" t="s">
         <v>560</v>
       </c>
       <c r="C56" s="8" t="s">
@@ -14955,13 +14955,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8" ht="30">
       <c r="A3" t="s">
@@ -15049,13 +15049,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">

</xml_diff>

<commit_message>
QA: cerrar los ultimos 4 puntos abiertos - techo real de automatizacion alcanzado
Reintegros VAL-002 confirmado como el mismo bug ya filed (BUG-007/IMAS-4279,
En Progreso), Encuesta CE confirmada como config de Hotjar sin hook propio de
la app, Plan sin condicionado confirmado como campo real del backend pero sin
cuenta identificable en el pool, Atencion de Red y Cambio de mascota
reconfirmados como gaps de producto/datos, no de esfuerzo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Casos de Prueba.xlsx
+++ b/documentation/Casos de Prueba.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\ike\vetify-automation\automation\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ike\vetify-automation\automation\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC03823F-BDAF-4524-B9EA-0983DDACD442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42E3632-39DC-4CEC-B65A-A0667ECD9908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2685" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2686" uniqueCount="786">
   <si>
     <t>Total de Casos de Prueba</t>
   </si>
@@ -2705,9 +2705,6 @@
     <t>La cuenta Adquirente muestra el item Vetify Plus en el menu; la cuenta OSDE Capitado NO lo muestra -- confirmado en vivo 2026-08-30, coincide con la regla de negocio ya documentada (Vetify Plus aplica a todos los productos menos OSDE).</t>
   </si>
   <si>
-    <t>PROBADO EN VIVO 2026-08-30 con 2 cuentas distintas (Vetify Adquirente y OSDE Capitado con historial real de reintegros pagados). AMBAS fallan al llegar al selector de Mascota en el wizard Nuevo reintegro: la primera con un error generico Algo salio mal, la segunda con No hay mascotas registradas para tu documento pese a tener reintegros pagados a nombre de esa mascota. Posible bug real, no confirmado si es de datos de las cuentas de prueba o de la funcionalidad en si -- pendiente de que Alan lo revise directamente antes de automatizar.</t>
-  </si>
-  <si>
     <t>Depende de destrabar la fila anterior (Solicitud de reintegro) para poder llegar a este paso del wizard.</t>
   </si>
   <si>
@@ -2739,6 +2736,27 @@
   </si>
   <si>
     <t>Mismo hallazgo que la fila anterior (Consulta de condicionado) -- automatizacion del popup de PDF no resuelta pese a 7 rondas de intentos.</t>
+  </si>
+  <si>
+    <t>Usuario completa la carga de una credencial de mascota por primera vez.</t>
+  </si>
+  <si>
+    <t>1. Completar el formulario de alta de mascota. 2. Llegar a la pantalla de felicitacion (credencial lista). 3. Observar si aparece alguna encuesta de satisfaccion.</t>
+  </si>
+  <si>
+    <t>PROBADO EN VIVO 2026-08-30: se inspeccionaron los 19 bundles JS que carga la webapp. El unico codigo relacionado a survey es la libreria de terceros Hotjar; en el codigo propio de la app (_app) la unica llamada a window.hj es hj(identify) para analytics, sin ningun trigger custom atado a completar una credencial. Si esta encuesta existe, es config del dashboard de Hotjar (targeting por URL o tiempo), invisible al codigo y no deterministica. No es automatizable con Playwright de forma confiable.</t>
+  </si>
+  <si>
+    <t>Cuenta con un plan/producto cuyo campo pathCondicionado no tenga PDF mapeado.</t>
+  </si>
+  <si>
+    <t>1. Ir a Planes y coberturas con esa cuenta. 2. Expandir el plan. 3. Observar el comportamiento sin condicionado disponible.</t>
+  </si>
+  <si>
+    <t>PROBADO EN VIVO 2026-08-30: se confirmo que pathCondicionado es un campo real devuelto por el backend (GET plans engage por dni) -- el escenario es tecnicamente posible. Se intento escanear las 5 cuentas con storageState cacheado pegandole directo a la API (APIRequestContext), pero devolvio 401 en las 5: esa API usa un bearer token de localStorage que solo se adjunta con un navegador real, no replicable solo con cookies. Encontrar una cuenta real con este dato faltante necesitaria loguearse una por una (unas 24 cuentas) sin garantia de exito, o que dev/PO indique que producto/grupo especifico lo tiene. Ademas comparte el mismo bloqueo de popup+PDF ya documentado sin resolver en el caso base (CP-01/CP-02 de esta misma seccion).</t>
+  </si>
+  <si>
+    <t>PROBADO EN VIVO 2026-08-30 con 3 cuentas distintas en total. La llamada que falla es GET reintegros mascotas, 400 codigo VAL-002 Holder document must be a 7 or 8 digit DNI -- confirmado que es el mismo bug ya reportado en docs/bugs/BUG-007, Jira IMAS-4279, estado En Progreso (Mariana Navarro). No es un misterio nuevo: es un bug de backend ya trackeado que bloquea el wizard para toda cuenta cuyo DNI no tenga 7-8 digitos. Automatizacion queda pendiente de que se resuelva IMAS-4279, no de mas investigacion propia.</t>
   </si>
 </sst>
 </file>
@@ -3170,6 +3188,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3190,28 +3217,19 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -5063,734 +5081,734 @@
   <sheetData>
     <row r="2" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="3" spans="3:24">
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="51"/>
-      <c r="K3" s="49" t="s">
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="54"/>
+      <c r="K3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="51"/>
-      <c r="S3" s="49" t="s">
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="54"/>
+      <c r="S3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
-      <c r="V3" s="50"/>
-      <c r="W3" s="50"/>
-      <c r="X3" s="51"/>
+      <c r="T3" s="53"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="54"/>
     </row>
     <row r="4" spans="3:24">
-      <c r="C4" s="45"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="44"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="43"/>
-      <c r="O4" s="43"/>
-      <c r="P4" s="44"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="43"/>
-      <c r="U4" s="43"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="43"/>
-      <c r="X4" s="44"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="47"/>
+      <c r="S4" s="48"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="46"/>
+      <c r="V4" s="46"/>
+      <c r="W4" s="46"/>
+      <c r="X4" s="47"/>
     </row>
     <row r="5" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C5" s="42">
+      <c r="C5" s="45">
         <f>COUNTA('Flujo de Compra'!C3:C496,'Gestión de Usuario'!C3:C357,Perfil!C3:C199,Credenciales!C3:C199,Videollamadas!C3:C199,Reintegros!C2:C199,Misceláneas!C2:C199,'Control de Acceso'!C2:C199,'Sistema Caído'!C2:C199,'Funcionalidades Pendientes'!C2:C199)</f>
         <v>302</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-      <c r="K5" s="42">
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
+      <c r="K5" s="45">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")+COUNTIF(Reintegros!H:H,"Si")+COUNTIF(Misceláneas!H:H,"Si")+COUNTIF('Control de Acceso'!H:H,"Si")+COUNTIF('Sistema Caído'!H:H,"Si")+COUNTIF('Funcionalidades Pendientes'!H:H,"Si")</f>
         <v>222</v>
       </c>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="44"/>
-      <c r="S5" s="53">
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="47"/>
+      <c r="S5" s="56">
         <f>K5/C5</f>
         <v>0.73509933774834435</v>
       </c>
-      <c r="T5" s="43"/>
-      <c r="U5" s="43"/>
-      <c r="V5" s="43"/>
-      <c r="W5" s="43"/>
-      <c r="X5" s="44"/>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="47"/>
     </row>
     <row r="6" spans="3:24">
-      <c r="C6" s="45"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="43"/>
-      <c r="O6" s="43"/>
-      <c r="P6" s="44"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="43"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="43"/>
-      <c r="W6" s="43"/>
-      <c r="X6" s="44"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="47"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="46"/>
+      <c r="U6" s="46"/>
+      <c r="V6" s="46"/>
+      <c r="W6" s="46"/>
+      <c r="X6" s="47"/>
     </row>
     <row r="7" spans="3:24">
-      <c r="C7" s="45"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="44"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="44"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="43"/>
-      <c r="V7" s="43"/>
-      <c r="W7" s="43"/>
-      <c r="X7" s="44"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="47"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
+      <c r="O7" s="46"/>
+      <c r="P7" s="47"/>
+      <c r="S7" s="48"/>
+      <c r="T7" s="46"/>
+      <c r="U7" s="46"/>
+      <c r="V7" s="46"/>
+      <c r="W7" s="46"/>
+      <c r="X7" s="47"/>
     </row>
     <row r="8" spans="3:24">
-      <c r="C8" s="45"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="44"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="44"/>
-      <c r="S8" s="45"/>
-      <c r="T8" s="43"/>
-      <c r="U8" s="43"/>
-      <c r="V8" s="43"/>
-      <c r="W8" s="43"/>
-      <c r="X8" s="44"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="47"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="46"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="46"/>
+      <c r="O8" s="46"/>
+      <c r="P8" s="47"/>
+      <c r="S8" s="48"/>
+      <c r="T8" s="46"/>
+      <c r="U8" s="46"/>
+      <c r="V8" s="46"/>
+      <c r="W8" s="46"/>
+      <c r="X8" s="47"/>
     </row>
     <row r="9" spans="3:24">
-      <c r="C9" s="45"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="44"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="43"/>
-      <c r="U9" s="43"/>
-      <c r="V9" s="43"/>
-      <c r="W9" s="43"/>
-      <c r="X9" s="44"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46"/>
+      <c r="P9" s="47"/>
+      <c r="S9" s="48"/>
+      <c r="T9" s="46"/>
+      <c r="U9" s="46"/>
+      <c r="V9" s="46"/>
+      <c r="W9" s="46"/>
+      <c r="X9" s="47"/>
     </row>
     <row r="10" spans="3:24">
-      <c r="C10" s="45"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="44"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="43"/>
-      <c r="U10" s="43"/>
-      <c r="V10" s="43"/>
-      <c r="W10" s="43"/>
-      <c r="X10" s="44"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46"/>
+      <c r="P10" s="47"/>
+      <c r="S10" s="48"/>
+      <c r="T10" s="46"/>
+      <c r="U10" s="46"/>
+      <c r="V10" s="46"/>
+      <c r="W10" s="46"/>
+      <c r="X10" s="47"/>
     </row>
     <row r="11" spans="3:24">
-      <c r="C11" s="45"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="44"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="43"/>
-      <c r="U11" s="43"/>
-      <c r="V11" s="43"/>
-      <c r="W11" s="43"/>
-      <c r="X11" s="44"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="47"/>
+      <c r="S11" s="48"/>
+      <c r="T11" s="46"/>
+      <c r="U11" s="46"/>
+      <c r="V11" s="46"/>
+      <c r="W11" s="46"/>
+      <c r="X11" s="47"/>
     </row>
     <row r="12" spans="3:24">
-      <c r="C12" s="45"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="44"/>
-      <c r="S12" s="45"/>
-      <c r="T12" s="43"/>
-      <c r="U12" s="43"/>
-      <c r="V12" s="43"/>
-      <c r="W12" s="43"/>
-      <c r="X12" s="44"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="47"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="46"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
+      <c r="O12" s="46"/>
+      <c r="P12" s="47"/>
+      <c r="S12" s="48"/>
+      <c r="T12" s="46"/>
+      <c r="U12" s="46"/>
+      <c r="V12" s="46"/>
+      <c r="W12" s="46"/>
+      <c r="X12" s="47"/>
     </row>
     <row r="13" spans="3:24">
-      <c r="C13" s="45"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="44"/>
-      <c r="S13" s="45"/>
-      <c r="T13" s="43"/>
-      <c r="U13" s="43"/>
-      <c r="V13" s="43"/>
-      <c r="W13" s="43"/>
-      <c r="X13" s="44"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="47"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="47"/>
+      <c r="S13" s="48"/>
+      <c r="T13" s="46"/>
+      <c r="U13" s="46"/>
+      <c r="V13" s="46"/>
+      <c r="W13" s="46"/>
+      <c r="X13" s="47"/>
     </row>
     <row r="14" spans="3:24">
-      <c r="C14" s="45"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="44"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="43"/>
-      <c r="U14" s="43"/>
-      <c r="V14" s="43"/>
-      <c r="W14" s="43"/>
-      <c r="X14" s="44"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="47"/>
+      <c r="S14" s="48"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="47"/>
     </row>
     <row r="15" spans="3:24">
-      <c r="C15" s="45"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="43"/>
-      <c r="N15" s="43"/>
-      <c r="O15" s="43"/>
-      <c r="P15" s="44"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="43"/>
-      <c r="U15" s="43"/>
-      <c r="V15" s="43"/>
-      <c r="W15" s="43"/>
-      <c r="X15" s="44"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="47"/>
+      <c r="S15" s="48"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="47"/>
     </row>
     <row r="16" spans="3:24">
-      <c r="C16" s="45"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="44"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="43"/>
-      <c r="M16" s="43"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="44"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="43"/>
-      <c r="U16" s="43"/>
-      <c r="V16" s="43"/>
-      <c r="W16" s="43"/>
-      <c r="X16" s="44"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
+      <c r="P16" s="47"/>
+      <c r="S16" s="48"/>
+      <c r="T16" s="46"/>
+      <c r="U16" s="46"/>
+      <c r="V16" s="46"/>
+      <c r="W16" s="46"/>
+      <c r="X16" s="47"/>
     </row>
     <row r="17" spans="3:24">
-      <c r="C17" s="45"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="43"/>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="44"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="43"/>
-      <c r="U17" s="43"/>
-      <c r="V17" s="43"/>
-      <c r="W17" s="43"/>
-      <c r="X17" s="44"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="46"/>
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+      <c r="O17" s="46"/>
+      <c r="P17" s="47"/>
+      <c r="S17" s="48"/>
+      <c r="T17" s="46"/>
+      <c r="U17" s="46"/>
+      <c r="V17" s="46"/>
+      <c r="W17" s="46"/>
+      <c r="X17" s="47"/>
     </row>
     <row r="18" spans="3:24">
-      <c r="C18" s="45"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="43"/>
-      <c r="N18" s="43"/>
-      <c r="O18" s="43"/>
-      <c r="P18" s="44"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="43"/>
-      <c r="U18" s="43"/>
-      <c r="V18" s="43"/>
-      <c r="W18" s="43"/>
-      <c r="X18" s="44"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="47"/>
+      <c r="S18" s="48"/>
+      <c r="T18" s="46"/>
+      <c r="U18" s="46"/>
+      <c r="V18" s="46"/>
+      <c r="W18" s="46"/>
+      <c r="X18" s="47"/>
     </row>
     <row r="19" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C19" s="46"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
-      <c r="K19" s="46"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="48"/>
-      <c r="S19" s="46"/>
-      <c r="T19" s="47"/>
-      <c r="U19" s="47"/>
-      <c r="V19" s="47"/>
-      <c r="W19" s="47"/>
-      <c r="X19" s="48"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="51"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="51"/>
+      <c r="S19" s="49"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="50"/>
+      <c r="V19" s="50"/>
+      <c r="W19" s="50"/>
+      <c r="X19" s="51"/>
     </row>
     <row r="22" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="23" spans="3:24">
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="51"/>
-      <c r="K23" s="49" t="s">
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="54"/>
+      <c r="K23" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="L23" s="50"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
-      <c r="O23" s="50"/>
-      <c r="P23" s="51"/>
-      <c r="S23" s="49" t="s">
+      <c r="L23" s="53"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="53"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="54"/>
+      <c r="S23" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T23" s="50"/>
-      <c r="U23" s="50"/>
-      <c r="V23" s="50"/>
-      <c r="W23" s="50"/>
-      <c r="X23" s="51"/>
+      <c r="T23" s="53"/>
+      <c r="U23" s="53"/>
+      <c r="V23" s="53"/>
+      <c r="W23" s="53"/>
+      <c r="X23" s="54"/>
     </row>
     <row r="24" spans="3:24">
-      <c r="C24" s="45"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="44"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="43"/>
-      <c r="U24" s="43"/>
-      <c r="V24" s="43"/>
-      <c r="W24" s="43"/>
-      <c r="X24" s="44"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="47"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="47"/>
+      <c r="S24" s="48"/>
+      <c r="T24" s="46"/>
+      <c r="U24" s="46"/>
+      <c r="V24" s="46"/>
+      <c r="W24" s="46"/>
+      <c r="X24" s="47"/>
     </row>
     <row r="25" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C25" s="42">
+      <c r="C25" s="45">
         <f>COUNTIF('Flujo de Compra'!G:G,"Si")+COUNTIF('Gestión de Usuario'!G:G,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!G:G,"Si")+COUNTIF(Videollamadas!G:G,"Si")+COUNTIF(Reintegros!G:G,"Si")+COUNTIF(Misceláneas!G:G,"Si")+COUNTIF('Control de Acceso'!G:G,"Si")+COUNTIF('Sistema Caído'!G:G,"Si")+COUNTIF('Funcionalidades Pendientes'!G:G,"Si")</f>
         <v>166</v>
       </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
-      <c r="K25" s="42">
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
+      <c r="K25" s="45">
         <f>COUNTIFS('Flujo de Compra'!G:G,"Si",'Flujo de Compra'!H:H,"Si")+COUNTIFS('Gestión de Usuario'!G:G,"Si",'Gestión de Usuario'!H:H,"Si")+COUNTIFS(Perfil!G:G,"Si",Perfil!H:H,"Si")+COUNTIFS(Credenciales!G:G,"Si",Credenciales!H:H,"Si")+COUNTIFS(Videollamadas!G:G,"Si",Videollamadas!H:H,"Si")+COUNTIFS(Reintegros!G:G,"Si",Reintegros!H:H,"Si")+COUNTIFS(Misceláneas!G:G,"Si",Misceláneas!H:H,"Si")+COUNTIFS('Control de Acceso'!G:G,"Si",'Control de Acceso'!H:H,"Si")+COUNTIFS('Sistema Caído'!G:G,"Si",'Sistema Caído'!H:H,"Si")+COUNTIFS('Funcionalidades Pendientes'!G:G,"Si",'Funcionalidades Pendientes'!H:H,"Si")</f>
         <v>132</v>
       </c>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
-      <c r="N25" s="43"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="44"/>
-      <c r="S25" s="53">
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="47"/>
+      <c r="S25" s="56">
         <f>K25/C25</f>
         <v>0.79518072289156627</v>
       </c>
-      <c r="T25" s="43"/>
-      <c r="U25" s="43"/>
-      <c r="V25" s="43"/>
-      <c r="W25" s="43"/>
-      <c r="X25" s="44"/>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+      <c r="V25" s="46"/>
+      <c r="W25" s="46"/>
+      <c r="X25" s="47"/>
     </row>
     <row r="26" spans="3:24">
-      <c r="C26" s="45"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="44"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
-      <c r="N26" s="43"/>
-      <c r="O26" s="43"/>
-      <c r="P26" s="44"/>
-      <c r="S26" s="45"/>
-      <c r="T26" s="43"/>
-      <c r="U26" s="43"/>
-      <c r="V26" s="43"/>
-      <c r="W26" s="43"/>
-      <c r="X26" s="44"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="47"/>
+      <c r="S26" s="48"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+      <c r="V26" s="46"/>
+      <c r="W26" s="46"/>
+      <c r="X26" s="47"/>
     </row>
     <row r="27" spans="3:24">
-      <c r="C27" s="45"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="44"/>
-      <c r="S27" s="45"/>
-      <c r="T27" s="43"/>
-      <c r="U27" s="43"/>
-      <c r="V27" s="43"/>
-      <c r="W27" s="43"/>
-      <c r="X27" s="44"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="47"/>
+      <c r="S27" s="48"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+      <c r="V27" s="46"/>
+      <c r="W27" s="46"/>
+      <c r="X27" s="47"/>
     </row>
     <row r="28" spans="3:24">
-      <c r="C28" s="45"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="44"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="43"/>
-      <c r="P28" s="44"/>
-      <c r="S28" s="45"/>
-      <c r="T28" s="43"/>
-      <c r="U28" s="43"/>
-      <c r="V28" s="43"/>
-      <c r="W28" s="43"/>
-      <c r="X28" s="44"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="47"/>
+      <c r="K28" s="48"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
+      <c r="S28" s="48"/>
+      <c r="T28" s="46"/>
+      <c r="U28" s="46"/>
+      <c r="V28" s="46"/>
+      <c r="W28" s="46"/>
+      <c r="X28" s="47"/>
     </row>
     <row r="29" spans="3:24">
-      <c r="C29" s="45"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="43"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="44"/>
-      <c r="S29" s="45"/>
-      <c r="T29" s="43"/>
-      <c r="U29" s="43"/>
-      <c r="V29" s="43"/>
-      <c r="W29" s="43"/>
-      <c r="X29" s="44"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="47"/>
+      <c r="K29" s="48"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="47"/>
+      <c r="S29" s="48"/>
+      <c r="T29" s="46"/>
+      <c r="U29" s="46"/>
+      <c r="V29" s="46"/>
+      <c r="W29" s="46"/>
+      <c r="X29" s="47"/>
     </row>
     <row r="30" spans="3:24">
-      <c r="C30" s="45"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
-      <c r="K30" s="45"/>
-      <c r="L30" s="43"/>
-      <c r="M30" s="43"/>
-      <c r="N30" s="43"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="44"/>
-      <c r="S30" s="45"/>
-      <c r="T30" s="43"/>
-      <c r="U30" s="43"/>
-      <c r="V30" s="43"/>
-      <c r="W30" s="43"/>
-      <c r="X30" s="44"/>
+      <c r="C30" s="48"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="47"/>
+      <c r="K30" s="48"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="47"/>
+      <c r="S30" s="48"/>
+      <c r="T30" s="46"/>
+      <c r="U30" s="46"/>
+      <c r="V30" s="46"/>
+      <c r="W30" s="46"/>
+      <c r="X30" s="47"/>
     </row>
     <row r="31" spans="3:24">
-      <c r="C31" s="45"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="44"/>
-      <c r="K31" s="45"/>
-      <c r="L31" s="43"/>
-      <c r="M31" s="43"/>
-      <c r="N31" s="43"/>
-      <c r="O31" s="43"/>
-      <c r="P31" s="44"/>
-      <c r="S31" s="45"/>
-      <c r="T31" s="43"/>
-      <c r="U31" s="43"/>
-      <c r="V31" s="43"/>
-      <c r="W31" s="43"/>
-      <c r="X31" s="44"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="47"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="47"/>
+      <c r="S31" s="48"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+      <c r="V31" s="46"/>
+      <c r="W31" s="46"/>
+      <c r="X31" s="47"/>
     </row>
     <row r="32" spans="3:24">
-      <c r="C32" s="45"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="44"/>
-      <c r="K32" s="45"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="43"/>
-      <c r="N32" s="43"/>
-      <c r="O32" s="43"/>
-      <c r="P32" s="44"/>
-      <c r="S32" s="45"/>
-      <c r="T32" s="43"/>
-      <c r="U32" s="43"/>
-      <c r="V32" s="43"/>
-      <c r="W32" s="43"/>
-      <c r="X32" s="44"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="47"/>
+      <c r="K32" s="48"/>
+      <c r="L32" s="46"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
+      <c r="P32" s="47"/>
+      <c r="S32" s="48"/>
+      <c r="T32" s="46"/>
+      <c r="U32" s="46"/>
+      <c r="V32" s="46"/>
+      <c r="W32" s="46"/>
+      <c r="X32" s="47"/>
     </row>
     <row r="33" spans="3:24">
-      <c r="C33" s="45"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="44"/>
-      <c r="K33" s="45"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="43"/>
-      <c r="P33" s="44"/>
-      <c r="S33" s="45"/>
-      <c r="T33" s="43"/>
-      <c r="U33" s="43"/>
-      <c r="V33" s="43"/>
-      <c r="W33" s="43"/>
-      <c r="X33" s="44"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="47"/>
+      <c r="K33" s="48"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="47"/>
+      <c r="S33" s="48"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+      <c r="V33" s="46"/>
+      <c r="W33" s="46"/>
+      <c r="X33" s="47"/>
     </row>
     <row r="34" spans="3:24">
-      <c r="C34" s="45"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="44"/>
-      <c r="K34" s="45"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="44"/>
-      <c r="S34" s="45"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="44"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="47"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="46"/>
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="47"/>
+      <c r="S34" s="48"/>
+      <c r="T34" s="46"/>
+      <c r="U34" s="46"/>
+      <c r="V34" s="46"/>
+      <c r="W34" s="46"/>
+      <c r="X34" s="47"/>
     </row>
     <row r="35" spans="3:24">
-      <c r="C35" s="45"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="44"/>
-      <c r="K35" s="45"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="44"/>
-      <c r="S35" s="45"/>
-      <c r="T35" s="43"/>
-      <c r="U35" s="43"/>
-      <c r="V35" s="43"/>
-      <c r="W35" s="43"/>
-      <c r="X35" s="44"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="47"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="47"/>
+      <c r="S35" s="48"/>
+      <c r="T35" s="46"/>
+      <c r="U35" s="46"/>
+      <c r="V35" s="46"/>
+      <c r="W35" s="46"/>
+      <c r="X35" s="47"/>
     </row>
     <row r="36" spans="3:24">
-      <c r="C36" s="45"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="44"/>
-      <c r="K36" s="45"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="44"/>
-      <c r="S36" s="45"/>
-      <c r="T36" s="43"/>
-      <c r="U36" s="43"/>
-      <c r="V36" s="43"/>
-      <c r="W36" s="43"/>
-      <c r="X36" s="44"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="47"/>
+      <c r="K36" s="48"/>
+      <c r="L36" s="46"/>
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="47"/>
+      <c r="S36" s="48"/>
+      <c r="T36" s="46"/>
+      <c r="U36" s="46"/>
+      <c r="V36" s="46"/>
+      <c r="W36" s="46"/>
+      <c r="X36" s="47"/>
     </row>
     <row r="37" spans="3:24">
-      <c r="C37" s="45"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
-      <c r="K37" s="45"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="44"/>
-      <c r="S37" s="45"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="44"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="46"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="47"/>
+      <c r="K37" s="48"/>
+      <c r="L37" s="46"/>
+      <c r="M37" s="46"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="46"/>
+      <c r="P37" s="47"/>
+      <c r="S37" s="48"/>
+      <c r="T37" s="46"/>
+      <c r="U37" s="46"/>
+      <c r="V37" s="46"/>
+      <c r="W37" s="46"/>
+      <c r="X37" s="47"/>
     </row>
     <row r="38" spans="3:24">
-      <c r="C38" s="45"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="44"/>
-      <c r="K38" s="45"/>
-      <c r="L38" s="43"/>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="44"/>
-      <c r="S38" s="45"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="44"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="47"/>
+      <c r="K38" s="48"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="47"/>
+      <c r="S38" s="48"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="47"/>
     </row>
     <row r="39" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C39" s="46"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="48"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="47"/>
-      <c r="O39" s="47"/>
-      <c r="P39" s="48"/>
-      <c r="S39" s="46"/>
-      <c r="T39" s="47"/>
-      <c r="U39" s="47"/>
-      <c r="V39" s="47"/>
-      <c r="W39" s="47"/>
-      <c r="X39" s="48"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="50"/>
+      <c r="H39" s="51"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="51"/>
+      <c r="S39" s="49"/>
+      <c r="T39" s="50"/>
+      <c r="U39" s="50"/>
+      <c r="V39" s="50"/>
+      <c r="W39" s="50"/>
+      <c r="X39" s="51"/>
     </row>
     <row r="41" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="42" spans="3:24">
-      <c r="C42" s="49" t="s">
+      <c r="C42" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="50"/>
-      <c r="H42" s="51"/>
+      <c r="D42" s="53"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="53"/>
+      <c r="G42" s="53"/>
+      <c r="H42" s="54"/>
     </row>
     <row r="43" spans="3:24">
-      <c r="C43" s="45"/>
-      <c r="D43" s="43"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="43"/>
-      <c r="G43" s="43"/>
-      <c r="H43" s="44"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="47"/>
       <c r="K43" s="28"/>
       <c r="L43" s="28"/>
       <c r="M43" s="28"/>
@@ -5799,31 +5817,31 @@
       <c r="P43" s="28"/>
     </row>
     <row r="44" spans="3:24" ht="21" customHeight="1">
-      <c r="C44" s="53">
+      <c r="C44" s="56">
         <f>C25/C5</f>
         <v>0.54966887417218546</v>
       </c>
-      <c r="D44" s="43"/>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="44"/>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="47"/>
       <c r="K44" s="28"/>
-      <c r="L44" s="52" t="s">
+      <c r="L44" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="M44" s="43"/>
-      <c r="N44" s="43"/>
-      <c r="O44" s="43"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
+      <c r="O44" s="46"/>
       <c r="P44" s="29"/>
     </row>
     <row r="45" spans="3:24">
-      <c r="C45" s="45"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="44"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="47"/>
       <c r="K45" s="28"/>
       <c r="L45" s="30"/>
       <c r="M45" s="30"/>
@@ -5832,12 +5850,12 @@
       <c r="P45" s="29"/>
     </row>
     <row r="46" spans="3:24">
-      <c r="C46" s="45"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="44"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="46"/>
+      <c r="E46" s="46"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="46"/>
+      <c r="H46" s="47"/>
       <c r="K46" s="28"/>
       <c r="L46" s="31"/>
       <c r="M46" s="28" t="s">
@@ -5848,12 +5866,12 @@
       <c r="P46" s="28"/>
     </row>
     <row r="47" spans="3:24">
-      <c r="C47" s="45"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="43"/>
-      <c r="H47" s="44"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="46"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="46"/>
+      <c r="H47" s="47"/>
       <c r="K47" s="28"/>
       <c r="L47" s="32"/>
       <c r="M47" s="28" t="s">
@@ -5864,12 +5882,12 @@
       <c r="P47" s="28"/>
     </row>
     <row r="48" spans="3:24">
-      <c r="C48" s="45"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="48"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
       <c r="K48" s="28"/>
       <c r="L48" s="33"/>
       <c r="M48" s="28" t="s">
@@ -5880,12 +5898,12 @@
       <c r="P48" s="28"/>
     </row>
     <row r="49" spans="3:16">
-      <c r="C49" s="45"/>
-      <c r="D49" s="43"/>
-      <c r="E49" s="43"/>
-      <c r="F49" s="43"/>
-      <c r="G49" s="43"/>
-      <c r="H49" s="44"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="46"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="47"/>
       <c r="K49" s="28"/>
       <c r="L49" s="34"/>
       <c r="M49" s="28" t="s">
@@ -5896,12 +5914,12 @@
       <c r="P49" s="28"/>
     </row>
     <row r="50" spans="3:16">
-      <c r="C50" s="45"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="C50" s="48"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="47"/>
       <c r="K50" s="28"/>
       <c r="L50" s="35"/>
       <c r="M50" s="28" t="s">
@@ -5912,12 +5930,12 @@
       <c r="P50" s="28"/>
     </row>
     <row r="51" spans="3:16">
-      <c r="C51" s="45"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="47"/>
       <c r="K51" s="28"/>
       <c r="L51" s="28"/>
       <c r="M51" s="28"/>
@@ -5926,230 +5944,230 @@
       <c r="P51" s="28"/>
     </row>
     <row r="52" spans="3:16">
-      <c r="C52" s="45"/>
-      <c r="D52" s="43"/>
-      <c r="E52" s="43"/>
-      <c r="F52" s="43"/>
-      <c r="G52" s="43"/>
-      <c r="H52" s="44"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="47"/>
     </row>
     <row r="53" spans="3:16">
-      <c r="C53" s="45"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="44"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="47"/>
     </row>
     <row r="54" spans="3:16">
-      <c r="C54" s="45"/>
-      <c r="D54" s="43"/>
-      <c r="E54" s="43"/>
-      <c r="F54" s="43"/>
-      <c r="G54" s="43"/>
-      <c r="H54" s="44"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="47"/>
     </row>
     <row r="55" spans="3:16">
-      <c r="C55" s="45"/>
-      <c r="D55" s="43"/>
-      <c r="E55" s="43"/>
-      <c r="F55" s="43"/>
-      <c r="G55" s="43"/>
-      <c r="H55" s="44"/>
+      <c r="C55" s="48"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="47"/>
     </row>
     <row r="56" spans="3:16">
-      <c r="C56" s="45"/>
-      <c r="D56" s="43"/>
-      <c r="E56" s="43"/>
-      <c r="F56" s="43"/>
-      <c r="G56" s="43"/>
-      <c r="H56" s="44"/>
+      <c r="C56" s="48"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46"/>
+      <c r="F56" s="46"/>
+      <c r="G56" s="46"/>
+      <c r="H56" s="47"/>
     </row>
     <row r="57" spans="3:16">
-      <c r="C57" s="45"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="48"/>
+      <c r="D57" s="46"/>
+      <c r="E57" s="46"/>
+      <c r="F57" s="46"/>
+      <c r="G57" s="46"/>
+      <c r="H57" s="47"/>
     </row>
     <row r="58" spans="3:16" ht="15.75" customHeight="1">
-      <c r="C58" s="46"/>
-      <c r="D58" s="47"/>
-      <c r="E58" s="47"/>
-      <c r="F58" s="47"/>
-      <c r="G58" s="47"/>
-      <c r="H58" s="48"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="50"/>
+      <c r="E58" s="50"/>
+      <c r="F58" s="50"/>
+      <c r="G58" s="50"/>
+      <c r="H58" s="51"/>
     </row>
     <row r="62" spans="3:16">
-      <c r="C62" s="54" t="s">
+      <c r="C62" s="42" t="s">
         <v>585</v>
       </c>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="H62" s="54" t="s">
+      <c r="D62" s="42"/>
+      <c r="E62" s="42"/>
+      <c r="F62" s="42"/>
+      <c r="H62" s="42" t="s">
         <v>586</v>
       </c>
-      <c r="I62" s="54"/>
-      <c r="J62" s="54"/>
-      <c r="K62" s="54"/>
-      <c r="M62" s="54" t="s">
+      <c r="I62" s="42"/>
+      <c r="J62" s="42"/>
+      <c r="K62" s="42"/>
+      <c r="M62" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N62" s="54"/>
-      <c r="O62" s="54"/>
-      <c r="P62" s="54"/>
+      <c r="N62" s="42"/>
+      <c r="O62" s="42"/>
+      <c r="P62" s="42"/>
     </row>
     <row r="63" spans="3:16">
-      <c r="C63" s="54"/>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54"/>
-      <c r="F63" s="54"/>
-      <c r="H63" s="54"/>
-      <c r="I63" s="54"/>
-      <c r="J63" s="54"/>
-      <c r="K63" s="54"/>
-      <c r="M63" s="54"/>
-      <c r="N63" s="54"/>
-      <c r="O63" s="54"/>
-      <c r="P63" s="54"/>
+      <c r="C63" s="42"/>
+      <c r="D63" s="42"/>
+      <c r="E63" s="42"/>
+      <c r="F63" s="42"/>
+      <c r="H63" s="42"/>
+      <c r="I63" s="42"/>
+      <c r="J63" s="42"/>
+      <c r="K63" s="42"/>
+      <c r="M63" s="42"/>
+      <c r="N63" s="42"/>
+      <c r="O63" s="42"/>
+      <c r="P63" s="42"/>
     </row>
     <row r="64" spans="3:16">
-      <c r="C64" s="55">
+      <c r="C64" s="43">
         <f>COUNTIF('Flujo de Compra'!I:I,"Si")+COUNTIF('Gestión de Usuario'!I:I,"Si")+COUNTIF(Perfil!J:J,"Si")+COUNTIF(Credenciales!J:J,"Si")+COUNTIF(Videollamadas!J:J,"Si")</f>
-        <v>253</v>
-      </c>
-      <c r="D64" s="55"/>
-      <c r="E64" s="55"/>
-      <c r="F64" s="55"/>
-      <c r="H64" s="55">
+        <v>252</v>
+      </c>
+      <c r="D64" s="43"/>
+      <c r="E64" s="43"/>
+      <c r="F64" s="43"/>
+      <c r="H64" s="43">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")</f>
         <v>195</v>
       </c>
-      <c r="I64" s="55"/>
-      <c r="J64" s="55"/>
-      <c r="K64" s="55"/>
-      <c r="M64" s="56">
+      <c r="I64" s="43"/>
+      <c r="J64" s="43"/>
+      <c r="K64" s="43"/>
+      <c r="M64" s="44">
         <f t="shared" ref="M64" si="0">H64/C64</f>
-        <v>0.77075098814229248</v>
-      </c>
-      <c r="N64" s="56"/>
-      <c r="O64" s="56"/>
-      <c r="P64" s="56"/>
+        <v>0.77380952380952384</v>
+      </c>
+      <c r="N64" s="44"/>
+      <c r="O64" s="44"/>
+      <c r="P64" s="44"/>
     </row>
     <row r="65" spans="3:16">
-      <c r="C65" s="55"/>
-      <c r="D65" s="55"/>
-      <c r="E65" s="55"/>
-      <c r="F65" s="55"/>
-      <c r="H65" s="55"/>
-      <c r="I65" s="55"/>
-      <c r="J65" s="55"/>
-      <c r="K65" s="55"/>
-      <c r="M65" s="56"/>
-      <c r="N65" s="56"/>
-      <c r="O65" s="56"/>
-      <c r="P65" s="56"/>
+      <c r="C65" s="43"/>
+      <c r="D65" s="43"/>
+      <c r="E65" s="43"/>
+      <c r="F65" s="43"/>
+      <c r="H65" s="43"/>
+      <c r="I65" s="43"/>
+      <c r="J65" s="43"/>
+      <c r="K65" s="43"/>
+      <c r="M65" s="44"/>
+      <c r="N65" s="44"/>
+      <c r="O65" s="44"/>
+      <c r="P65" s="44"/>
     </row>
     <row r="66" spans="3:16">
-      <c r="C66" s="55"/>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55"/>
-      <c r="H66" s="55"/>
-      <c r="I66" s="55"/>
-      <c r="J66" s="55"/>
-      <c r="K66" s="55"/>
-      <c r="M66" s="56"/>
-      <c r="N66" s="56"/>
-      <c r="O66" s="56"/>
-      <c r="P66" s="56"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="H66" s="43"/>
+      <c r="I66" s="43"/>
+      <c r="J66" s="43"/>
+      <c r="K66" s="43"/>
+      <c r="M66" s="44"/>
+      <c r="N66" s="44"/>
+      <c r="O66" s="44"/>
+      <c r="P66" s="44"/>
     </row>
     <row r="69" spans="3:16">
-      <c r="C69" s="54" t="s">
+      <c r="C69" s="42" t="s">
         <v>588</v>
       </c>
-      <c r="D69" s="54"/>
-      <c r="E69" s="54"/>
-      <c r="F69" s="54"/>
-      <c r="H69" s="54" t="s">
+      <c r="D69" s="42"/>
+      <c r="E69" s="42"/>
+      <c r="F69" s="42"/>
+      <c r="H69" s="42" t="s">
         <v>589</v>
       </c>
-      <c r="I69" s="54"/>
-      <c r="J69" s="54"/>
-      <c r="K69" s="54"/>
-      <c r="M69" s="54" t="s">
+      <c r="I69" s="42"/>
+      <c r="J69" s="42"/>
+      <c r="K69" s="42"/>
+      <c r="M69" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N69" s="54"/>
-      <c r="O69" s="54"/>
-      <c r="P69" s="54"/>
+      <c r="N69" s="42"/>
+      <c r="O69" s="42"/>
+      <c r="P69" s="42"/>
     </row>
     <row r="70" spans="3:16">
-      <c r="C70" s="54"/>
-      <c r="D70" s="54"/>
-      <c r="E70" s="54"/>
-      <c r="F70" s="54"/>
-      <c r="H70" s="54"/>
-      <c r="I70" s="54"/>
-      <c r="J70" s="54"/>
-      <c r="K70" s="54"/>
-      <c r="M70" s="54"/>
-      <c r="N70" s="54"/>
-      <c r="O70" s="54"/>
-      <c r="P70" s="54"/>
+      <c r="C70" s="42"/>
+      <c r="D70" s="42"/>
+      <c r="E70" s="42"/>
+      <c r="F70" s="42"/>
+      <c r="H70" s="42"/>
+      <c r="I70" s="42"/>
+      <c r="J70" s="42"/>
+      <c r="K70" s="42"/>
+      <c r="M70" s="42"/>
+      <c r="N70" s="42"/>
+      <c r="O70" s="42"/>
+      <c r="P70" s="42"/>
     </row>
     <row r="71" spans="3:16">
-      <c r="C71" s="55">
+      <c r="C71" s="43">
         <f>COUNTIF(Perfil!K:K,"Si")+COUNTIF(Credenciales!K:K,"Si")+COUNTIF(Videollamadas!K:K,"Si")</f>
-        <v>74</v>
-      </c>
-      <c r="D71" s="55"/>
-      <c r="E71" s="55"/>
-      <c r="F71" s="55"/>
-      <c r="H71" s="55">
+        <v>73</v>
+      </c>
+      <c r="D71" s="43"/>
+      <c r="E71" s="43"/>
+      <c r="F71" s="43"/>
+      <c r="H71" s="43">
         <f>COUNTIF(Perfil!I:I,"Si")+COUNTIF(Credenciales!I:I,"Si")+COUNTIF(Videollamadas!I:I,"Si")</f>
         <v>60</v>
       </c>
-      <c r="I71" s="55"/>
-      <c r="J71" s="55"/>
-      <c r="K71" s="55"/>
-      <c r="M71" s="56">
+      <c r="I71" s="43"/>
+      <c r="J71" s="43"/>
+      <c r="K71" s="43"/>
+      <c r="M71" s="44">
         <f t="shared" ref="M71" si="1">H71/C71</f>
-        <v>0.81081081081081086</v>
-      </c>
-      <c r="N71" s="56"/>
-      <c r="O71" s="56"/>
-      <c r="P71" s="56"/>
+        <v>0.82191780821917804</v>
+      </c>
+      <c r="N71" s="44"/>
+      <c r="O71" s="44"/>
+      <c r="P71" s="44"/>
     </row>
     <row r="72" spans="3:16">
-      <c r="C72" s="55"/>
-      <c r="D72" s="55"/>
-      <c r="E72" s="55"/>
-      <c r="F72" s="55"/>
-      <c r="H72" s="55"/>
-      <c r="I72" s="55"/>
-      <c r="J72" s="55"/>
-      <c r="K72" s="55"/>
-      <c r="M72" s="56"/>
-      <c r="N72" s="56"/>
-      <c r="O72" s="56"/>
-      <c r="P72" s="56"/>
+      <c r="C72" s="43"/>
+      <c r="D72" s="43"/>
+      <c r="E72" s="43"/>
+      <c r="F72" s="43"/>
+      <c r="H72" s="43"/>
+      <c r="I72" s="43"/>
+      <c r="J72" s="43"/>
+      <c r="K72" s="43"/>
+      <c r="M72" s="44"/>
+      <c r="N72" s="44"/>
+      <c r="O72" s="44"/>
+      <c r="P72" s="44"/>
     </row>
     <row r="73" spans="3:16">
-      <c r="C73" s="55"/>
-      <c r="D73" s="55"/>
-      <c r="E73" s="55"/>
-      <c r="F73" s="55"/>
-      <c r="H73" s="55"/>
-      <c r="I73" s="55"/>
-      <c r="J73" s="55"/>
-      <c r="K73" s="55"/>
-      <c r="M73" s="56"/>
-      <c r="N73" s="56"/>
-      <c r="O73" s="56"/>
-      <c r="P73" s="56"/>
+      <c r="C73" s="43"/>
+      <c r="D73" s="43"/>
+      <c r="E73" s="43"/>
+      <c r="F73" s="43"/>
+      <c r="H73" s="43"/>
+      <c r="I73" s="43"/>
+      <c r="J73" s="43"/>
+      <c r="K73" s="43"/>
+      <c r="M73" s="44"/>
+      <c r="N73" s="44"/>
+      <c r="O73" s="44"/>
+      <c r="P73" s="44"/>
     </row>
     <row r="76" spans="3:16">
       <c r="C76" s="36" t="s">
@@ -6158,18 +6176,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C69:F70"/>
-    <mergeCell ref="C71:F73"/>
-    <mergeCell ref="H69:K70"/>
-    <mergeCell ref="H71:K73"/>
-    <mergeCell ref="M69:P70"/>
-    <mergeCell ref="M71:P73"/>
-    <mergeCell ref="C62:F63"/>
-    <mergeCell ref="C64:F66"/>
-    <mergeCell ref="H62:K63"/>
-    <mergeCell ref="H64:K66"/>
-    <mergeCell ref="M62:P63"/>
-    <mergeCell ref="M64:P66"/>
     <mergeCell ref="K5:P19"/>
     <mergeCell ref="K25:P39"/>
     <mergeCell ref="S3:X4"/>
@@ -6185,6 +6191,18 @@
     <mergeCell ref="C3:H4"/>
     <mergeCell ref="C25:H39"/>
     <mergeCell ref="K23:P24"/>
+    <mergeCell ref="C62:F63"/>
+    <mergeCell ref="C64:F66"/>
+    <mergeCell ref="H62:K63"/>
+    <mergeCell ref="H64:K66"/>
+    <mergeCell ref="M62:P63"/>
+    <mergeCell ref="M64:P66"/>
+    <mergeCell ref="C69:F70"/>
+    <mergeCell ref="C71:F73"/>
+    <mergeCell ref="H69:K70"/>
+    <mergeCell ref="H71:K73"/>
+    <mergeCell ref="M69:P70"/>
+    <mergeCell ref="M71:P73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6715,7 +6733,7 @@
         <v>756</v>
       </c>
       <c r="F16" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="G16" t="s">
         <v>28</v>
@@ -6741,7 +6759,7 @@
         <v>230</v>
       </c>
       <c r="F17" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="G17" t="s">
         <v>28</v>
@@ -6761,18 +6779,21 @@
         <v>724</v>
       </c>
       <c r="D18" t="s">
-        <v>230</v>
+        <v>782</v>
       </c>
       <c r="E18" t="s">
-        <v>230</v>
+        <v>783</v>
       </c>
       <c r="F18" t="s">
-        <v>230</v>
+        <v>784</v>
       </c>
       <c r="G18" t="s">
         <v>28</v>
       </c>
       <c r="H18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" t="s">
         <v>28</v>
       </c>
     </row>
@@ -6993,7 +7014,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -7002,7 +7023,7 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
       <c r="I2" s="12" t="s">
         <v>27</v>
       </c>
@@ -7011,7 +7032,7 @@
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -7239,7 +7260,7 @@
       <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="60" t="s">
+      <c r="B12" s="57" t="s">
         <v>51</v>
       </c>
       <c r="C12" s="22" t="s">
@@ -7305,7 +7326,7 @@
       <c r="A15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="59" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -7398,7 +7419,7 @@
       <c r="A19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="57" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="22" t="s">
@@ -7599,7 +7620,7 @@
       <c r="A27" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="61" t="s">
+      <c r="B27" s="59" t="s">
         <v>90</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -7719,7 +7740,7 @@
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="57" t="s">
         <v>104</v>
       </c>
       <c r="C32" s="22" t="s">
@@ -7866,7 +7887,7 @@
       <c r="A38" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="59" t="s">
         <v>120</v>
       </c>
       <c r="C38" s="18" t="s">
@@ -7919,7 +7940,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A40" s="57" t="s">
+      <c r="A40" s="60" t="s">
         <v>127</v>
       </c>
       <c r="B40" s="58"/>
@@ -7928,7 +7949,7 @@
       <c r="E40" s="58"/>
       <c r="F40" s="58"/>
       <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
+      <c r="H40" s="61"/>
       <c r="I40" s="12" t="s">
         <v>27</v>
       </c>
@@ -7937,7 +7958,7 @@
       <c r="A41" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="60" t="s">
+      <c r="B41" s="57" t="s">
         <v>22</v>
       </c>
       <c r="C41" s="22" t="s">
@@ -8165,7 +8186,7 @@
       <c r="A50" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="61" t="s">
+      <c r="B50" s="59" t="s">
         <v>51</v>
       </c>
       <c r="C50" s="18" t="s">
@@ -8231,7 +8252,7 @@
       <c r="A53" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="57" t="s">
         <v>58</v>
       </c>
       <c r="C53" s="22" t="s">
@@ -8324,7 +8345,7 @@
       <c r="A57" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="61" t="s">
+      <c r="B57" s="59" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="18" t="s">
@@ -8525,7 +8546,7 @@
       <c r="A65" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B65" s="60" t="s">
+      <c r="B65" s="57" t="s">
         <v>90</v>
       </c>
       <c r="C65" s="22" t="s">
@@ -8645,7 +8666,7 @@
       <c r="A70" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="59" t="s">
         <v>104</v>
       </c>
       <c r="C70" s="18" t="s">
@@ -8792,7 +8813,7 @@
       <c r="A76" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B76" s="60" t="s">
+      <c r="B76" s="57" t="s">
         <v>120</v>
       </c>
       <c r="C76" s="22" t="s">
@@ -8845,7 +8866,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A78" s="57" t="s">
+      <c r="A78" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B78" s="58"/>
@@ -8854,7 +8875,7 @@
       <c r="E78" s="58"/>
       <c r="F78" s="58"/>
       <c r="G78" s="58"/>
-      <c r="H78" s="59"/>
+      <c r="H78" s="61"/>
       <c r="I78" s="12" t="s">
         <v>27</v>
       </c>
@@ -8863,7 +8884,7 @@
       <c r="A79" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B79" s="61" t="s">
+      <c r="B79" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C79" s="18" t="s">
@@ -8954,7 +8975,7 @@
       <c r="A83" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B83" s="60" t="s">
+      <c r="B83" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C83" s="22" t="s">
@@ -9003,7 +9024,7 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A85" s="57" t="s">
+      <c r="A85" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B85" s="58"/>
@@ -9012,7 +9033,7 @@
       <c r="E85" s="58"/>
       <c r="F85" s="58"/>
       <c r="G85" s="58"/>
-      <c r="H85" s="59"/>
+      <c r="H85" s="61"/>
       <c r="I85" s="12" t="s">
         <v>27</v>
       </c>
@@ -9021,7 +9042,7 @@
       <c r="A86" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B86" s="61" t="s">
+      <c r="B86" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -9112,7 +9133,7 @@
       <c r="A90" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B90" s="60" t="s">
+      <c r="B90" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C90" s="22" t="s">
@@ -9172,12 +9193,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B86:B88"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A85:H85"/>
     <mergeCell ref="B32:B36"/>
@@ -9194,6 +9209,12 @@
     <mergeCell ref="B53:B55"/>
     <mergeCell ref="B19:B25"/>
     <mergeCell ref="B57:B63"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B86:B88"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="153" priority="564" operator="equal">
@@ -9423,7 +9444,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -9432,13 +9453,13 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
     </row>
     <row r="3" spans="1:9" ht="76.5" customHeight="1">
       <c r="A3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -9579,7 +9600,7 @@
       <c r="A9" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C9" s="22" t="s">
@@ -9697,7 +9718,7 @@
       <c r="A14" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -9844,7 +9865,7 @@
       <c r="A20" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -9988,7 +10009,7 @@
       <c r="A26" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -10077,7 +10098,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="60" t="s">
         <v>213</v>
       </c>
       <c r="B31" s="58"/>
@@ -10086,13 +10107,13 @@
       <c r="E31" s="58"/>
       <c r="F31" s="58"/>
       <c r="G31" s="58"/>
-      <c r="H31" s="59"/>
+      <c r="H31" s="61"/>
     </row>
     <row r="32" spans="1:9" ht="76.5" customHeight="1">
       <c r="A32" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -10233,7 +10254,7 @@
       <c r="A38" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C38" s="22" t="s">
@@ -10351,7 +10372,7 @@
       <c r="A43" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B43" s="61" t="s">
+      <c r="B43" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C43" s="18" t="s">
@@ -10498,7 +10519,7 @@
       <c r="A49" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B49" s="59" t="s">
+      <c r="B49" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -10642,7 +10663,7 @@
       <c r="A55" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -10731,7 +10752,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B60" s="58"/>
@@ -10740,13 +10761,13 @@
       <c r="E60" s="58"/>
       <c r="F60" s="58"/>
       <c r="G60" s="58"/>
-      <c r="H60" s="59"/>
+      <c r="H60" s="61"/>
     </row>
     <row r="61" spans="1:9" ht="76.5" customHeight="1">
       <c r="A61" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B61" s="61" t="s">
+      <c r="B61" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C61" s="18" t="s">
@@ -10887,7 +10908,7 @@
       <c r="A67" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B67" s="60" t="s">
+      <c r="B67" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C67" s="22" t="s">
@@ -11005,7 +11026,7 @@
       <c r="A72" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B72" s="61" t="s">
+      <c r="B72" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C72" s="18" t="s">
@@ -11152,7 +11173,7 @@
       <c r="A78" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B78" s="59" t="s">
+      <c r="B78" s="61" t="s">
         <v>611</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -11296,7 +11317,7 @@
       <c r="A84" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B84" s="59" t="s">
+      <c r="B84" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -11385,7 +11406,7 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A89" s="57" t="s">
+      <c r="A89" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B89" s="58"/>
@@ -11394,13 +11415,13 @@
       <c r="E89" s="58"/>
       <c r="F89" s="58"/>
       <c r="G89" s="58"/>
-      <c r="H89" s="59"/>
+      <c r="H89" s="61"/>
     </row>
     <row r="90" spans="1:9" ht="76.5" customHeight="1">
       <c r="A90" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="61" t="s">
+      <c r="B90" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C90" s="18" t="s">
@@ -11541,7 +11562,7 @@
       <c r="A96" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B96" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C96" s="22" t="s">
@@ -11659,7 +11680,7 @@
       <c r="A101" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B101" s="61" t="s">
+      <c r="B101" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C101" s="18" t="s">
@@ -11806,7 +11827,7 @@
       <c r="A107" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B107" s="59" t="s">
+      <c r="B107" s="61" t="s">
         <v>591</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -11950,7 +11971,7 @@
       <c r="A113" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B113" s="59" t="s">
+      <c r="B113" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -12040,6 +12061,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B101:B105"/>
+    <mergeCell ref="B107:B108"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="B96:B99"/>
     <mergeCell ref="A2:H2"/>
@@ -12056,14 +12085,6 @@
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="B55:B59"/>
     <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B101:B105"/>
-    <mergeCell ref="B107:B108"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="111" priority="525" operator="equal">
@@ -12469,7 +12490,7 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="59"/>
+      <c r="B2" s="61"/>
       <c r="C2" s="63"/>
       <c r="D2" s="58"/>
       <c r="E2" s="63"/>
@@ -12478,7 +12499,7 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="198" customHeight="1">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="61" t="s">
         <v>216</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -12510,8 +12531,8 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="76.5" customHeight="1">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="63" t="s">
         <v>221</v>
       </c>
@@ -12542,7 +12563,7 @@
     </row>
     <row r="5" spans="1:11" ht="45.75" customHeight="1">
       <c r="A5" s="63"/>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="63"/>
       <c r="D5" s="58"/>
       <c r="E5" s="6" t="s">
@@ -12554,7 +12575,7 @@
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:11" ht="121.5" customHeight="1">
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="63" t="s">
         <v>226</v>
       </c>
@@ -12584,7 +12605,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="45.75" customHeight="1">
-      <c r="B7" s="59"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="63"/>
       <c r="D7" s="58"/>
       <c r="E7" s="13" t="s">
@@ -12596,7 +12617,7 @@
       <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B8" s="59"/>
+      <c r="B8" s="61"/>
       <c r="C8" s="13" t="s">
         <v>229</v>
       </c>
@@ -12612,7 +12633,7 @@
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="13" t="s">
         <v>231</v>
       </c>
@@ -12628,7 +12649,7 @@
       <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="91.5" customHeight="1">
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="13" t="s">
         <v>232</v>
       </c>
@@ -12658,7 +12679,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="140.25" customHeight="1">
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="13" t="s">
         <v>235</v>
       </c>
@@ -12701,7 +12722,7 @@
       <c r="A13" s="62" t="s">
         <v>238</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="63"/>
       <c r="D13" s="58"/>
       <c r="E13" s="63"/>
@@ -12717,13 +12738,13 @@
         <v>702</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>773</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>774</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="F14" s="13" t="s">
         <v>775</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>776</v>
       </c>
       <c r="G14" s="13" t="s">
         <v>27</v>
@@ -12752,7 +12773,7 @@
         <v>230</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>27</v>
@@ -12900,7 +12921,7 @@
       <c r="A3" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>239</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -12935,7 +12956,7 @@
       <c r="A4" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="18" t="s">
         <v>244</v>
       </c>
@@ -12968,7 +12989,7 @@
       <c r="A5" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="18" t="s">
         <v>247</v>
       </c>
@@ -13001,7 +13022,7 @@
       <c r="A6" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="18" t="s">
         <v>251</v>
       </c>
@@ -13044,7 +13065,7 @@
       <c r="A8" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="57" t="s">
         <v>254</v>
       </c>
       <c r="C8" s="22" t="s">
@@ -13079,7 +13100,7 @@
       <c r="A9" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="22" t="s">
         <v>259</v>
       </c>
@@ -13112,7 +13133,7 @@
       <c r="A10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="64" t="s">
         <v>262</v>
       </c>
@@ -13125,7 +13146,7 @@
       <c r="F10" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G10" s="59" t="s">
+      <c r="G10" s="61" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="12" t="s">
@@ -13145,7 +13166,7 @@
       <c r="A11" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="58"/>
       <c r="D11" s="63"/>
       <c r="E11" s="11" t="s">
@@ -13154,7 +13175,7 @@
       <c r="F11" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G11" s="59"/>
+      <c r="G11" s="61"/>
       <c r="H11" s="12" t="s">
         <v>27</v>
       </c>
@@ -13172,7 +13193,7 @@
       <c r="A12" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="B12" s="59"/>
+      <c r="B12" s="61"/>
       <c r="C12" s="22" t="s">
         <v>267</v>
       </c>
@@ -13205,7 +13226,7 @@
       <c r="A13" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="22" t="s">
         <v>271</v>
       </c>
@@ -13238,7 +13259,7 @@
       <c r="A14" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="59"/>
+      <c r="B14" s="61"/>
       <c r="C14" s="22" t="s">
         <v>274</v>
       </c>
@@ -13271,7 +13292,7 @@
       <c r="A15" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B15" s="59"/>
+      <c r="B15" s="61"/>
       <c r="C15" s="22" t="s">
         <v>279</v>
       </c>
@@ -13304,7 +13325,7 @@
       <c r="A16" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="59"/>
+      <c r="B16" s="61"/>
       <c r="C16" s="22" t="s">
         <v>282</v>
       </c>
@@ -13337,7 +13358,7 @@
       <c r="A17" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B17" s="59"/>
+      <c r="B17" s="61"/>
       <c r="C17" s="22" t="s">
         <v>286</v>
       </c>
@@ -13370,7 +13391,7 @@
       <c r="A18" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="B18" s="59"/>
+      <c r="B18" s="61"/>
       <c r="C18" s="22" t="s">
         <v>289</v>
       </c>
@@ -13403,7 +13424,7 @@
       <c r="A19" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B19" s="59"/>
+      <c r="B19" s="61"/>
       <c r="C19" s="22" t="s">
         <v>294</v>
       </c>
@@ -13436,7 +13457,7 @@
       <c r="A20" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B20" s="59"/>
+      <c r="B20" s="61"/>
       <c r="C20" s="22" t="s">
         <v>298</v>
       </c>
@@ -13469,7 +13490,7 @@
       <c r="A21" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="B21" s="59"/>
+      <c r="B21" s="61"/>
       <c r="C21" s="22" t="s">
         <v>303</v>
       </c>
@@ -13502,7 +13523,7 @@
       <c r="A22" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B22" s="59"/>
+      <c r="B22" s="61"/>
       <c r="C22" s="22" t="s">
         <v>305</v>
       </c>
@@ -13535,7 +13556,7 @@
       <c r="A23" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="B23" s="59"/>
+      <c r="B23" s="61"/>
       <c r="C23" s="22" t="s">
         <v>310</v>
       </c>
@@ -13568,7 +13589,7 @@
       <c r="A24" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="B24" s="59"/>
+      <c r="B24" s="61"/>
       <c r="C24" s="22" t="s">
         <v>314</v>
       </c>
@@ -13601,7 +13622,7 @@
       <c r="A25" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="B25" s="59"/>
+      <c r="B25" s="61"/>
       <c r="C25" s="22" t="s">
         <v>316</v>
       </c>
@@ -13631,7 +13652,7 @@
       <c r="A26" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="B26" s="59"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="64" t="s">
         <v>321</v>
       </c>
@@ -13644,10 +13665,10 @@
       <c r="F26" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G26" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="59" t="s">
+      <c r="G26" s="61" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="61" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="12" t="s">
@@ -13661,7 +13682,7 @@
       <c r="A27" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B27" s="59"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="58"/>
       <c r="D27" s="63"/>
       <c r="E27" s="11" t="s">
@@ -13670,14 +13691,14 @@
       <c r="F27" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="G27" s="59"/>
+      <c r="G27" s="61"/>
       <c r="H27" s="63"/>
     </row>
     <row r="28" spans="1:11" ht="76.5" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="B28" s="59"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="22" t="s">
         <v>329</v>
       </c>
@@ -13710,7 +13731,7 @@
       <c r="A29" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="B29" s="59"/>
+      <c r="B29" s="61"/>
       <c r="C29" s="22" t="s">
         <v>334</v>
       </c>
@@ -13743,7 +13764,7 @@
       <c r="A30" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B30" s="59"/>
+      <c r="B30" s="61"/>
       <c r="C30" s="22" t="s">
         <v>338</v>
       </c>
@@ -13776,7 +13797,7 @@
       <c r="A31" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B31" s="59"/>
+      <c r="B31" s="61"/>
       <c r="C31" s="22" t="s">
         <v>341</v>
       </c>
@@ -13891,7 +13912,7 @@
       <c r="A36" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B36" s="61" t="s">
+      <c r="B36" s="59" t="s">
         <v>349</v>
       </c>
       <c r="C36" s="22" t="s">
@@ -13926,7 +13947,7 @@
       <c r="A37" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B37" s="59"/>
+      <c r="B37" s="61"/>
       <c r="C37" s="23" t="s">
         <v>354</v>
       </c>
@@ -13955,7 +13976,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="60">
+    <row r="38" spans="1:11" ht="240">
       <c r="B38" s="12" t="s">
         <v>704</v>
       </c>
@@ -13963,13 +13984,13 @@
         <v>705</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>230</v>
+        <v>779</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>230</v>
+        <v>780</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>230</v>
+        <v>781</v>
       </c>
       <c r="G38" s="12" t="s">
         <v>28</v>
@@ -13981,10 +14002,10 @@
         <v>28</v>
       </c>
       <c r="J38" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K38" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -14095,7 +14116,7 @@
       <c r="A3" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>359</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -14284,7 +14305,7 @@
       <c r="A10" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="57" t="s">
         <v>385</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -14572,7 +14593,7 @@
       <c r="A20" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="59" t="s">
         <v>422</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -15190,7 +15211,7 @@
       <c r="A40" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="57" t="s">
         <v>505</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -15346,7 +15367,7 @@
       <c r="A46" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="59" t="s">
         <v>526</v>
       </c>
       <c r="C46" s="8" t="s">
@@ -15624,7 +15645,7 @@
       <c r="A56" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B56" s="43" t="s">
+      <c r="B56" s="46" t="s">
         <v>560</v>
       </c>
       <c r="C56" s="8" t="s">
@@ -15901,13 +15922,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:9" ht="30">
       <c r="A3" t="s">
@@ -15952,7 +15973,7 @@
         <v>230</v>
       </c>
       <c r="F4" t="s">
-        <v>768</v>
+        <v>785</v>
       </c>
       <c r="G4" t="s">
         <v>27</v>
@@ -15978,7 +15999,7 @@
         <v>230</v>
       </c>
       <c r="F5" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="G5" t="s">
         <v>27</v>
@@ -16004,7 +16025,7 @@
         <v>230</v>
       </c>
       <c r="F6" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="G6" t="s">
         <v>27</v>
@@ -16030,7 +16051,7 @@
         <v>230</v>
       </c>
       <c r="F7" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="G7" t="s">
         <v>28</v>
@@ -16050,13 +16071,13 @@
         <v>700</v>
       </c>
       <c r="D8" t="s">
+        <v>770</v>
+      </c>
+      <c r="E8" t="s">
         <v>771</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>772</v>
-      </c>
-      <c r="F8" t="s">
-        <v>773</v>
       </c>
       <c r="G8" t="s">
         <v>27</v>
@@ -16128,13 +16149,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">

</xml_diff>

<commit_message>
QA: automatizar IMAS-4408 escenarios 2/3 (unico plan Inactivo/Dado de baja) via mock de red
Resuelve IMP-015 sin necesitar la cuenta real que la escalacion a Oscar
denego por ahora: page.route()+fulfill() reemplaza de forma confiable
la respuesta de pets/my-products (Home/Mascotas/Planes/Videollamada) y
reintegros/mascotas (Reintegros) para simular una cuenta sin ningun
plan operable, sin depender de ninguna cuenta real ni consumir el pool.

Nuevo: src/helpers/mockPlanState.ts, tests/projects/vetify-webapp/
plan-state.spec.ts (verificado Desktop+Mobile), POM minimo
NuevoReintegroPage.ts, locator petCredentialCards en HomePage.ts.

CP09/CP10 pasan de bloqueados a verificados en el diseno de casos.
+1 fila en Casos de Prueba.xlsx (309 total, 229 automatizados, 74%).

De paso: pauscalzo@hotmail.com (cuenta de evidencia del Escenario 1)
degrado desde el 2026-08-28 -- ya no sirve como evidencia limpia sin
re-verificar.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Casos de Prueba.xlsx
+++ b/documentation/Casos de Prueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ike\vetify-automation\automation\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F29E309-7E6E-4E39-9E79-7BE971ADC978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089ACAFD-0963-4ED9-B2AA-E9D22267A88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="12645" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2735" uniqueCount="804">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2746" uniqueCount="809">
   <si>
     <t>Total de Casos de Prueba</t>
   </si>
@@ -2811,6 +2811,21 @@
   </si>
   <si>
     <t>El item Cooper es visible dentro de Beneficios. Verificado en Desktop y Mobile (Android). Nota: el menu de OSDE Adquirente depende del producto real (policyId) de la cuenta, no del segmento -- no automatizado con una asercion fija a proposito, ver docs/conocimiento-sistema.md.</t>
+  </si>
+  <si>
+    <t>TS-06 Estado del plan (IMAS-4408)</t>
+  </si>
+  <si>
+    <t>Cuenta cuyo unico plan no esta operable no muestra ninguna credencial ni permite operar</t>
+  </si>
+  <si>
+    <t>Usuario cuyo unico plan paso a Inactivo (falta de pago) o fue Dado de baja definitivamente.</t>
+  </si>
+  <si>
+    <t>1. Cargar Home, Mascotas, Planes y coberturas. 2. Intentar agendar videollamada. 3. Intentar iniciar un reintegro nuevo.</t>
+  </si>
+  <si>
+    <t>Ninguna pantalla muestra credencial ni permite operar (Home vacio, Mascotas sin tarjetas, Planes No hay planes por el momento, Videollamada bloquea con Completa su credencial, Reintegros No hay mascotas registradas). Login sigue funcionando con normalidad. Simulado con mock de red (page.route) sobre pets/my-products y reintegros/mascotas, sin depender de una cuenta real con este estado (IMP-015: no hay self-service para conseguirla, escalado a Oscar 2026-08-31, respuesta no por ahora).</t>
   </si>
 </sst>
 </file>
@@ -3242,6 +3257,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3262,28 +3286,19 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -5135,734 +5150,734 @@
   <sheetData>
     <row r="2" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="3" spans="3:24">
-      <c r="C3" s="49" t="s">
+      <c r="C3" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="51"/>
-      <c r="K3" s="49" t="s">
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="54"/>
+      <c r="K3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="51"/>
-      <c r="S3" s="49" t="s">
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="54"/>
+      <c r="S3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
-      <c r="V3" s="50"/>
-      <c r="W3" s="50"/>
-      <c r="X3" s="51"/>
+      <c r="T3" s="53"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="54"/>
     </row>
     <row r="4" spans="3:24">
-      <c r="C4" s="45"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="44"/>
-      <c r="K4" s="45"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="43"/>
-      <c r="O4" s="43"/>
-      <c r="P4" s="44"/>
-      <c r="S4" s="45"/>
-      <c r="T4" s="43"/>
-      <c r="U4" s="43"/>
-      <c r="V4" s="43"/>
-      <c r="W4" s="43"/>
-      <c r="X4" s="44"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="47"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="46"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="47"/>
+      <c r="S4" s="48"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="46"/>
+      <c r="V4" s="46"/>
+      <c r="W4" s="46"/>
+      <c r="X4" s="47"/>
     </row>
     <row r="5" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C5" s="42">
+      <c r="C5" s="45">
         <f>COUNTA('Flujo de Compra'!C3:C496,'Gestión de Usuario'!C3:C357,Perfil!C3:C199,Credenciales!C3:C199,Videollamadas!C3:C199,Reintegros!C2:C199,Misceláneas!C2:C199,'Control de Acceso'!C2:C199,'Sistema Caído'!C2:C199,'Funcionalidades Pendientes'!C2:C199)</f>
-        <v>308</v>
-      </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-      <c r="K5" s="42">
+        <v>309</v>
+      </c>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
+      <c r="K5" s="45">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")+COUNTIF(Reintegros!H:H,"Si")+COUNTIF(Misceláneas!H:H,"Si")+COUNTIF('Control de Acceso'!H:H,"Si")+COUNTIF('Sistema Caído'!H:H,"Si")+COUNTIF('Funcionalidades Pendientes'!H:H,"Si")</f>
-        <v>228</v>
-      </c>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="43"/>
-      <c r="O5" s="43"/>
-      <c r="P5" s="44"/>
-      <c r="S5" s="53">
+        <v>229</v>
+      </c>
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="47"/>
+      <c r="S5" s="56">
         <f>K5/C5</f>
-        <v>0.74025974025974028</v>
-      </c>
-      <c r="T5" s="43"/>
-      <c r="U5" s="43"/>
-      <c r="V5" s="43"/>
-      <c r="W5" s="43"/>
-      <c r="X5" s="44"/>
+        <v>0.74110032362459544</v>
+      </c>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="47"/>
     </row>
     <row r="6" spans="3:24">
-      <c r="C6" s="45"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="44"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="43"/>
-      <c r="O6" s="43"/>
-      <c r="P6" s="44"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="43"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="43"/>
-      <c r="W6" s="43"/>
-      <c r="X6" s="44"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
+      <c r="O6" s="46"/>
+      <c r="P6" s="47"/>
+      <c r="S6" s="48"/>
+      <c r="T6" s="46"/>
+      <c r="U6" s="46"/>
+      <c r="V6" s="46"/>
+      <c r="W6" s="46"/>
+      <c r="X6" s="47"/>
     </row>
     <row r="7" spans="3:24">
-      <c r="C7" s="45"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="44"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="43"/>
-      <c r="O7" s="43"/>
-      <c r="P7" s="44"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="43"/>
-      <c r="U7" s="43"/>
-      <c r="V7" s="43"/>
-      <c r="W7" s="43"/>
-      <c r="X7" s="44"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="46"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="46"/>
+      <c r="G7" s="46"/>
+      <c r="H7" s="47"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="46"/>
+      <c r="N7" s="46"/>
+      <c r="O7" s="46"/>
+      <c r="P7" s="47"/>
+      <c r="S7" s="48"/>
+      <c r="T7" s="46"/>
+      <c r="U7" s="46"/>
+      <c r="V7" s="46"/>
+      <c r="W7" s="46"/>
+      <c r="X7" s="47"/>
     </row>
     <row r="8" spans="3:24">
-      <c r="C8" s="45"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="44"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
-      <c r="N8" s="43"/>
-      <c r="O8" s="43"/>
-      <c r="P8" s="44"/>
-      <c r="S8" s="45"/>
-      <c r="T8" s="43"/>
-      <c r="U8" s="43"/>
-      <c r="V8" s="43"/>
-      <c r="W8" s="43"/>
-      <c r="X8" s="44"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="46"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="47"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="46"/>
+      <c r="M8" s="46"/>
+      <c r="N8" s="46"/>
+      <c r="O8" s="46"/>
+      <c r="P8" s="47"/>
+      <c r="S8" s="48"/>
+      <c r="T8" s="46"/>
+      <c r="U8" s="46"/>
+      <c r="V8" s="46"/>
+      <c r="W8" s="46"/>
+      <c r="X8" s="47"/>
     </row>
     <row r="9" spans="3:24">
-      <c r="C9" s="45"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="44"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="43"/>
-      <c r="P9" s="44"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="43"/>
-      <c r="U9" s="43"/>
-      <c r="V9" s="43"/>
-      <c r="W9" s="43"/>
-      <c r="X9" s="44"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="46"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="46"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="46"/>
+      <c r="M9" s="46"/>
+      <c r="N9" s="46"/>
+      <c r="O9" s="46"/>
+      <c r="P9" s="47"/>
+      <c r="S9" s="48"/>
+      <c r="T9" s="46"/>
+      <c r="U9" s="46"/>
+      <c r="V9" s="46"/>
+      <c r="W9" s="46"/>
+      <c r="X9" s="47"/>
     </row>
     <row r="10" spans="3:24">
-      <c r="C10" s="45"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
-      <c r="N10" s="43"/>
-      <c r="O10" s="43"/>
-      <c r="P10" s="44"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="43"/>
-      <c r="U10" s="43"/>
-      <c r="V10" s="43"/>
-      <c r="W10" s="43"/>
-      <c r="X10" s="44"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="46"/>
+      <c r="M10" s="46"/>
+      <c r="N10" s="46"/>
+      <c r="O10" s="46"/>
+      <c r="P10" s="47"/>
+      <c r="S10" s="48"/>
+      <c r="T10" s="46"/>
+      <c r="U10" s="46"/>
+      <c r="V10" s="46"/>
+      <c r="W10" s="46"/>
+      <c r="X10" s="47"/>
     </row>
     <row r="11" spans="3:24">
-      <c r="C11" s="45"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="44"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="43"/>
-      <c r="O11" s="43"/>
-      <c r="P11" s="44"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="43"/>
-      <c r="U11" s="43"/>
-      <c r="V11" s="43"/>
-      <c r="W11" s="43"/>
-      <c r="X11" s="44"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="46"/>
+      <c r="M11" s="46"/>
+      <c r="N11" s="46"/>
+      <c r="O11" s="46"/>
+      <c r="P11" s="47"/>
+      <c r="S11" s="48"/>
+      <c r="T11" s="46"/>
+      <c r="U11" s="46"/>
+      <c r="V11" s="46"/>
+      <c r="W11" s="46"/>
+      <c r="X11" s="47"/>
     </row>
     <row r="12" spans="3:24">
-      <c r="C12" s="45"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="43"/>
-      <c r="P12" s="44"/>
-      <c r="S12" s="45"/>
-      <c r="T12" s="43"/>
-      <c r="U12" s="43"/>
-      <c r="V12" s="43"/>
-      <c r="W12" s="43"/>
-      <c r="X12" s="44"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="47"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="46"/>
+      <c r="M12" s="46"/>
+      <c r="N12" s="46"/>
+      <c r="O12" s="46"/>
+      <c r="P12" s="47"/>
+      <c r="S12" s="48"/>
+      <c r="T12" s="46"/>
+      <c r="U12" s="46"/>
+      <c r="V12" s="46"/>
+      <c r="W12" s="46"/>
+      <c r="X12" s="47"/>
     </row>
     <row r="13" spans="3:24">
-      <c r="C13" s="45"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="44"/>
-      <c r="S13" s="45"/>
-      <c r="T13" s="43"/>
-      <c r="U13" s="43"/>
-      <c r="V13" s="43"/>
-      <c r="W13" s="43"/>
-      <c r="X13" s="44"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="47"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="46"/>
+      <c r="M13" s="46"/>
+      <c r="N13" s="46"/>
+      <c r="O13" s="46"/>
+      <c r="P13" s="47"/>
+      <c r="S13" s="48"/>
+      <c r="T13" s="46"/>
+      <c r="U13" s="46"/>
+      <c r="V13" s="46"/>
+      <c r="W13" s="46"/>
+      <c r="X13" s="47"/>
     </row>
     <row r="14" spans="3:24">
-      <c r="C14" s="45"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
-      <c r="O14" s="43"/>
-      <c r="P14" s="44"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="43"/>
-      <c r="U14" s="43"/>
-      <c r="V14" s="43"/>
-      <c r="W14" s="43"/>
-      <c r="X14" s="44"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="46"/>
+      <c r="M14" s="46"/>
+      <c r="N14" s="46"/>
+      <c r="O14" s="46"/>
+      <c r="P14" s="47"/>
+      <c r="S14" s="48"/>
+      <c r="T14" s="46"/>
+      <c r="U14" s="46"/>
+      <c r="V14" s="46"/>
+      <c r="W14" s="46"/>
+      <c r="X14" s="47"/>
     </row>
     <row r="15" spans="3:24">
-      <c r="C15" s="45"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="44"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="43"/>
-      <c r="N15" s="43"/>
-      <c r="O15" s="43"/>
-      <c r="P15" s="44"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="43"/>
-      <c r="U15" s="43"/>
-      <c r="V15" s="43"/>
-      <c r="W15" s="43"/>
-      <c r="X15" s="44"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+      <c r="O15" s="46"/>
+      <c r="P15" s="47"/>
+      <c r="S15" s="48"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="47"/>
     </row>
     <row r="16" spans="3:24">
-      <c r="C16" s="45"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="44"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="43"/>
-      <c r="M16" s="43"/>
-      <c r="N16" s="43"/>
-      <c r="O16" s="43"/>
-      <c r="P16" s="44"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="43"/>
-      <c r="U16" s="43"/>
-      <c r="V16" s="43"/>
-      <c r="W16" s="43"/>
-      <c r="X16" s="44"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
+      <c r="P16" s="47"/>
+      <c r="S16" s="48"/>
+      <c r="T16" s="46"/>
+      <c r="U16" s="46"/>
+      <c r="V16" s="46"/>
+      <c r="W16" s="46"/>
+      <c r="X16" s="47"/>
     </row>
     <row r="17" spans="3:24">
-      <c r="C17" s="45"/>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="44"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="43"/>
-      <c r="M17" s="43"/>
-      <c r="N17" s="43"/>
-      <c r="O17" s="43"/>
-      <c r="P17" s="44"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="43"/>
-      <c r="U17" s="43"/>
-      <c r="V17" s="43"/>
-      <c r="W17" s="43"/>
-      <c r="X17" s="44"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="46"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="46"/>
+      <c r="M17" s="46"/>
+      <c r="N17" s="46"/>
+      <c r="O17" s="46"/>
+      <c r="P17" s="47"/>
+      <c r="S17" s="48"/>
+      <c r="T17" s="46"/>
+      <c r="U17" s="46"/>
+      <c r="V17" s="46"/>
+      <c r="W17" s="46"/>
+      <c r="X17" s="47"/>
     </row>
     <row r="18" spans="3:24">
-      <c r="C18" s="45"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="44"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="43"/>
-      <c r="N18" s="43"/>
-      <c r="O18" s="43"/>
-      <c r="P18" s="44"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="43"/>
-      <c r="U18" s="43"/>
-      <c r="V18" s="43"/>
-      <c r="W18" s="43"/>
-      <c r="X18" s="44"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="46"/>
+      <c r="M18" s="46"/>
+      <c r="N18" s="46"/>
+      <c r="O18" s="46"/>
+      <c r="P18" s="47"/>
+      <c r="S18" s="48"/>
+      <c r="T18" s="46"/>
+      <c r="U18" s="46"/>
+      <c r="V18" s="46"/>
+      <c r="W18" s="46"/>
+      <c r="X18" s="47"/>
     </row>
     <row r="19" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C19" s="46"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
-      <c r="K19" s="46"/>
-      <c r="L19" s="47"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="47"/>
-      <c r="P19" s="48"/>
-      <c r="S19" s="46"/>
-      <c r="T19" s="47"/>
-      <c r="U19" s="47"/>
-      <c r="V19" s="47"/>
-      <c r="W19" s="47"/>
-      <c r="X19" s="48"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="51"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="50"/>
+      <c r="P19" s="51"/>
+      <c r="S19" s="49"/>
+      <c r="T19" s="50"/>
+      <c r="U19" s="50"/>
+      <c r="V19" s="50"/>
+      <c r="W19" s="50"/>
+      <c r="X19" s="51"/>
     </row>
     <row r="22" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="23" spans="3:24">
-      <c r="C23" s="49" t="s">
+      <c r="C23" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="51"/>
-      <c r="K23" s="49" t="s">
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="54"/>
+      <c r="K23" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="L23" s="50"/>
-      <c r="M23" s="50"/>
-      <c r="N23" s="50"/>
-      <c r="O23" s="50"/>
-      <c r="P23" s="51"/>
-      <c r="S23" s="49" t="s">
+      <c r="L23" s="53"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="53"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="54"/>
+      <c r="S23" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="T23" s="50"/>
-      <c r="U23" s="50"/>
-      <c r="V23" s="50"/>
-      <c r="W23" s="50"/>
-      <c r="X23" s="51"/>
+      <c r="T23" s="53"/>
+      <c r="U23" s="53"/>
+      <c r="V23" s="53"/>
+      <c r="W23" s="53"/>
+      <c r="X23" s="54"/>
     </row>
     <row r="24" spans="3:24">
-      <c r="C24" s="45"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="43"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="43"/>
-      <c r="H24" s="44"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
-      <c r="N24" s="43"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="44"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="43"/>
-      <c r="U24" s="43"/>
-      <c r="V24" s="43"/>
-      <c r="W24" s="43"/>
-      <c r="X24" s="44"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="47"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="46"/>
+      <c r="M24" s="46"/>
+      <c r="N24" s="46"/>
+      <c r="O24" s="46"/>
+      <c r="P24" s="47"/>
+      <c r="S24" s="48"/>
+      <c r="T24" s="46"/>
+      <c r="U24" s="46"/>
+      <c r="V24" s="46"/>
+      <c r="W24" s="46"/>
+      <c r="X24" s="47"/>
     </row>
     <row r="25" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C25" s="42">
+      <c r="C25" s="45">
         <f>COUNTIF('Flujo de Compra'!G:G,"Si")+COUNTIF('Gestión de Usuario'!G:G,"Si")+COUNTIF(Perfil!G:G,"Si")+COUNTIF(Credenciales!G:G,"Si")+COUNTIF(Videollamadas!G:G,"Si")+COUNTIF(Reintegros!G:G,"Si")+COUNTIF(Misceláneas!G:G,"Si")+COUNTIF('Control de Acceso'!G:G,"Si")+COUNTIF('Sistema Caído'!G:G,"Si")+COUNTIF('Funcionalidades Pendientes'!G:G,"Si")</f>
-        <v>172</v>
-      </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
-      <c r="K25" s="42">
+        <v>173</v>
+      </c>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
+      <c r="K25" s="45">
         <f>COUNTIFS('Flujo de Compra'!G:G,"Si",'Flujo de Compra'!H:H,"Si")+COUNTIFS('Gestión de Usuario'!G:G,"Si",'Gestión de Usuario'!H:H,"Si")+COUNTIFS(Perfil!G:G,"Si",Perfil!H:H,"Si")+COUNTIFS(Credenciales!G:G,"Si",Credenciales!H:H,"Si")+COUNTIFS(Videollamadas!G:G,"Si",Videollamadas!H:H,"Si")+COUNTIFS(Reintegros!G:G,"Si",Reintegros!H:H,"Si")+COUNTIFS(Misceláneas!G:G,"Si",Misceláneas!H:H,"Si")+COUNTIFS('Control de Acceso'!G:G,"Si",'Control de Acceso'!H:H,"Si")+COUNTIFS('Sistema Caído'!G:G,"Si",'Sistema Caído'!H:H,"Si")+COUNTIFS('Funcionalidades Pendientes'!G:G,"Si",'Funcionalidades Pendientes'!H:H,"Si")</f>
-        <v>138</v>
-      </c>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
-      <c r="N25" s="43"/>
-      <c r="O25" s="43"/>
-      <c r="P25" s="44"/>
-      <c r="S25" s="53">
+        <v>139</v>
+      </c>
+      <c r="L25" s="46"/>
+      <c r="M25" s="46"/>
+      <c r="N25" s="46"/>
+      <c r="O25" s="46"/>
+      <c r="P25" s="47"/>
+      <c r="S25" s="56">
         <f>K25/C25</f>
-        <v>0.80232558139534882</v>
-      </c>
-      <c r="T25" s="43"/>
-      <c r="U25" s="43"/>
-      <c r="V25" s="43"/>
-      <c r="W25" s="43"/>
-      <c r="X25" s="44"/>
+        <v>0.80346820809248554</v>
+      </c>
+      <c r="T25" s="46"/>
+      <c r="U25" s="46"/>
+      <c r="V25" s="46"/>
+      <c r="W25" s="46"/>
+      <c r="X25" s="47"/>
     </row>
     <row r="26" spans="3:24">
-      <c r="C26" s="45"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
-      <c r="H26" s="44"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
-      <c r="N26" s="43"/>
-      <c r="O26" s="43"/>
-      <c r="P26" s="44"/>
-      <c r="S26" s="45"/>
-      <c r="T26" s="43"/>
-      <c r="U26" s="43"/>
-      <c r="V26" s="43"/>
-      <c r="W26" s="43"/>
-      <c r="X26" s="44"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="46"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="46"/>
+      <c r="M26" s="46"/>
+      <c r="N26" s="46"/>
+      <c r="O26" s="46"/>
+      <c r="P26" s="47"/>
+      <c r="S26" s="48"/>
+      <c r="T26" s="46"/>
+      <c r="U26" s="46"/>
+      <c r="V26" s="46"/>
+      <c r="W26" s="46"/>
+      <c r="X26" s="47"/>
     </row>
     <row r="27" spans="3:24">
-      <c r="C27" s="45"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="44"/>
-      <c r="S27" s="45"/>
-      <c r="T27" s="43"/>
-      <c r="U27" s="43"/>
-      <c r="V27" s="43"/>
-      <c r="W27" s="43"/>
-      <c r="X27" s="44"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="46"/>
+      <c r="N27" s="46"/>
+      <c r="O27" s="46"/>
+      <c r="P27" s="47"/>
+      <c r="S27" s="48"/>
+      <c r="T27" s="46"/>
+      <c r="U27" s="46"/>
+      <c r="V27" s="46"/>
+      <c r="W27" s="46"/>
+      <c r="X27" s="47"/>
     </row>
     <row r="28" spans="3:24">
-      <c r="C28" s="45"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="43"/>
-      <c r="H28" s="44"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
-      <c r="N28" s="43"/>
-      <c r="O28" s="43"/>
-      <c r="P28" s="44"/>
-      <c r="S28" s="45"/>
-      <c r="T28" s="43"/>
-      <c r="U28" s="43"/>
-      <c r="V28" s="43"/>
-      <c r="W28" s="43"/>
-      <c r="X28" s="44"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="47"/>
+      <c r="K28" s="48"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="46"/>
+      <c r="N28" s="46"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
+      <c r="S28" s="48"/>
+      <c r="T28" s="46"/>
+      <c r="U28" s="46"/>
+      <c r="V28" s="46"/>
+      <c r="W28" s="46"/>
+      <c r="X28" s="47"/>
     </row>
     <row r="29" spans="3:24">
-      <c r="C29" s="45"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="43"/>
-      <c r="H29" s="44"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="43"/>
-      <c r="M29" s="43"/>
-      <c r="N29" s="43"/>
-      <c r="O29" s="43"/>
-      <c r="P29" s="44"/>
-      <c r="S29" s="45"/>
-      <c r="T29" s="43"/>
-      <c r="U29" s="43"/>
-      <c r="V29" s="43"/>
-      <c r="W29" s="43"/>
-      <c r="X29" s="44"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="47"/>
+      <c r="K29" s="48"/>
+      <c r="L29" s="46"/>
+      <c r="M29" s="46"/>
+      <c r="N29" s="46"/>
+      <c r="O29" s="46"/>
+      <c r="P29" s="47"/>
+      <c r="S29" s="48"/>
+      <c r="T29" s="46"/>
+      <c r="U29" s="46"/>
+      <c r="V29" s="46"/>
+      <c r="W29" s="46"/>
+      <c r="X29" s="47"/>
     </row>
     <row r="30" spans="3:24">
-      <c r="C30" s="45"/>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="44"/>
-      <c r="K30" s="45"/>
-      <c r="L30" s="43"/>
-      <c r="M30" s="43"/>
-      <c r="N30" s="43"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="44"/>
-      <c r="S30" s="45"/>
-      <c r="T30" s="43"/>
-      <c r="U30" s="43"/>
-      <c r="V30" s="43"/>
-      <c r="W30" s="43"/>
-      <c r="X30" s="44"/>
+      <c r="C30" s="48"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="47"/>
+      <c r="K30" s="48"/>
+      <c r="L30" s="46"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
+      <c r="O30" s="46"/>
+      <c r="P30" s="47"/>
+      <c r="S30" s="48"/>
+      <c r="T30" s="46"/>
+      <c r="U30" s="46"/>
+      <c r="V30" s="46"/>
+      <c r="W30" s="46"/>
+      <c r="X30" s="47"/>
     </row>
     <row r="31" spans="3:24">
-      <c r="C31" s="45"/>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="44"/>
-      <c r="K31" s="45"/>
-      <c r="L31" s="43"/>
-      <c r="M31" s="43"/>
-      <c r="N31" s="43"/>
-      <c r="O31" s="43"/>
-      <c r="P31" s="44"/>
-      <c r="S31" s="45"/>
-      <c r="T31" s="43"/>
-      <c r="U31" s="43"/>
-      <c r="V31" s="43"/>
-      <c r="W31" s="43"/>
-      <c r="X31" s="44"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="46"/>
+      <c r="H31" s="47"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="46"/>
+      <c r="M31" s="46"/>
+      <c r="N31" s="46"/>
+      <c r="O31" s="46"/>
+      <c r="P31" s="47"/>
+      <c r="S31" s="48"/>
+      <c r="T31" s="46"/>
+      <c r="U31" s="46"/>
+      <c r="V31" s="46"/>
+      <c r="W31" s="46"/>
+      <c r="X31" s="47"/>
     </row>
     <row r="32" spans="3:24">
-      <c r="C32" s="45"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="44"/>
-      <c r="K32" s="45"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="43"/>
-      <c r="N32" s="43"/>
-      <c r="O32" s="43"/>
-      <c r="P32" s="44"/>
-      <c r="S32" s="45"/>
-      <c r="T32" s="43"/>
-      <c r="U32" s="43"/>
-      <c r="V32" s="43"/>
-      <c r="W32" s="43"/>
-      <c r="X32" s="44"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="46"/>
+      <c r="H32" s="47"/>
+      <c r="K32" s="48"/>
+      <c r="L32" s="46"/>
+      <c r="M32" s="46"/>
+      <c r="N32" s="46"/>
+      <c r="O32" s="46"/>
+      <c r="P32" s="47"/>
+      <c r="S32" s="48"/>
+      <c r="T32" s="46"/>
+      <c r="U32" s="46"/>
+      <c r="V32" s="46"/>
+      <c r="W32" s="46"/>
+      <c r="X32" s="47"/>
     </row>
     <row r="33" spans="3:24">
-      <c r="C33" s="45"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="44"/>
-      <c r="K33" s="45"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="43"/>
-      <c r="P33" s="44"/>
-      <c r="S33" s="45"/>
-      <c r="T33" s="43"/>
-      <c r="U33" s="43"/>
-      <c r="V33" s="43"/>
-      <c r="W33" s="43"/>
-      <c r="X33" s="44"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="46"/>
+      <c r="G33" s="46"/>
+      <c r="H33" s="47"/>
+      <c r="K33" s="48"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="47"/>
+      <c r="S33" s="48"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+      <c r="V33" s="46"/>
+      <c r="W33" s="46"/>
+      <c r="X33" s="47"/>
     </row>
     <row r="34" spans="3:24">
-      <c r="C34" s="45"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="44"/>
-      <c r="K34" s="45"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
-      <c r="P34" s="44"/>
-      <c r="S34" s="45"/>
-      <c r="T34" s="43"/>
-      <c r="U34" s="43"/>
-      <c r="V34" s="43"/>
-      <c r="W34" s="43"/>
-      <c r="X34" s="44"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="46"/>
+      <c r="E34" s="46"/>
+      <c r="F34" s="46"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="47"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="46"/>
+      <c r="M34" s="46"/>
+      <c r="N34" s="46"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="47"/>
+      <c r="S34" s="48"/>
+      <c r="T34" s="46"/>
+      <c r="U34" s="46"/>
+      <c r="V34" s="46"/>
+      <c r="W34" s="46"/>
+      <c r="X34" s="47"/>
     </row>
     <row r="35" spans="3:24">
-      <c r="C35" s="45"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="44"/>
-      <c r="K35" s="45"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
-      <c r="P35" s="44"/>
-      <c r="S35" s="45"/>
-      <c r="T35" s="43"/>
-      <c r="U35" s="43"/>
-      <c r="V35" s="43"/>
-      <c r="W35" s="43"/>
-      <c r="X35" s="44"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="46"/>
+      <c r="E35" s="46"/>
+      <c r="F35" s="46"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="47"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="46"/>
+      <c r="M35" s="46"/>
+      <c r="N35" s="46"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="47"/>
+      <c r="S35" s="48"/>
+      <c r="T35" s="46"/>
+      <c r="U35" s="46"/>
+      <c r="V35" s="46"/>
+      <c r="W35" s="46"/>
+      <c r="X35" s="47"/>
     </row>
     <row r="36" spans="3:24">
-      <c r="C36" s="45"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="44"/>
-      <c r="K36" s="45"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="44"/>
-      <c r="S36" s="45"/>
-      <c r="T36" s="43"/>
-      <c r="U36" s="43"/>
-      <c r="V36" s="43"/>
-      <c r="W36" s="43"/>
-      <c r="X36" s="44"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="46"/>
+      <c r="E36" s="46"/>
+      <c r="F36" s="46"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="47"/>
+      <c r="K36" s="48"/>
+      <c r="L36" s="46"/>
+      <c r="M36" s="46"/>
+      <c r="N36" s="46"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="47"/>
+      <c r="S36" s="48"/>
+      <c r="T36" s="46"/>
+      <c r="U36" s="46"/>
+      <c r="V36" s="46"/>
+      <c r="W36" s="46"/>
+      <c r="X36" s="47"/>
     </row>
     <row r="37" spans="3:24">
-      <c r="C37" s="45"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="44"/>
-      <c r="K37" s="45"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
-      <c r="P37" s="44"/>
-      <c r="S37" s="45"/>
-      <c r="T37" s="43"/>
-      <c r="U37" s="43"/>
-      <c r="V37" s="43"/>
-      <c r="W37" s="43"/>
-      <c r="X37" s="44"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="46"/>
+      <c r="E37" s="46"/>
+      <c r="F37" s="46"/>
+      <c r="G37" s="46"/>
+      <c r="H37" s="47"/>
+      <c r="K37" s="48"/>
+      <c r="L37" s="46"/>
+      <c r="M37" s="46"/>
+      <c r="N37" s="46"/>
+      <c r="O37" s="46"/>
+      <c r="P37" s="47"/>
+      <c r="S37" s="48"/>
+      <c r="T37" s="46"/>
+      <c r="U37" s="46"/>
+      <c r="V37" s="46"/>
+      <c r="W37" s="46"/>
+      <c r="X37" s="47"/>
     </row>
     <row r="38" spans="3:24">
-      <c r="C38" s="45"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="43"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="43"/>
-      <c r="H38" s="44"/>
-      <c r="K38" s="45"/>
-      <c r="L38" s="43"/>
-      <c r="M38" s="43"/>
-      <c r="N38" s="43"/>
-      <c r="O38" s="43"/>
-      <c r="P38" s="44"/>
-      <c r="S38" s="45"/>
-      <c r="T38" s="43"/>
-      <c r="U38" s="43"/>
-      <c r="V38" s="43"/>
-      <c r="W38" s="43"/>
-      <c r="X38" s="44"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="46"/>
+      <c r="E38" s="46"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="47"/>
+      <c r="K38" s="48"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="47"/>
+      <c r="S38" s="48"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="47"/>
     </row>
     <row r="39" spans="3:24" ht="15.75" customHeight="1">
-      <c r="C39" s="46"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="48"/>
-      <c r="K39" s="46"/>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="47"/>
-      <c r="O39" s="47"/>
-      <c r="P39" s="48"/>
-      <c r="S39" s="46"/>
-      <c r="T39" s="47"/>
-      <c r="U39" s="47"/>
-      <c r="V39" s="47"/>
-      <c r="W39" s="47"/>
-      <c r="X39" s="48"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="50"/>
+      <c r="H39" s="51"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="51"/>
+      <c r="S39" s="49"/>
+      <c r="T39" s="50"/>
+      <c r="U39" s="50"/>
+      <c r="V39" s="50"/>
+      <c r="W39" s="50"/>
+      <c r="X39" s="51"/>
     </row>
     <row r="41" spans="3:24" ht="15.75" customHeight="1"/>
     <row r="42" spans="3:24">
-      <c r="C42" s="49" t="s">
+      <c r="C42" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="50"/>
-      <c r="H42" s="51"/>
+      <c r="D42" s="53"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="53"/>
+      <c r="G42" s="53"/>
+      <c r="H42" s="54"/>
     </row>
     <row r="43" spans="3:24">
-      <c r="C43" s="45"/>
-      <c r="D43" s="43"/>
-      <c r="E43" s="43"/>
-      <c r="F43" s="43"/>
-      <c r="G43" s="43"/>
-      <c r="H43" s="44"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="47"/>
       <c r="K43" s="28"/>
       <c r="L43" s="28"/>
       <c r="M43" s="28"/>
@@ -5871,31 +5886,31 @@
       <c r="P43" s="28"/>
     </row>
     <row r="44" spans="3:24" ht="21" customHeight="1">
-      <c r="C44" s="53">
+      <c r="C44" s="56">
         <f>C25/C5</f>
-        <v>0.55844155844155841</v>
-      </c>
-      <c r="D44" s="43"/>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="44"/>
+        <v>0.55987055016181231</v>
+      </c>
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="47"/>
       <c r="K44" s="28"/>
-      <c r="L44" s="52" t="s">
+      <c r="L44" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="M44" s="43"/>
-      <c r="N44" s="43"/>
-      <c r="O44" s="43"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
+      <c r="O44" s="46"/>
       <c r="P44" s="29"/>
     </row>
     <row r="45" spans="3:24">
-      <c r="C45" s="45"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="44"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="46"/>
+      <c r="E45" s="46"/>
+      <c r="F45" s="46"/>
+      <c r="G45" s="46"/>
+      <c r="H45" s="47"/>
       <c r="K45" s="28"/>
       <c r="L45" s="30"/>
       <c r="M45" s="30"/>
@@ -5904,12 +5919,12 @@
       <c r="P45" s="29"/>
     </row>
     <row r="46" spans="3:24">
-      <c r="C46" s="45"/>
-      <c r="D46" s="43"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="44"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="46"/>
+      <c r="E46" s="46"/>
+      <c r="F46" s="46"/>
+      <c r="G46" s="46"/>
+      <c r="H46" s="47"/>
       <c r="K46" s="28"/>
       <c r="L46" s="31"/>
       <c r="M46" s="28" t="s">
@@ -5920,12 +5935,12 @@
       <c r="P46" s="28"/>
     </row>
     <row r="47" spans="3:24">
-      <c r="C47" s="45"/>
-      <c r="D47" s="43"/>
-      <c r="E47" s="43"/>
-      <c r="F47" s="43"/>
-      <c r="G47" s="43"/>
-      <c r="H47" s="44"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="46"/>
+      <c r="F47" s="46"/>
+      <c r="G47" s="46"/>
+      <c r="H47" s="47"/>
       <c r="K47" s="28"/>
       <c r="L47" s="32"/>
       <c r="M47" s="28" t="s">
@@ -5936,12 +5951,12 @@
       <c r="P47" s="28"/>
     </row>
     <row r="48" spans="3:24">
-      <c r="C48" s="45"/>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="44"/>
+      <c r="C48" s="48"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="46"/>
+      <c r="F48" s="46"/>
+      <c r="G48" s="46"/>
+      <c r="H48" s="47"/>
       <c r="K48" s="28"/>
       <c r="L48" s="33"/>
       <c r="M48" s="28" t="s">
@@ -5952,12 +5967,12 @@
       <c r="P48" s="28"/>
     </row>
     <row r="49" spans="3:16">
-      <c r="C49" s="45"/>
-      <c r="D49" s="43"/>
-      <c r="E49" s="43"/>
-      <c r="F49" s="43"/>
-      <c r="G49" s="43"/>
-      <c r="H49" s="44"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="46"/>
+      <c r="F49" s="46"/>
+      <c r="G49" s="46"/>
+      <c r="H49" s="47"/>
       <c r="K49" s="28"/>
       <c r="L49" s="34"/>
       <c r="M49" s="28" t="s">
@@ -5968,12 +5983,12 @@
       <c r="P49" s="28"/>
     </row>
     <row r="50" spans="3:16">
-      <c r="C50" s="45"/>
-      <c r="D50" s="43"/>
-      <c r="E50" s="43"/>
-      <c r="F50" s="43"/>
-      <c r="G50" s="43"/>
-      <c r="H50" s="44"/>
+      <c r="C50" s="48"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="46"/>
+      <c r="F50" s="46"/>
+      <c r="G50" s="46"/>
+      <c r="H50" s="47"/>
       <c r="K50" s="28"/>
       <c r="L50" s="35"/>
       <c r="M50" s="28" t="s">
@@ -5984,12 +5999,12 @@
       <c r="P50" s="28"/>
     </row>
     <row r="51" spans="3:16">
-      <c r="C51" s="45"/>
-      <c r="D51" s="43"/>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="43"/>
-      <c r="H51" s="44"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
+      <c r="F51" s="46"/>
+      <c r="G51" s="46"/>
+      <c r="H51" s="47"/>
       <c r="K51" s="28"/>
       <c r="L51" s="28"/>
       <c r="M51" s="28"/>
@@ -5998,230 +6013,230 @@
       <c r="P51" s="28"/>
     </row>
     <row r="52" spans="3:16">
-      <c r="C52" s="45"/>
-      <c r="D52" s="43"/>
-      <c r="E52" s="43"/>
-      <c r="F52" s="43"/>
-      <c r="G52" s="43"/>
-      <c r="H52" s="44"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="46"/>
+      <c r="F52" s="46"/>
+      <c r="G52" s="46"/>
+      <c r="H52" s="47"/>
     </row>
     <row r="53" spans="3:16">
-      <c r="C53" s="45"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="44"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="46"/>
+      <c r="E53" s="46"/>
+      <c r="F53" s="46"/>
+      <c r="G53" s="46"/>
+      <c r="H53" s="47"/>
     </row>
     <row r="54" spans="3:16">
-      <c r="C54" s="45"/>
-      <c r="D54" s="43"/>
-      <c r="E54" s="43"/>
-      <c r="F54" s="43"/>
-      <c r="G54" s="43"/>
-      <c r="H54" s="44"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="46"/>
+      <c r="E54" s="46"/>
+      <c r="F54" s="46"/>
+      <c r="G54" s="46"/>
+      <c r="H54" s="47"/>
     </row>
     <row r="55" spans="3:16">
-      <c r="C55" s="45"/>
-      <c r="D55" s="43"/>
-      <c r="E55" s="43"/>
-      <c r="F55" s="43"/>
-      <c r="G55" s="43"/>
-      <c r="H55" s="44"/>
+      <c r="C55" s="48"/>
+      <c r="D55" s="46"/>
+      <c r="E55" s="46"/>
+      <c r="F55" s="46"/>
+      <c r="G55" s="46"/>
+      <c r="H55" s="47"/>
     </row>
     <row r="56" spans="3:16">
-      <c r="C56" s="45"/>
-      <c r="D56" s="43"/>
-      <c r="E56" s="43"/>
-      <c r="F56" s="43"/>
-      <c r="G56" s="43"/>
-      <c r="H56" s="44"/>
+      <c r="C56" s="48"/>
+      <c r="D56" s="46"/>
+      <c r="E56" s="46"/>
+      <c r="F56" s="46"/>
+      <c r="G56" s="46"/>
+      <c r="H56" s="47"/>
     </row>
     <row r="57" spans="3:16">
-      <c r="C57" s="45"/>
-      <c r="D57" s="43"/>
-      <c r="E57" s="43"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="44"/>
+      <c r="C57" s="48"/>
+      <c r="D57" s="46"/>
+      <c r="E57" s="46"/>
+      <c r="F57" s="46"/>
+      <c r="G57" s="46"/>
+      <c r="H57" s="47"/>
     </row>
     <row r="58" spans="3:16" ht="15.75" customHeight="1">
-      <c r="C58" s="46"/>
-      <c r="D58" s="47"/>
-      <c r="E58" s="47"/>
-      <c r="F58" s="47"/>
-      <c r="G58" s="47"/>
-      <c r="H58" s="48"/>
+      <c r="C58" s="49"/>
+      <c r="D58" s="50"/>
+      <c r="E58" s="50"/>
+      <c r="F58" s="50"/>
+      <c r="G58" s="50"/>
+      <c r="H58" s="51"/>
     </row>
     <row r="62" spans="3:16">
-      <c r="C62" s="54" t="s">
+      <c r="C62" s="42" t="s">
         <v>585</v>
       </c>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54"/>
-      <c r="F62" s="54"/>
-      <c r="H62" s="54" t="s">
+      <c r="D62" s="42"/>
+      <c r="E62" s="42"/>
+      <c r="F62" s="42"/>
+      <c r="H62" s="42" t="s">
         <v>586</v>
       </c>
-      <c r="I62" s="54"/>
-      <c r="J62" s="54"/>
-      <c r="K62" s="54"/>
-      <c r="M62" s="54" t="s">
+      <c r="I62" s="42"/>
+      <c r="J62" s="42"/>
+      <c r="K62" s="42"/>
+      <c r="M62" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N62" s="54"/>
-      <c r="O62" s="54"/>
-      <c r="P62" s="54"/>
+      <c r="N62" s="42"/>
+      <c r="O62" s="42"/>
+      <c r="P62" s="42"/>
     </row>
     <row r="63" spans="3:16">
-      <c r="C63" s="54"/>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54"/>
-      <c r="F63" s="54"/>
-      <c r="H63" s="54"/>
-      <c r="I63" s="54"/>
-      <c r="J63" s="54"/>
-      <c r="K63" s="54"/>
-      <c r="M63" s="54"/>
-      <c r="N63" s="54"/>
-      <c r="O63" s="54"/>
-      <c r="P63" s="54"/>
+      <c r="C63" s="42"/>
+      <c r="D63" s="42"/>
+      <c r="E63" s="42"/>
+      <c r="F63" s="42"/>
+      <c r="H63" s="42"/>
+      <c r="I63" s="42"/>
+      <c r="J63" s="42"/>
+      <c r="K63" s="42"/>
+      <c r="M63" s="42"/>
+      <c r="N63" s="42"/>
+      <c r="O63" s="42"/>
+      <c r="P63" s="42"/>
     </row>
     <row r="64" spans="3:16">
-      <c r="C64" s="55">
+      <c r="C64" s="43">
         <f>COUNTIF('Flujo de Compra'!I:I,"Si")+COUNTIF('Gestión de Usuario'!I:I,"Si")+COUNTIF(Perfil!J:J,"Si")+COUNTIF(Credenciales!J:J,"Si")+COUNTIF(Videollamadas!J:J,"Si")</f>
-        <v>252</v>
-      </c>
-      <c r="D64" s="55"/>
-      <c r="E64" s="55"/>
-      <c r="F64" s="55"/>
-      <c r="H64" s="55">
+        <v>253</v>
+      </c>
+      <c r="D64" s="43"/>
+      <c r="E64" s="43"/>
+      <c r="F64" s="43"/>
+      <c r="H64" s="43">
         <f>COUNTIF('Flujo de Compra'!H:H,"Si")+COUNTIF('Gestión de Usuario'!H:H,"Si")+COUNTIF(Perfil!H:H,"Si")+COUNTIF(Credenciales!H:H,"Si")+COUNTIF(Videollamadas!H:H,"Si")</f>
-        <v>195</v>
-      </c>
-      <c r="I64" s="55"/>
-      <c r="J64" s="55"/>
-      <c r="K64" s="55"/>
-      <c r="M64" s="56">
+        <v>196</v>
+      </c>
+      <c r="I64" s="43"/>
+      <c r="J64" s="43"/>
+      <c r="K64" s="43"/>
+      <c r="M64" s="44">
         <f t="shared" ref="M64" si="0">H64/C64</f>
-        <v>0.77380952380952384</v>
-      </c>
-      <c r="N64" s="56"/>
-      <c r="O64" s="56"/>
-      <c r="P64" s="56"/>
+        <v>0.77470355731225293</v>
+      </c>
+      <c r="N64" s="44"/>
+      <c r="O64" s="44"/>
+      <c r="P64" s="44"/>
     </row>
     <row r="65" spans="3:16">
-      <c r="C65" s="55"/>
-      <c r="D65" s="55"/>
-      <c r="E65" s="55"/>
-      <c r="F65" s="55"/>
-      <c r="H65" s="55"/>
-      <c r="I65" s="55"/>
-      <c r="J65" s="55"/>
-      <c r="K65" s="55"/>
-      <c r="M65" s="56"/>
-      <c r="N65" s="56"/>
-      <c r="O65" s="56"/>
-      <c r="P65" s="56"/>
+      <c r="C65" s="43"/>
+      <c r="D65" s="43"/>
+      <c r="E65" s="43"/>
+      <c r="F65" s="43"/>
+      <c r="H65" s="43"/>
+      <c r="I65" s="43"/>
+      <c r="J65" s="43"/>
+      <c r="K65" s="43"/>
+      <c r="M65" s="44"/>
+      <c r="N65" s="44"/>
+      <c r="O65" s="44"/>
+      <c r="P65" s="44"/>
     </row>
     <row r="66" spans="3:16">
-      <c r="C66" s="55"/>
-      <c r="D66" s="55"/>
-      <c r="E66" s="55"/>
-      <c r="F66" s="55"/>
-      <c r="H66" s="55"/>
-      <c r="I66" s="55"/>
-      <c r="J66" s="55"/>
-      <c r="K66" s="55"/>
-      <c r="M66" s="56"/>
-      <c r="N66" s="56"/>
-      <c r="O66" s="56"/>
-      <c r="P66" s="56"/>
+      <c r="C66" s="43"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="H66" s="43"/>
+      <c r="I66" s="43"/>
+      <c r="J66" s="43"/>
+      <c r="K66" s="43"/>
+      <c r="M66" s="44"/>
+      <c r="N66" s="44"/>
+      <c r="O66" s="44"/>
+      <c r="P66" s="44"/>
     </row>
     <row r="69" spans="3:16">
-      <c r="C69" s="54" t="s">
+      <c r="C69" s="42" t="s">
         <v>588</v>
       </c>
-      <c r="D69" s="54"/>
-      <c r="E69" s="54"/>
-      <c r="F69" s="54"/>
-      <c r="H69" s="54" t="s">
+      <c r="D69" s="42"/>
+      <c r="E69" s="42"/>
+      <c r="F69" s="42"/>
+      <c r="H69" s="42" t="s">
         <v>589</v>
       </c>
-      <c r="I69" s="54"/>
-      <c r="J69" s="54"/>
-      <c r="K69" s="54"/>
-      <c r="M69" s="54" t="s">
+      <c r="I69" s="42"/>
+      <c r="J69" s="42"/>
+      <c r="K69" s="42"/>
+      <c r="M69" s="42" t="s">
         <v>587</v>
       </c>
-      <c r="N69" s="54"/>
-      <c r="O69" s="54"/>
-      <c r="P69" s="54"/>
+      <c r="N69" s="42"/>
+      <c r="O69" s="42"/>
+      <c r="P69" s="42"/>
     </row>
     <row r="70" spans="3:16">
-      <c r="C70" s="54"/>
-      <c r="D70" s="54"/>
-      <c r="E70" s="54"/>
-      <c r="F70" s="54"/>
-      <c r="H70" s="54"/>
-      <c r="I70" s="54"/>
-      <c r="J70" s="54"/>
-      <c r="K70" s="54"/>
-      <c r="M70" s="54"/>
-      <c r="N70" s="54"/>
-      <c r="O70" s="54"/>
-      <c r="P70" s="54"/>
+      <c r="C70" s="42"/>
+      <c r="D70" s="42"/>
+      <c r="E70" s="42"/>
+      <c r="F70" s="42"/>
+      <c r="H70" s="42"/>
+      <c r="I70" s="42"/>
+      <c r="J70" s="42"/>
+      <c r="K70" s="42"/>
+      <c r="M70" s="42"/>
+      <c r="N70" s="42"/>
+      <c r="O70" s="42"/>
+      <c r="P70" s="42"/>
     </row>
     <row r="71" spans="3:16">
-      <c r="C71" s="55">
+      <c r="C71" s="43">
         <f>COUNTIF(Perfil!K:K,"Si")+COUNTIF(Credenciales!K:K,"Si")+COUNTIF(Videollamadas!K:K,"Si")</f>
-        <v>73</v>
-      </c>
-      <c r="D71" s="55"/>
-      <c r="E71" s="55"/>
-      <c r="F71" s="55"/>
-      <c r="H71" s="55">
+        <v>74</v>
+      </c>
+      <c r="D71" s="43"/>
+      <c r="E71" s="43"/>
+      <c r="F71" s="43"/>
+      <c r="H71" s="43">
         <f>COUNTIF(Perfil!I:I,"Si")+COUNTIF(Credenciales!I:I,"Si")+COUNTIF(Videollamadas!I:I,"Si")</f>
-        <v>60</v>
-      </c>
-      <c r="I71" s="55"/>
-      <c r="J71" s="55"/>
-      <c r="K71" s="55"/>
-      <c r="M71" s="56">
+        <v>61</v>
+      </c>
+      <c r="I71" s="43"/>
+      <c r="J71" s="43"/>
+      <c r="K71" s="43"/>
+      <c r="M71" s="44">
         <f t="shared" ref="M71" si="1">H71/C71</f>
-        <v>0.82191780821917804</v>
-      </c>
-      <c r="N71" s="56"/>
-      <c r="O71" s="56"/>
-      <c r="P71" s="56"/>
+        <v>0.82432432432432434</v>
+      </c>
+      <c r="N71" s="44"/>
+      <c r="O71" s="44"/>
+      <c r="P71" s="44"/>
     </row>
     <row r="72" spans="3:16">
-      <c r="C72" s="55"/>
-      <c r="D72" s="55"/>
-      <c r="E72" s="55"/>
-      <c r="F72" s="55"/>
-      <c r="H72" s="55"/>
-      <c r="I72" s="55"/>
-      <c r="J72" s="55"/>
-      <c r="K72" s="55"/>
-      <c r="M72" s="56"/>
-      <c r="N72" s="56"/>
-      <c r="O72" s="56"/>
-      <c r="P72" s="56"/>
+      <c r="C72" s="43"/>
+      <c r="D72" s="43"/>
+      <c r="E72" s="43"/>
+      <c r="F72" s="43"/>
+      <c r="H72" s="43"/>
+      <c r="I72" s="43"/>
+      <c r="J72" s="43"/>
+      <c r="K72" s="43"/>
+      <c r="M72" s="44"/>
+      <c r="N72" s="44"/>
+      <c r="O72" s="44"/>
+      <c r="P72" s="44"/>
     </row>
     <row r="73" spans="3:16">
-      <c r="C73" s="55"/>
-      <c r="D73" s="55"/>
-      <c r="E73" s="55"/>
-      <c r="F73" s="55"/>
-      <c r="H73" s="55"/>
-      <c r="I73" s="55"/>
-      <c r="J73" s="55"/>
-      <c r="K73" s="55"/>
-      <c r="M73" s="56"/>
-      <c r="N73" s="56"/>
-      <c r="O73" s="56"/>
-      <c r="P73" s="56"/>
+      <c r="C73" s="43"/>
+      <c r="D73" s="43"/>
+      <c r="E73" s="43"/>
+      <c r="F73" s="43"/>
+      <c r="H73" s="43"/>
+      <c r="I73" s="43"/>
+      <c r="J73" s="43"/>
+      <c r="K73" s="43"/>
+      <c r="M73" s="44"/>
+      <c r="N73" s="44"/>
+      <c r="O73" s="44"/>
+      <c r="P73" s="44"/>
     </row>
     <row r="76" spans="3:16">
       <c r="C76" s="36" t="s">
@@ -6230,18 +6245,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C69:F70"/>
-    <mergeCell ref="C71:F73"/>
-    <mergeCell ref="H69:K70"/>
-    <mergeCell ref="H71:K73"/>
-    <mergeCell ref="M69:P70"/>
-    <mergeCell ref="M71:P73"/>
-    <mergeCell ref="C62:F63"/>
-    <mergeCell ref="C64:F66"/>
-    <mergeCell ref="H62:K63"/>
-    <mergeCell ref="H64:K66"/>
-    <mergeCell ref="M62:P63"/>
-    <mergeCell ref="M64:P66"/>
     <mergeCell ref="K5:P19"/>
     <mergeCell ref="K25:P39"/>
     <mergeCell ref="S3:X4"/>
@@ -6257,6 +6260,18 @@
     <mergeCell ref="C3:H4"/>
     <mergeCell ref="C25:H39"/>
     <mergeCell ref="K23:P24"/>
+    <mergeCell ref="C62:F63"/>
+    <mergeCell ref="C64:F66"/>
+    <mergeCell ref="H62:K63"/>
+    <mergeCell ref="H64:K66"/>
+    <mergeCell ref="M62:P63"/>
+    <mergeCell ref="M64:P66"/>
+    <mergeCell ref="C69:F70"/>
+    <mergeCell ref="C71:F73"/>
+    <mergeCell ref="H69:K70"/>
+    <mergeCell ref="H71:K73"/>
+    <mergeCell ref="M69:P70"/>
+    <mergeCell ref="M71:P73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -7227,7 +7242,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -7236,7 +7251,7 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
       <c r="I2" s="12" t="s">
         <v>27</v>
       </c>
@@ -7245,7 +7260,7 @@
       <c r="A3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>22</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -7473,7 +7488,7 @@
       <c r="A12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="60" t="s">
+      <c r="B12" s="57" t="s">
         <v>51</v>
       </c>
       <c r="C12" s="22" t="s">
@@ -7539,7 +7554,7 @@
       <c r="A15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="59" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="18" t="s">
@@ -7632,7 +7647,7 @@
       <c r="A19" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="57" t="s">
         <v>69</v>
       </c>
       <c r="C19" s="22" t="s">
@@ -7833,7 +7848,7 @@
       <c r="A27" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="61" t="s">
+      <c r="B27" s="59" t="s">
         <v>90</v>
       </c>
       <c r="C27" s="18" t="s">
@@ -7953,7 +7968,7 @@
       <c r="A32" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="60" t="s">
+      <c r="B32" s="57" t="s">
         <v>104</v>
       </c>
       <c r="C32" s="22" t="s">
@@ -8100,7 +8115,7 @@
       <c r="A38" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="61" t="s">
+      <c r="B38" s="59" t="s">
         <v>120</v>
       </c>
       <c r="C38" s="18" t="s">
@@ -8153,7 +8168,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A40" s="57" t="s">
+      <c r="A40" s="60" t="s">
         <v>127</v>
       </c>
       <c r="B40" s="58"/>
@@ -8162,7 +8177,7 @@
       <c r="E40" s="58"/>
       <c r="F40" s="58"/>
       <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
+      <c r="H40" s="61"/>
       <c r="I40" s="12" t="s">
         <v>27</v>
       </c>
@@ -8171,7 +8186,7 @@
       <c r="A41" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="60" t="s">
+      <c r="B41" s="57" t="s">
         <v>22</v>
       </c>
       <c r="C41" s="22" t="s">
@@ -8399,7 +8414,7 @@
       <c r="A50" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B50" s="61" t="s">
+      <c r="B50" s="59" t="s">
         <v>51</v>
       </c>
       <c r="C50" s="18" t="s">
@@ -8465,7 +8480,7 @@
       <c r="A53" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="60" t="s">
+      <c r="B53" s="57" t="s">
         <v>58</v>
       </c>
       <c r="C53" s="22" t="s">
@@ -8558,7 +8573,7 @@
       <c r="A57" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="61" t="s">
+      <c r="B57" s="59" t="s">
         <v>69</v>
       </c>
       <c r="C57" s="18" t="s">
@@ -8759,7 +8774,7 @@
       <c r="A65" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B65" s="60" t="s">
+      <c r="B65" s="57" t="s">
         <v>90</v>
       </c>
       <c r="C65" s="22" t="s">
@@ -8879,7 +8894,7 @@
       <c r="A70" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B70" s="61" t="s">
+      <c r="B70" s="59" t="s">
         <v>104</v>
       </c>
       <c r="C70" s="18" t="s">
@@ -9026,7 +9041,7 @@
       <c r="A76" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B76" s="60" t="s">
+      <c r="B76" s="57" t="s">
         <v>120</v>
       </c>
       <c r="C76" s="22" t="s">
@@ -9079,7 +9094,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A78" s="57" t="s">
+      <c r="A78" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B78" s="58"/>
@@ -9088,7 +9103,7 @@
       <c r="E78" s="58"/>
       <c r="F78" s="58"/>
       <c r="G78" s="58"/>
-      <c r="H78" s="59"/>
+      <c r="H78" s="61"/>
       <c r="I78" s="12" t="s">
         <v>27</v>
       </c>
@@ -9097,7 +9112,7 @@
       <c r="A79" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B79" s="61" t="s">
+      <c r="B79" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C79" s="18" t="s">
@@ -9188,7 +9203,7 @@
       <c r="A83" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B83" s="60" t="s">
+      <c r="B83" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C83" s="22" t="s">
@@ -9237,7 +9252,7 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A85" s="57" t="s">
+      <c r="A85" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B85" s="58"/>
@@ -9246,7 +9261,7 @@
       <c r="E85" s="58"/>
       <c r="F85" s="58"/>
       <c r="G85" s="58"/>
-      <c r="H85" s="59"/>
+      <c r="H85" s="61"/>
       <c r="I85" s="12" t="s">
         <v>27</v>
       </c>
@@ -9255,7 +9270,7 @@
       <c r="A86" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B86" s="61" t="s">
+      <c r="B86" s="59" t="s">
         <v>141</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -9346,7 +9361,7 @@
       <c r="A90" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B90" s="60" t="s">
+      <c r="B90" s="57" t="s">
         <v>153</v>
       </c>
       <c r="C90" s="22" t="s">
@@ -9406,12 +9421,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B90:B91"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B86:B88"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A85:H85"/>
     <mergeCell ref="B32:B36"/>
@@ -9428,6 +9437,12 @@
     <mergeCell ref="B53:B55"/>
     <mergeCell ref="B19:B25"/>
     <mergeCell ref="B57:B63"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B90:B91"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B86:B88"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="153" priority="564" operator="equal">
@@ -9657,7 +9672,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="58"/>
@@ -9666,13 +9681,13 @@
       <c r="E2" s="58"/>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="H2" s="61"/>
     </row>
     <row r="3" spans="1:9" ht="76.5" customHeight="1">
       <c r="A3" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -9813,7 +9828,7 @@
       <c r="A9" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C9" s="22" t="s">
@@ -9931,7 +9946,7 @@
       <c r="A14" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -10078,7 +10093,7 @@
       <c r="A20" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -10222,7 +10237,7 @@
       <c r="A26" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -10311,7 +10326,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="60" t="s">
         <v>213</v>
       </c>
       <c r="B31" s="58"/>
@@ -10320,13 +10335,13 @@
       <c r="E31" s="58"/>
       <c r="F31" s="58"/>
       <c r="G31" s="58"/>
-      <c r="H31" s="59"/>
+      <c r="H31" s="61"/>
     </row>
     <row r="32" spans="1:9" ht="76.5" customHeight="1">
       <c r="A32" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B32" s="61" t="s">
+      <c r="B32" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C32" s="18" t="s">
@@ -10467,7 +10482,7 @@
       <c r="A38" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C38" s="22" t="s">
@@ -10585,7 +10600,7 @@
       <c r="A43" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B43" s="61" t="s">
+      <c r="B43" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C43" s="18" t="s">
@@ -10732,7 +10747,7 @@
       <c r="A49" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B49" s="59" t="s">
+      <c r="B49" s="61" t="s">
         <v>612</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -10876,7 +10891,7 @@
       <c r="A55" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="59" t="s">
+      <c r="B55" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C55" s="6" t="s">
@@ -10965,7 +10980,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A60" s="57" t="s">
+      <c r="A60" s="60" t="s">
         <v>140</v>
       </c>
       <c r="B60" s="58"/>
@@ -10974,13 +10989,13 @@
       <c r="E60" s="58"/>
       <c r="F60" s="58"/>
       <c r="G60" s="58"/>
-      <c r="H60" s="59"/>
+      <c r="H60" s="61"/>
     </row>
     <row r="61" spans="1:9" ht="76.5" customHeight="1">
       <c r="A61" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B61" s="61" t="s">
+      <c r="B61" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C61" s="18" t="s">
@@ -11121,7 +11136,7 @@
       <c r="A67" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B67" s="60" t="s">
+      <c r="B67" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C67" s="22" t="s">
@@ -11239,7 +11254,7 @@
       <c r="A72" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B72" s="61" t="s">
+      <c r="B72" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C72" s="18" t="s">
@@ -11386,7 +11401,7 @@
       <c r="A78" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B78" s="59" t="s">
+      <c r="B78" s="61" t="s">
         <v>611</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -11530,7 +11545,7 @@
       <c r="A84" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B84" s="59" t="s">
+      <c r="B84" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -11619,7 +11634,7 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="23.25" customHeight="1">
-      <c r="A89" s="57" t="s">
+      <c r="A89" s="60" t="s">
         <v>159</v>
       </c>
       <c r="B89" s="58"/>
@@ -11628,13 +11643,13 @@
       <c r="E89" s="58"/>
       <c r="F89" s="58"/>
       <c r="G89" s="58"/>
-      <c r="H89" s="59"/>
+      <c r="H89" s="61"/>
     </row>
     <row r="90" spans="1:9" ht="76.5" customHeight="1">
       <c r="A90" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="61" t="s">
+      <c r="B90" s="59" t="s">
         <v>162</v>
       </c>
       <c r="C90" s="18" t="s">
@@ -11775,7 +11790,7 @@
       <c r="A96" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="B96" s="60" t="s">
+      <c r="B96" s="57" t="s">
         <v>182</v>
       </c>
       <c r="C96" s="22" t="s">
@@ -11893,7 +11908,7 @@
       <c r="A101" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="B101" s="61" t="s">
+      <c r="B101" s="59" t="s">
         <v>192</v>
       </c>
       <c r="C101" s="18" t="s">
@@ -12040,7 +12055,7 @@
       <c r="A107" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B107" s="59" t="s">
+      <c r="B107" s="61" t="s">
         <v>591</v>
       </c>
       <c r="C107" s="6" t="s">
@@ -12184,7 +12199,7 @@
       <c r="A113" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B113" s="59" t="s">
+      <c r="B113" s="61" t="s">
         <v>208</v>
       </c>
       <c r="C113" s="6" t="s">
@@ -12274,6 +12289,14 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B113:B117"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B101:B105"/>
+    <mergeCell ref="B107:B108"/>
     <mergeCell ref="B9:B12"/>
     <mergeCell ref="B96:B99"/>
     <mergeCell ref="A2:H2"/>
@@ -12290,14 +12313,6 @@
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="B55:B59"/>
     <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B113:B117"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="B26:B30"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B101:B105"/>
-    <mergeCell ref="B107:B108"/>
   </mergeCells>
   <conditionalFormatting sqref="G1">
     <cfRule type="cellIs" dxfId="111" priority="525" operator="equal">
@@ -12703,7 +12718,7 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="59"/>
+      <c r="B2" s="61"/>
       <c r="C2" s="63"/>
       <c r="D2" s="58"/>
       <c r="E2" s="63"/>
@@ -12712,7 +12727,7 @@
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="198" customHeight="1">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="61" t="s">
         <v>216</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -12744,8 +12759,8 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="76.5" customHeight="1">
-      <c r="A4" s="59"/>
-      <c r="B4" s="59"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="63" t="s">
         <v>221</v>
       </c>
@@ -12776,7 +12791,7 @@
     </row>
     <row r="5" spans="1:11" ht="45.75" customHeight="1">
       <c r="A5" s="63"/>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="63"/>
       <c r="D5" s="58"/>
       <c r="E5" s="6" t="s">
@@ -12788,7 +12803,7 @@
       <c r="G5" s="12"/>
     </row>
     <row r="6" spans="1:11" ht="121.5" customHeight="1">
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="63" t="s">
         <v>226</v>
       </c>
@@ -12818,7 +12833,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="45.75" customHeight="1">
-      <c r="B7" s="59"/>
+      <c r="B7" s="61"/>
       <c r="C7" s="63"/>
       <c r="D7" s="58"/>
       <c r="E7" s="13" t="s">
@@ -12830,7 +12845,7 @@
       <c r="G7" s="12"/>
     </row>
     <row r="8" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B8" s="59"/>
+      <c r="B8" s="61"/>
       <c r="C8" s="13" t="s">
         <v>229</v>
       </c>
@@ -12846,7 +12861,7 @@
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:11" ht="30.75" customHeight="1">
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="13" t="s">
         <v>231</v>
       </c>
@@ -12862,7 +12877,7 @@
       <c r="G9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="91.5" customHeight="1">
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="13" t="s">
         <v>232</v>
       </c>
@@ -12892,7 +12907,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" ht="140.25" customHeight="1">
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="13" t="s">
         <v>235</v>
       </c>
@@ -12935,7 +12950,7 @@
       <c r="A13" s="62" t="s">
         <v>238</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="63"/>
       <c r="D13" s="58"/>
       <c r="E13" s="63"/>
@@ -13069,7 +13084,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="12" customWidth="1"/>
@@ -13134,7 +13149,7 @@
       <c r="A3" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>239</v>
       </c>
       <c r="C3" s="18" t="s">
@@ -13169,7 +13184,7 @@
       <c r="A4" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B4" s="61"/>
       <c r="C4" s="18" t="s">
         <v>244</v>
       </c>
@@ -13202,7 +13217,7 @@
       <c r="A5" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="B5" s="59"/>
+      <c r="B5" s="61"/>
       <c r="C5" s="18" t="s">
         <v>247</v>
       </c>
@@ -13235,7 +13250,7 @@
       <c r="A6" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="B6" s="59"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="18" t="s">
         <v>251</v>
       </c>
@@ -13278,7 +13293,7 @@
       <c r="A8" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="57" t="s">
         <v>254</v>
       </c>
       <c r="C8" s="22" t="s">
@@ -13313,7 +13328,7 @@
       <c r="A9" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="59"/>
+      <c r="B9" s="61"/>
       <c r="C9" s="22" t="s">
         <v>259</v>
       </c>
@@ -13346,7 +13361,7 @@
       <c r="A10" s="10" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="59"/>
+      <c r="B10" s="61"/>
       <c r="C10" s="64" t="s">
         <v>262</v>
       </c>
@@ -13359,7 +13374,7 @@
       <c r="F10" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G10" s="59" t="s">
+      <c r="G10" s="61" t="s">
         <v>28</v>
       </c>
       <c r="H10" s="12" t="s">
@@ -13379,7 +13394,7 @@
       <c r="A11" s="10" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="59"/>
+      <c r="B11" s="61"/>
       <c r="C11" s="58"/>
       <c r="D11" s="63"/>
       <c r="E11" s="11" t="s">
@@ -13388,7 +13403,7 @@
       <c r="F11" s="11" t="s">
         <v>265</v>
       </c>
-      <c r="G11" s="59"/>
+      <c r="G11" s="61"/>
       <c r="H11" s="12" t="s">
         <v>27</v>
       </c>
@@ -13406,7 +13421,7 @@
       <c r="A12" s="10" t="s">
         <v>179</v>
       </c>
-      <c r="B12" s="59"/>
+      <c r="B12" s="61"/>
       <c r="C12" s="22" t="s">
         <v>267</v>
       </c>
@@ -13439,7 +13454,7 @@
       <c r="A13" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="B13" s="59"/>
+      <c r="B13" s="61"/>
       <c r="C13" s="22" t="s">
         <v>271</v>
       </c>
@@ -13472,7 +13487,7 @@
       <c r="A14" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="B14" s="59"/>
+      <c r="B14" s="61"/>
       <c r="C14" s="22" t="s">
         <v>274</v>
       </c>
@@ -13505,7 +13520,7 @@
       <c r="A15" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="B15" s="59"/>
+      <c r="B15" s="61"/>
       <c r="C15" s="22" t="s">
         <v>279</v>
       </c>
@@ -13538,7 +13553,7 @@
       <c r="A16" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="B16" s="59"/>
+      <c r="B16" s="61"/>
       <c r="C16" s="22" t="s">
         <v>282</v>
       </c>
@@ -13571,7 +13586,7 @@
       <c r="A17" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="B17" s="59"/>
+      <c r="B17" s="61"/>
       <c r="C17" s="22" t="s">
         <v>286</v>
       </c>
@@ -13604,7 +13619,7 @@
       <c r="A18" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="B18" s="59"/>
+      <c r="B18" s="61"/>
       <c r="C18" s="22" t="s">
         <v>289</v>
       </c>
@@ -13637,7 +13652,7 @@
       <c r="A19" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="B19" s="59"/>
+      <c r="B19" s="61"/>
       <c r="C19" s="22" t="s">
         <v>294</v>
       </c>
@@ -13670,7 +13685,7 @@
       <c r="A20" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="B20" s="59"/>
+      <c r="B20" s="61"/>
       <c r="C20" s="22" t="s">
         <v>298</v>
       </c>
@@ -13703,7 +13718,7 @@
       <c r="A21" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="B21" s="59"/>
+      <c r="B21" s="61"/>
       <c r="C21" s="22" t="s">
         <v>303</v>
       </c>
@@ -13736,7 +13751,7 @@
       <c r="A22" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B22" s="59"/>
+      <c r="B22" s="61"/>
       <c r="C22" s="22" t="s">
         <v>305</v>
       </c>
@@ -13769,7 +13784,7 @@
       <c r="A23" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="B23" s="59"/>
+      <c r="B23" s="61"/>
       <c r="C23" s="22" t="s">
         <v>310</v>
       </c>
@@ -13802,7 +13817,7 @@
       <c r="A24" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="B24" s="59"/>
+      <c r="B24" s="61"/>
       <c r="C24" s="22" t="s">
         <v>314</v>
       </c>
@@ -13835,7 +13850,7 @@
       <c r="A25" s="10" t="s">
         <v>315</v>
       </c>
-      <c r="B25" s="59"/>
+      <c r="B25" s="61"/>
       <c r="C25" s="22" t="s">
         <v>316</v>
       </c>
@@ -13865,7 +13880,7 @@
       <c r="A26" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="B26" s="59"/>
+      <c r="B26" s="61"/>
       <c r="C26" s="64" t="s">
         <v>321</v>
       </c>
@@ -13878,10 +13893,10 @@
       <c r="F26" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G26" s="59" t="s">
-        <v>28</v>
-      </c>
-      <c r="H26" s="59" t="s">
+      <c r="G26" s="61" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="61" t="s">
         <v>28</v>
       </c>
       <c r="I26" s="12" t="s">
@@ -13895,7 +13910,7 @@
       <c r="A27" s="10" t="s">
         <v>325</v>
       </c>
-      <c r="B27" s="59"/>
+      <c r="B27" s="61"/>
       <c r="C27" s="58"/>
       <c r="D27" s="63"/>
       <c r="E27" s="11" t="s">
@@ -13904,14 +13919,14 @@
       <c r="F27" s="11" t="s">
         <v>327</v>
       </c>
-      <c r="G27" s="59"/>
+      <c r="G27" s="61"/>
       <c r="H27" s="63"/>
     </row>
     <row r="28" spans="1:11" ht="76.5" customHeight="1">
       <c r="A28" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="B28" s="59"/>
+      <c r="B28" s="61"/>
       <c r="C28" s="22" t="s">
         <v>329</v>
       </c>
@@ -13944,7 +13959,7 @@
       <c r="A29" s="10" t="s">
         <v>333</v>
       </c>
-      <c r="B29" s="59"/>
+      <c r="B29" s="61"/>
       <c r="C29" s="22" t="s">
         <v>334</v>
       </c>
@@ -13977,7 +13992,7 @@
       <c r="A30" s="10" t="s">
         <v>337</v>
       </c>
-      <c r="B30" s="59"/>
+      <c r="B30" s="61"/>
       <c r="C30" s="22" t="s">
         <v>338</v>
       </c>
@@ -14010,7 +14025,7 @@
       <c r="A31" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="B31" s="59"/>
+      <c r="B31" s="61"/>
       <c r="C31" s="22" t="s">
         <v>341</v>
       </c>
@@ -14125,7 +14140,7 @@
       <c r="A36" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="B36" s="61" t="s">
+      <c r="B36" s="59" t="s">
         <v>349</v>
       </c>
       <c r="C36" s="22" t="s">
@@ -14160,7 +14175,7 @@
       <c r="A37" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="B37" s="59"/>
+      <c r="B37" s="61"/>
       <c r="C37" s="23" t="s">
         <v>354</v>
       </c>
@@ -14219,6 +14234,41 @@
       </c>
       <c r="K38" s="13" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="255">
+      <c r="A39" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>804</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>806</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>807</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>808</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H39" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="I39" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J39" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K39" s="13" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -14329,7 +14379,7 @@
       <c r="A3" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="59" t="s">
         <v>359</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -14518,7 +14568,7 @@
       <c r="A10" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="B10" s="60" t="s">
+      <c r="B10" s="57" t="s">
         <v>385</v>
       </c>
       <c r="C10" s="11" t="s">
@@ -14806,7 +14856,7 @@
       <c r="A20" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="59" t="s">
         <v>422</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -15424,7 +15474,7 @@
       <c r="A40" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="57" t="s">
         <v>505</v>
       </c>
       <c r="C40" s="11" t="s">
@@ -15580,7 +15630,7 @@
       <c r="A46" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="59" t="s">
         <v>526</v>
       </c>
       <c r="C46" s="8" t="s">
@@ -15858,7 +15908,7 @@
       <c r="A56" s="7" t="s">
         <v>358</v>
       </c>
-      <c r="B56" s="43" t="s">
+      <c r="B56" s="46" t="s">
         <v>560</v>
       </c>
       <c r="C56" s="8" t="s">
@@ -16135,13 +16185,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:9" ht="30">
       <c r="A3" t="s">
@@ -16362,13 +16412,13 @@
       <c r="A2" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">

</xml_diff>